<commit_message>
Only find existing features for vertical sections and drill holes.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@44728 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1372" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="224">
   <si>
     <t xml:space="preserve">Outcrop / 2</t>
   </si>
@@ -589,6 +589,9 @@
   </si>
   <si>
     <t xml:space="preserve">FOLDER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR_NUMBER something. Not sure if it should be FIELD_NUMBER or FEATURE_NAME.</t>
   </si>
   <si>
     <t xml:space="preserve">#COLLECTOR$PERSON_ID$NAME</t>
@@ -3817,11 +3820,9 @@
       <c r="E3" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="F3" s="1"/>
       <c r="H3" s="1" t="s">
-        <v>8</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4141,7 +4142,7 @@
         <v>19</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H20" s="1"/>
     </row>
@@ -4193,7 +4194,7 @@
         <v>22</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4210,7 +4211,7 @@
         <v>23</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4227,7 +4228,7 @@
         <v>24</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4244,7 +4245,7 @@
         <v>25</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4369,11 +4370,11 @@
         <v>32</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F33" s="1"/>
       <c r="H33" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4381,7 +4382,7 @@
         <v>0</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>2</v>
@@ -4390,11 +4391,11 @@
         <v>33</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F34" s="1"/>
       <c r="H34" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4402,7 +4403,7 @@
         <v>0</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>5</v>
@@ -4411,11 +4412,11 @@
         <v>34</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F35" s="1"/>
       <c r="H35" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4423,7 +4424,7 @@
         <v>0</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>2</v>
@@ -4432,11 +4433,11 @@
         <v>35</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F36" s="1"/>
       <c r="H36" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4444,7 +4445,7 @@
         <v>0</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>5</v>
@@ -4453,11 +4454,11 @@
         <v>36</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F37" s="1"/>
       <c r="H37" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4465,7 +4466,7 @@
         <v>0</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>2</v>
@@ -4474,11 +4475,11 @@
         <v>37</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F38" s="1"/>
       <c r="H38" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4486,7 +4487,7 @@
         <v>0</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>5</v>
@@ -4495,11 +4496,11 @@
         <v>38</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F39" s="1"/>
       <c r="H39" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4507,7 +4508,7 @@
         <v>0</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>2</v>
@@ -4516,11 +4517,11 @@
         <v>39</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F40" s="1"/>
       <c r="H40" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4528,7 +4529,7 @@
         <v>0</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>2</v>
@@ -4537,13 +4538,13 @@
         <v>40</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4954,15 +4955,16 @@
       <c r="B66" s="0" t="s">
         <v>128</v>
       </c>
+      <c r="C66" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="D66" s="0" t="n">
         <v>2</v>
       </c>
       <c r="E66" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="F66" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="F66" s="1"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
@@ -4992,7 +4994,7 @@
         <v>4</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5006,7 +5008,7 @@
         <v>5</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5085,7 +5087,7 @@
         <v>10</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H74" s="1" t="s">
         <v>136</v>
@@ -5139,7 +5141,7 @@
         <v>13</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5156,7 +5158,7 @@
         <v>14</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5173,7 +5175,7 @@
         <v>15</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5190,7 +5192,7 @@
         <v>16</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5322,7 +5324,7 @@
         <v>127</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>2</v>
@@ -5331,11 +5333,11 @@
         <v>24</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F88" s="1"/>
       <c r="H88" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5343,7 +5345,7 @@
         <v>127</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>5</v>
@@ -5352,11 +5354,11 @@
         <v>25</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F89" s="1"/>
       <c r="H89" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5364,7 +5366,7 @@
         <v>127</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>2</v>
@@ -5373,11 +5375,11 @@
         <v>26</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F90" s="1"/>
       <c r="H90" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5385,7 +5387,7 @@
         <v>127</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>5</v>
@@ -5394,11 +5396,11 @@
         <v>27</v>
       </c>
       <c r="E91" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F91" s="1"/>
       <c r="H91" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5406,7 +5408,7 @@
         <v>127</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>2</v>
@@ -5415,11 +5417,11 @@
         <v>28</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F92" s="1"/>
       <c r="H92" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5427,7 +5429,7 @@
         <v>127</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>5</v>
@@ -5436,11 +5438,11 @@
         <v>29</v>
       </c>
       <c r="E93" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F93" s="1"/>
       <c r="H93" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5448,7 +5450,7 @@
         <v>127</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>2</v>
@@ -5457,11 +5459,11 @@
         <v>30</v>
       </c>
       <c r="E94" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F94" s="1"/>
       <c r="H94" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5469,7 +5471,7 @@
         <v>127</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>2</v>
@@ -5478,13 +5480,13 @@
         <v>31</v>
       </c>
       <c r="E95" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F95" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5921,15 +5923,16 @@
       <c r="B122" s="0" t="s">
         <v>151</v>
       </c>
+      <c r="C122" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="D122" s="0" t="n">
         <v>2</v>
       </c>
       <c r="E122" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="F122" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="F122" s="1"/>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="1" t="s">
@@ -5942,7 +5945,7 @@
         <v>3</v>
       </c>
       <c r="F123" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5956,7 +5959,7 @@
         <v>4</v>
       </c>
       <c r="F124" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6023,7 +6026,7 @@
         <v>9</v>
       </c>
       <c r="F129" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6074,7 +6077,7 @@
         <v>12</v>
       </c>
       <c r="F132" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H132" s="1" t="s">
         <v>139</v>
@@ -6094,7 +6097,7 @@
         <v>13</v>
       </c>
       <c r="F133" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H133" s="1"/>
     </row>
@@ -6112,7 +6115,7 @@
         <v>14</v>
       </c>
       <c r="F134" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="H134" s="1"/>
     </row>
@@ -6130,7 +6133,7 @@
         <v>15</v>
       </c>
       <c r="F135" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H135" s="1"/>
     </row>
@@ -6263,7 +6266,7 @@
         <v>150</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C143" s="1" t="s">
         <v>2</v>
@@ -6272,11 +6275,11 @@
         <v>23</v>
       </c>
       <c r="E143" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F143" s="1"/>
       <c r="H143" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6284,7 +6287,7 @@
         <v>150</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>5</v>
@@ -6293,11 +6296,11 @@
         <v>24</v>
       </c>
       <c r="E144" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F144" s="1"/>
       <c r="H144" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6305,7 +6308,7 @@
         <v>150</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>2</v>
@@ -6314,11 +6317,11 @@
         <v>25</v>
       </c>
       <c r="E145" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F145" s="1"/>
       <c r="H145" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6326,7 +6329,7 @@
         <v>150</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>5</v>
@@ -6335,11 +6338,11 @@
         <v>26</v>
       </c>
       <c r="E146" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F146" s="1"/>
       <c r="H146" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6347,7 +6350,7 @@
         <v>150</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>2</v>
@@ -6356,11 +6359,11 @@
         <v>27</v>
       </c>
       <c r="E147" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F147" s="1"/>
       <c r="H147" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6368,7 +6371,7 @@
         <v>150</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>5</v>
@@ -6377,11 +6380,11 @@
         <v>28</v>
       </c>
       <c r="E148" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F148" s="1"/>
       <c r="H148" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6389,7 +6392,7 @@
         <v>150</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>2</v>
@@ -6398,11 +6401,11 @@
         <v>29</v>
       </c>
       <c r="E149" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F149" s="1"/>
       <c r="H149" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6410,7 +6413,7 @@
         <v>150</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C150" s="1" t="s">
         <v>2</v>
@@ -6419,13 +6422,13 @@
         <v>30</v>
       </c>
       <c r="E150" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F150" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H150" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6881,7 +6884,7 @@
         <v>3</v>
       </c>
       <c r="F178" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6895,7 +6898,7 @@
         <v>4</v>
       </c>
       <c r="F179" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7052,7 +7055,7 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" operator="between" prompt="The importer only looks at the trailing &quot;/ Number&quot; part of this text to match it with something in the database." promptTitle="Drop-down list" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C65 C71 C73:C95 C97:C102 C104:C119 C130:C157 C159:C174" type="list">
+    <dataValidation allowBlank="true" operator="between" prompt="The importer only looks at the trailing &quot;/ Number&quot; part of this text to match it with something in the database." promptTitle="Drop-down list" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C66 C71 C73:C95 C97:C102 C104:C119 C122 C130:C157 C159:C174" type="list">
       <formula1>_Lists!$C$2:$C$11</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Make some columns work because they weren't SELECTIONs.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@44742 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1363" uniqueCount="224">
   <si>
     <t xml:space="preserve">Outcrop / 2</t>
   </si>
@@ -5081,7 +5081,7 @@
         <v>49</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D74" s="0" t="n">
         <v>10</v>
@@ -5531,9 +5531,7 @@
       <c r="B98" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C98" s="1" t="s">
-        <v>29</v>
-      </c>
+      <c r="C98" s="1"/>
       <c r="D98" s="0" t="n">
         <v>34</v>
       </c>
@@ -5565,9 +5563,7 @@
       <c r="B100" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C100" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="C100" s="1"/>
       <c r="D100" s="0" t="n">
         <v>36</v>
       </c>
@@ -5630,9 +5626,7 @@
       <c r="B104" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C104" s="1" t="s">
-        <v>146</v>
-      </c>
+      <c r="C104" s="1"/>
       <c r="D104" s="0" t="n">
         <v>40</v>
       </c>
@@ -5800,9 +5794,7 @@
       <c r="B114" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C114" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="C114" s="1"/>
       <c r="D114" s="0" t="n">
         <v>50</v>
       </c>
@@ -6477,9 +6469,7 @@
       <c r="B153" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C153" s="1" t="s">
-        <v>29</v>
-      </c>
+      <c r="C153" s="1"/>
       <c r="D153" s="0" t="n">
         <v>33</v>
       </c>
@@ -6511,9 +6501,7 @@
       <c r="B155" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C155" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="C155" s="1"/>
       <c r="D155" s="0" t="n">
         <v>35</v>
       </c>
@@ -6576,9 +6564,7 @@
       <c r="B159" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C159" s="1" t="s">
-        <v>146</v>
-      </c>
+      <c r="C159" s="1"/>
       <c r="D159" s="0" t="n">
         <v>39</v>
       </c>
@@ -6746,9 +6732,7 @@
       <c r="B169" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C169" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="C169" s="1"/>
       <c r="D169" s="0" t="n">
         <v>49</v>
       </c>

</xml_diff>

<commit_message>
Two more columns in the drillhole spreadsheet.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@44745 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1363" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1368" uniqueCount="226">
   <si>
     <t xml:space="preserve">Outcrop / 2</t>
   </si>
@@ -694,6 +694,12 @@
   </si>
   <si>
     <t xml:space="preserve">TOP_DEPTH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRILL_TYPE_ID$NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should this be called “Drill type”?</t>
   </si>
 </sst>
 </file>
@@ -5316,6 +5322,9 @@
       <c r="D87" s="0" t="n">
         <v>23</v>
       </c>
+      <c r="E87" s="0" t="s">
+        <v>195</v>
+      </c>
       <c r="F87" s="1"/>
       <c r="H87" s="1"/>
     </row>
@@ -5901,6 +5910,9 @@
       <c r="B121" s="0" t="s">
         <v>1</v>
       </c>
+      <c r="C121" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="D121" s="0" t="n">
         <v>1</v>
       </c>
@@ -5977,6 +5989,12 @@
       </c>
       <c r="D126" s="0" t="n">
         <v>6</v>
+      </c>
+      <c r="F126" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="H126" s="0" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6250,6 +6268,9 @@
       <c r="D142" s="0" t="n">
         <v>22</v>
       </c>
+      <c r="E142" s="0" t="s">
+        <v>195</v>
+      </c>
       <c r="F142" s="1"/>
       <c r="H142" s="1"/>
     </row>
@@ -7039,7 +7060,7 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" operator="between" prompt="The importer only looks at the trailing &quot;/ Number&quot; part of this text to match it with something in the database." promptTitle="Drop-down list" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C66 C71 C73:C95 C97:C102 C104:C119 C122 C130:C157 C159:C174" type="list">
+    <dataValidation allowBlank="true" operator="between" prompt="The importer only looks at the trailing &quot;/ Number&quot; part of this text to match it with something in the database." promptTitle="Drop-down list" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C66 C71 C73:C95 C97:C102 C104:C119 C121:C122 C130:C157 C159:C174" type="list">
       <formula1>_Lists!$C$2:$C$11</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Comments on headings now work.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@44906 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -9,7 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="_Cover sheet" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="_Lists" sheetId="2" state="hidden" r:id="rId3"/>
+    <sheet name="_Lists" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="Metaimporter" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1368" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1462" uniqueCount="269">
   <si>
     <t xml:space="preserve">Outcrop / 2</t>
   </si>
@@ -540,7 +540,7 @@
     <t xml:space="preserve">Auto-increment ID / 9</t>
   </si>
   <si>
-    <t xml:space="preserve">Find in selection, else create / 5</t>
+    <t xml:space="preserve">Find only / 1</t>
   </si>
   <si>
     <t xml:space="preserve">no</t>
@@ -552,7 +552,7 @@
     <t xml:space="preserve">Composition / 7</t>
   </si>
   <si>
-    <t xml:space="preserve">Find value, else create. / 7</t>
+    <t xml:space="preserve">Find, else create / 2</t>
   </si>
   <si>
     <t xml:space="preserve">Metaimporter / 1</t>
@@ -591,28 +591,115 @@
     <t xml:space="preserve">FOLDER</t>
   </si>
   <si>
-    <t xml:space="preserve">FR_NUMBER something. Not sure if it should be FIELD_NUMBER or FEATURE_NAME.</t>
+    <t xml:space="preserve">Folders are your groupings of imported data within FRED. Just choose one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the field number that you yourself have created.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is used to find a curator for the data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If this is a recollection of a previous collection, enter the Fossil Record Number of the earlier collection here. This must match an existing FRN in FRED.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This gets added to the audit trail for this entry.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Choose the coordinate system you used to enter the following coordinates.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the easting or longitude coordinate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the northing or latitude coordinate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter how this coordinate was found.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If using a map, what was the scale on that map?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If using a map, when was that map made?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How accurate your coordinate measurement was, in metres. If blank, 10m is used.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you have any comments about how the coordinates were found?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Describe the location of the coordinate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which country was this sample found in?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter a description of the locality, should we ever need to find it again.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When was the collection collected?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the accuracy of the date?</t>
   </si>
   <si>
     <t xml:space="preserve">#COLLECTOR$PERSON_ID$NAME</t>
   </si>
   <si>
+    <t xml:space="preserve">Enter the collector. If not in the list, enter a new name. Names must match the exact spelling as the entry in FRED.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the fossil “in place”?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List the fossils not collected. This is free text.</t>
+  </si>
+  <si>
     <t xml:space="preserve">#SENT_TO$FOSSIL_GROUP_ID$NAME</t>
   </si>
   <si>
+    <t xml:space="preserve">Which study area was this fossil sent to?</t>
+  </si>
+  <si>
     <t xml:space="preserve">#SENT_TO$PERSON_ID$NAME</t>
   </si>
   <si>
+    <t xml:space="preserve">Enter the person that this fossil was sent to. If the person is not found, a new person will be created in FRED; the name must match exactly.</t>
+  </si>
+  <si>
     <t xml:space="preserve">#SENT_TO$LAB_ID$LAB_NAME</t>
   </si>
   <si>
+    <t xml:space="preserve">Which lab was this fossil sent to?</t>
+  </si>
+  <si>
     <t xml:space="preserve">#SENT_TO$COMMENTS</t>
   </si>
   <si>
+    <t xml:space="preserve">Enter how this collection is significant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the stratigraphic unit. This must match exactly an entry from StratLex.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the lower bound for the known stage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the upport bound for the known stage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the lower bound for the inferred stage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the upper bound for the inferred stage.</t>
+  </si>
+  <si>
     <t xml:space="preserve">SAMPLES_NEARBY</t>
   </si>
   <si>
-    <t xml:space="preserve">Nearby samples; make a vertical list. TODO: show this as a vertical list.</t>
+    <t xml:space="preserve">List the field numbers (as per the “Field number”) column of nearby samples. This is a multi-value column; enter multiple field numbers, one per cell, in a vertical list under this row.</t>
   </si>
   <si>
     <t xml:space="preserve">Sample Relationship Mod</t>
@@ -621,85 +708,127 @@
     <t xml:space="preserve">SAMPLE_RELATIONSHIP_MOD</t>
   </si>
   <si>
+    <t xml:space="preserve">For a Sample Relationship, “c.” or “?”.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample Relationship Distance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAMPLE_RELATIONSHIP_DISTANCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The distance or distance range of the sample relationship, in metres. Use decimal numbers; for a range use a dash, e.g. “1.0m – 1.1m”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample Relationship Prep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAMPLE_RELATIONSHIP_PREP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For a Sample Relationship, whether the sample is “above” or “below” the next related field.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample Relationship Reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAMPLE_RELATIONSHIP_REFERENCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Another sample, either already in FRED or in this spreadsheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strat. Relationship Mod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STRAT_RELATIONSHIP_MOD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For a Stratigraphic Relationship, “c.” or “?”. TODO: what do these mean?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strat. Relationship Distance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STRAT_RELATIONSHIP_DISTANCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The distance or distance range of the stratigraphic relationship, in metres. Use decimal numbers; for a range use a dash, e.g. “1.0m – 1.1m”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strat. Relationship Prep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STRAT_RELATIONSHIP_PREP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For a Stratigraphic Relationship, a relation to a strategraphic reference horizon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strat. Unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STRAT_RELATIONSHIP_STRAT_UNIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#RELATIONSHIP$STRAT_UNIT_ID$SU_NAME_STANDARD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The stratigraphic unit in the Stratigraphic Relationship.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If available, enter a reference where a map or column of the collection site may be found, ideally reference to an entry in the New Zealand Measured Section database.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The dip, in degrees (0 for horizontal strata)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The cardinal direction of the dip.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The strike direction, in degrees true (leave blank for horizontal strata)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter any other brief observations of the stratigraphy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Was a comparator used?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter one of “marine” or “non-marine”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter any additional notes on the nature of the rock.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use this field to reference any correspondence, publications or other information source.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the name of a previously entered and approved vertical section.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOTTOM_DEPTH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the bottom depth of the sample.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOP_DEPTH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the top depth of the sample.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the unit used in measuring the top and bottom depths.</t>
+  </si>
+  <si>
     <t xml:space="preserve">For a Sample Relationship, “c.” or “?”. TODO: what do these mean?</t>
   </si>
   <si>
-    <t xml:space="preserve">Sample Relationship Distance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAMPLE_RELATIONSHIP_DISTANCE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The distance or distance range of the sample relationship, in metres. Use decimal numbers; for a range use a dash, e.g. “1.0m – 1.1m”</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sample Relationship Prep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAMPLE_RELATIONSHIP_PREP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For a Sample Relationship, whether the sample is “above” or “below” the next related field.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sample Relationship Reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAMPLE_RELATIONSHIP_REFERENCE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Another sample, either already in FRED or in this spreadsheet.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strat. Relationship Mod</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STRAT_RELATIONSHIP_MOD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For a Stratigraphic Relationship, “c.” or “?”. TODO: what do these mean?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strat. Relationship Distance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STRAT_RELATIONSHIP_DISTANCE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The distance or distance range of the stratigraphic relationship, in metres. Use decimal numbers; for a range use a dash, e.g. “1.0m – 1.1m”</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strat. Relationship Prep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STRAT_RELATIONSHIP_PREP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For a Stratigraphic Relationship, a relation to a strategraphic reference horizon.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strat. Unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STRAT_RELATIONSHIP_STRAT_UNIT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#RELATIONSHIP$STRAT_UNIT_ID$SU_NAME_STANDARD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The stratigraphic unit in the Stratigraphic Relationship.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOTTOM_DEPTH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOP_DEPTH</t>
+    <t xml:space="preserve">TODO: What does this column do?</t>
   </si>
   <si>
     <t xml:space="preserve">DRILL_TYPE_ID$NAME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Should this be called “Drill type”?</t>
   </si>
 </sst>
 </file>
@@ -3751,7 +3880,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.85"/>
@@ -3807,7 +3936,7 @@
         <v>188</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>3</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3828,7 +3957,7 @@
       </c>
       <c r="F3" s="1"/>
       <c r="H3" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3847,7 +3976,9 @@
       <c r="F4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="1"/>
+      <c r="H4" s="1" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
@@ -3864,7 +3995,7 @@
       </c>
       <c r="F5" s="1"/>
       <c r="H5" s="1" t="s">
-        <v>12</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3883,7 +4014,9 @@
       <c r="F6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="1"/>
+      <c r="H6" s="1" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
@@ -3904,7 +4037,9 @@
       <c r="F7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="1"/>
+      <c r="H7" s="1" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
@@ -3924,7 +4059,7 @@
       </c>
       <c r="F8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>21</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3944,7 +4079,9 @@
         <v>23</v>
       </c>
       <c r="F9" s="1"/>
-      <c r="H9" s="1"/>
+      <c r="H9" s="1" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
@@ -3964,7 +4101,7 @@
       </c>
       <c r="F10" s="1"/>
       <c r="H10" s="1" t="s">
-        <v>26</v>
+        <v>197</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3981,7 +4118,9 @@
         <v>10</v>
       </c>
       <c r="F11" s="1"/>
-      <c r="H11" s="1"/>
+      <c r="H11" s="1" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
@@ -3999,7 +4138,9 @@
       <c r="F12" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="1"/>
+      <c r="H12" s="1" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
@@ -4018,7 +4159,9 @@
         <v>32</v>
       </c>
       <c r="F13" s="1"/>
-      <c r="H13" s="1"/>
+      <c r="H13" s="1" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
@@ -4036,7 +4179,9 @@
       <c r="F14" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H14" s="1"/>
+      <c r="H14" s="1" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
@@ -4057,7 +4202,9 @@
       <c r="F15" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H15" s="1"/>
+      <c r="H15" s="1" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
@@ -4077,7 +4224,7 @@
       </c>
       <c r="F16" s="1"/>
       <c r="H16" s="1" t="s">
-        <v>41</v>
+        <v>203</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4095,7 +4242,7 @@
       </c>
       <c r="F17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>43</v>
+        <v>204</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4114,7 +4261,9 @@
       <c r="F18" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H18" s="1"/>
+      <c r="H18" s="1" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
@@ -4132,7 +4281,9 @@
       <c r="F19" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="H19" s="1"/>
+      <c r="H19" s="1" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
@@ -4148,9 +4299,14 @@
         <v>19</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="H20" s="1"/>
+        <v>207</v>
+      </c>
+      <c r="G20" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
@@ -4166,7 +4322,9 @@
       <c r="F21" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="H21" s="1"/>
+      <c r="H21" s="1" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
@@ -4184,7 +4342,9 @@
       <c r="F22" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="H22" s="1"/>
+      <c r="H22" s="1" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
@@ -4200,7 +4360,10 @@
         <v>22</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>191</v>
+        <v>211</v>
+      </c>
+      <c r="H23" s="0" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4217,7 +4380,13 @@
         <v>23</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>192</v>
+        <v>213</v>
+      </c>
+      <c r="G24" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="H24" s="0" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4234,7 +4403,10 @@
         <v>24</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>193</v>
+        <v>215</v>
+      </c>
+      <c r="H25" s="0" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4251,7 +4423,7 @@
         <v>25</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>194</v>
+        <v>217</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4270,7 +4442,9 @@
       <c r="F27" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H27" s="1"/>
+      <c r="H27" s="1" t="s">
+        <v>218</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
@@ -4288,7 +4462,9 @@
       <c r="F28" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="H28" s="1"/>
+      <c r="H28" s="1" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
@@ -4306,7 +4482,9 @@
       <c r="F29" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="H29" s="1"/>
+      <c r="H29" s="1" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
@@ -4324,7 +4502,9 @@
       <c r="F30" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="H30" s="1"/>
+      <c r="H30" s="1" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
@@ -4342,7 +4522,9 @@
       <c r="F31" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="H31" s="1"/>
+      <c r="H31" s="1" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
@@ -4360,7 +4542,9 @@
       <c r="F32" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="H32" s="1"/>
+      <c r="H32" s="1" t="s">
+        <v>223</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
@@ -4376,11 +4560,11 @@
         <v>32</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>195</v>
+        <v>224</v>
       </c>
       <c r="F33" s="1"/>
       <c r="H33" s="1" t="s">
-        <v>196</v>
+        <v>225</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4388,7 +4572,7 @@
         <v>0</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>197</v>
+        <v>226</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>2</v>
@@ -4397,11 +4581,11 @@
         <v>33</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>198</v>
+        <v>227</v>
       </c>
       <c r="F34" s="1"/>
       <c r="H34" s="1" t="s">
-        <v>199</v>
+        <v>228</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4409,7 +4593,7 @@
         <v>0</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>200</v>
+        <v>229</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>5</v>
@@ -4418,11 +4602,11 @@
         <v>34</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>201</v>
+        <v>230</v>
       </c>
       <c r="F35" s="1"/>
       <c r="H35" s="1" t="s">
-        <v>202</v>
+        <v>231</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4430,7 +4614,7 @@
         <v>0</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>203</v>
+        <v>232</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>2</v>
@@ -4439,11 +4623,11 @@
         <v>35</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>204</v>
+        <v>233</v>
       </c>
       <c r="F36" s="1"/>
       <c r="H36" s="1" t="s">
-        <v>205</v>
+        <v>234</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4451,7 +4635,7 @@
         <v>0</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>206</v>
+        <v>235</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>5</v>
@@ -4460,11 +4644,11 @@
         <v>36</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>207</v>
+        <v>236</v>
       </c>
       <c r="F37" s="1"/>
       <c r="H37" s="1" t="s">
-        <v>208</v>
+        <v>237</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4472,7 +4656,7 @@
         <v>0</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>209</v>
+        <v>238</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>2</v>
@@ -4481,11 +4665,11 @@
         <v>37</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>210</v>
+        <v>239</v>
       </c>
       <c r="F38" s="1"/>
       <c r="H38" s="1" t="s">
-        <v>211</v>
+        <v>240</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4493,7 +4677,7 @@
         <v>0</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>212</v>
+        <v>241</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>5</v>
@@ -4502,11 +4686,11 @@
         <v>38</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>213</v>
+        <v>242</v>
       </c>
       <c r="F39" s="1"/>
       <c r="H39" s="1" t="s">
-        <v>214</v>
+        <v>243</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4514,7 +4698,7 @@
         <v>0</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>215</v>
+        <v>244</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>2</v>
@@ -4523,11 +4707,11 @@
         <v>39</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>216</v>
+        <v>245</v>
       </c>
       <c r="F40" s="1"/>
       <c r="H40" s="1" t="s">
-        <v>217</v>
+        <v>246</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4535,7 +4719,7 @@
         <v>0</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>218</v>
+        <v>247</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>2</v>
@@ -4544,13 +4728,13 @@
         <v>40</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>219</v>
+        <v>248</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>220</v>
+        <v>249</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>221</v>
+        <v>250</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4572,7 +4756,9 @@
       <c r="F42" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="H42" s="1"/>
+      <c r="H42" s="1" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
@@ -4590,7 +4776,9 @@
       <c r="F43" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="H43" s="1"/>
+      <c r="H43" s="1" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
@@ -4606,6 +4794,9 @@
       <c r="F44" s="1" t="s">
         <v>88</v>
       </c>
+      <c r="H44" s="0" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
@@ -4621,6 +4812,9 @@
       <c r="F45" s="1" t="s">
         <v>90</v>
       </c>
+      <c r="H45" s="0" t="s">
+        <v>254</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
@@ -4653,6 +4847,9 @@
       <c r="F47" s="1" t="s">
         <v>94</v>
       </c>
+      <c r="H47" s="0" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
@@ -4685,6 +4882,9 @@
       <c r="F49" s="1" t="s">
         <v>98</v>
       </c>
+      <c r="H49" s="0" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
@@ -4887,6 +5087,9 @@
       <c r="F61" s="1" t="s">
         <v>121</v>
       </c>
+      <c r="H61" s="0" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
@@ -4919,6 +5122,9 @@
       <c r="F63" s="1" t="s">
         <v>124</v>
       </c>
+      <c r="H63" s="0" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
@@ -4936,6 +5142,9 @@
       <c r="F64" s="1" t="s">
         <v>126</v>
       </c>
+      <c r="H64" s="0" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
@@ -4953,6 +5162,9 @@
       <c r="E65" s="0" t="s">
         <v>188</v>
       </c>
+      <c r="H65" s="1" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
@@ -4971,6 +5183,9 @@
         <v>6</v>
       </c>
       <c r="F66" s="1"/>
+      <c r="H66" s="1" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
@@ -4988,6 +5203,9 @@
       <c r="F67" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="H67" s="1" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
@@ -5000,7 +5218,10 @@
         <v>4</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>222</v>
+        <v>261</v>
+      </c>
+      <c r="H68" s="0" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5014,7 +5235,10 @@
         <v>5</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>223</v>
+        <v>263</v>
+      </c>
+      <c r="H69" s="0" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5030,6 +5254,9 @@
       <c r="F70" s="0" t="s">
         <v>132</v>
       </c>
+      <c r="H70" s="0" t="s">
+        <v>265</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
@@ -5047,6 +5274,9 @@
       <c r="F71" s="1" t="s">
         <v>46</v>
       </c>
+      <c r="H71" s="1" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
@@ -5061,22 +5291,31 @@
       <c r="F72" s="1" t="s">
         <v>48</v>
       </c>
+      <c r="H72" s="1" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="D73" s="0" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>46</v>
+        <v>207</v>
+      </c>
+      <c r="G73" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5084,19 +5323,17 @@
         <v>127</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>2</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="C74" s="1"/>
       <c r="D74" s="0" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>190</v>
+        <v>52</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>136</v>
+        <v>209</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5104,50 +5341,65 @@
         <v>127</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C75" s="1"/>
+        <v>53</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="D75" s="0" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="H75" s="1"/>
+        <v>54</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D76" s="0" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H76" s="1"/>
+        <v>211</v>
+      </c>
+      <c r="G76" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="H76" s="0" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D77" s="0" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>191</v>
+        <v>213</v>
+      </c>
+      <c r="G77" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="H77" s="0" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5155,16 +5407,22 @@
         <v>127</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D78" s="0" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>192</v>
+        <v>215</v>
+      </c>
+      <c r="G78" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="H78" s="0" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5172,16 +5430,19 @@
         <v>127</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D79" s="0" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>193</v>
+        <v>217</v>
+      </c>
+      <c r="G79" s="0" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5189,16 +5450,19 @@
         <v>127</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D80" s="0" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>194</v>
+        <v>64</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5206,147 +5470,162 @@
         <v>127</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D81" s="0" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H81" s="1"/>
+        <v>66</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D82" s="0" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H82" s="1"/>
+        <v>68</v>
+      </c>
+      <c r="H82" s="1" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D83" s="0" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="H83" s="1"/>
+        <v>70</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D84" s="0" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="H84" s="1"/>
+        <v>72</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D85" s="0" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H85" s="1"/>
+        <v>74</v>
+      </c>
+      <c r="H85" s="1" t="s">
+        <v>223</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>73</v>
+        <v>140</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D86" s="0" t="n">
-        <v>22</v>
-      </c>
-      <c r="F86" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="H86" s="1"/>
+        <v>23</v>
+      </c>
+      <c r="E86" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="F86" s="1"/>
+      <c r="H86" s="1" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>140</v>
+        <v>226</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D87" s="0" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>195</v>
+        <v>227</v>
       </c>
       <c r="F87" s="1"/>
-      <c r="H87" s="1"/>
+      <c r="H87" s="1" t="s">
+        <v>266</v>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>197</v>
+        <v>229</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D88" s="0" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>198</v>
+        <v>230</v>
       </c>
       <c r="F88" s="1"/>
       <c r="H88" s="1" t="s">
-        <v>199</v>
+        <v>231</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5354,20 +5633,20 @@
         <v>127</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>200</v>
+        <v>232</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D89" s="0" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>201</v>
+        <v>233</v>
       </c>
       <c r="F89" s="1"/>
       <c r="H89" s="1" t="s">
-        <v>202</v>
+        <v>234</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5375,20 +5654,20 @@
         <v>127</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>203</v>
+        <v>235</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D90" s="0" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>204</v>
+        <v>236</v>
       </c>
       <c r="F90" s="1"/>
       <c r="H90" s="1" t="s">
-        <v>205</v>
+        <v>237</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5396,20 +5675,20 @@
         <v>127</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>206</v>
+        <v>238</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D91" s="0" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E91" s="0" t="s">
-        <v>207</v>
+        <v>239</v>
       </c>
       <c r="F91" s="1"/>
       <c r="H91" s="1" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5417,20 +5696,20 @@
         <v>127</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>209</v>
+        <v>241</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D92" s="0" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>210</v>
+        <v>242</v>
       </c>
       <c r="F92" s="1"/>
       <c r="H92" s="1" t="s">
-        <v>211</v>
+        <v>243</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5438,20 +5717,20 @@
         <v>127</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>212</v>
+        <v>244</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D93" s="0" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E93" s="0" t="s">
-        <v>213</v>
+        <v>245</v>
       </c>
       <c r="F93" s="1"/>
       <c r="H93" s="1" t="s">
-        <v>214</v>
+        <v>246</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5459,60 +5738,62 @@
         <v>127</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>215</v>
+        <v>247</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D94" s="0" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E94" s="0" t="s">
-        <v>216</v>
-      </c>
-      <c r="F94" s="1"/>
+        <v>248</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>249</v>
+      </c>
       <c r="H94" s="1" t="s">
-        <v>217</v>
+        <v>250</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B95" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>2</v>
+      <c r="B95" s="0" t="s">
+        <v>82</v>
       </c>
       <c r="D95" s="0" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E95" s="0" t="s">
-        <v>219</v>
+        <v>83</v>
       </c>
       <c r="F95" s="1" t="s">
-        <v>220</v>
+        <v>84</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>221</v>
+        <v>251</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B96" s="0" t="s">
-        <v>82</v>
+      <c r="B96" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="D96" s="0" t="n">
-        <v>32</v>
-      </c>
-      <c r="E96" s="0" t="s">
-        <v>83</v>
+        <v>33</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
+      </c>
+      <c r="H96" s="1" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5520,32 +5801,37 @@
         <v>127</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C97" s="1" t="s">
-        <v>19</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="C97" s="1"/>
       <c r="D97" s="0" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="H97" s="1"/>
+        <v>88</v>
+      </c>
+      <c r="H97" s="0" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C98" s="1"/>
+        <v>89</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="D98" s="0" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
+      </c>
+      <c r="H98" s="0" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5553,16 +5839,14 @@
         <v>127</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>19</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="C99" s="1"/>
       <c r="D99" s="0" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5570,14 +5854,19 @@
         <v>127</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C100" s="1"/>
+        <v>93</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="D100" s="0" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
+      </c>
+      <c r="H100" s="0" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5585,47 +5874,48 @@
         <v>127</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D101" s="0" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F101" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B102" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>2</v>
+      <c r="B102" s="0" t="s">
+        <v>144</v>
       </c>
       <c r="D102" s="0" t="n">
-        <v>38</v>
-      </c>
-      <c r="F102" s="1" t="s">
-        <v>96</v>
+        <v>39</v>
+      </c>
+      <c r="F102" s="0" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B103" s="0" t="s">
-        <v>144</v>
-      </c>
+      <c r="B103" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C103" s="1"/>
       <c r="D103" s="0" t="n">
-        <v>39</v>
-      </c>
-      <c r="F103" s="0" t="s">
-        <v>145</v>
+        <v>40</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="H103" s="0" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5633,14 +5923,16 @@
         <v>127</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C104" s="1"/>
+        <v>99</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>2</v>
+      </c>
       <c r="D104" s="0" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F104" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5648,16 +5940,16 @@
         <v>127</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D105" s="0" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5665,16 +5957,16 @@
         <v>127</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D106" s="0" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F106" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5682,16 +5974,16 @@
         <v>127</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D107" s="0" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5699,16 +5991,16 @@
         <v>127</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D108" s="0" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F108" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5716,16 +6008,16 @@
         <v>127</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D109" s="0" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5733,16 +6025,16 @@
         <v>127</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D110" s="0" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5750,16 +6042,16 @@
         <v>127</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D111" s="0" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F111" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5767,16 +6059,16 @@
         <v>127</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D112" s="0" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F112" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5784,16 +6076,14 @@
         <v>127</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>2</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="C113" s="1"/>
       <c r="D113" s="0" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F113" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5801,106 +6091,123 @@
         <v>127</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="C114" s="1"/>
+        <v>119</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="D114" s="0" t="n">
-        <v>50</v>
-      </c>
-      <c r="F114" s="1" t="s">
-        <v>118</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="F114" s="1"/>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D115" s="0" t="n">
-        <v>51</v>
-      </c>
-      <c r="F115" s="1"/>
+        <v>52</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="H115" s="0" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D116" s="0" t="n">
-        <v>52</v>
-      </c>
-      <c r="F116" s="1" t="s">
-        <v>121</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="F116" s="1"/>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D117" s="0" t="n">
-        <v>53</v>
-      </c>
-      <c r="F117" s="1"/>
+        <v>54</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="H117" s="0" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D118" s="0" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F118" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
+      </c>
+      <c r="H118" s="0" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B119" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C119" s="1" t="s">
-        <v>5</v>
+      <c r="B119" s="0" t="s">
+        <v>149</v>
       </c>
       <c r="D119" s="0" t="n">
-        <v>55</v>
-      </c>
-      <c r="F119" s="1" t="s">
-        <v>126</v>
+        <v>56</v>
+      </c>
+      <c r="H119" s="0" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="1" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="B120" s="0" t="s">
-        <v>149</v>
+        <v>1</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="D120" s="0" t="n">
-        <v>56</v>
+        <v>1</v>
+      </c>
+      <c r="E120" s="0" t="s">
+        <v>188</v>
+      </c>
+      <c r="H120" s="1" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5908,16 +6215,20 @@
         <v>150</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>1</v>
+        <v>151</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D121" s="0" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E121" s="0" t="s">
-        <v>188</v>
+        <v>6</v>
+      </c>
+      <c r="F121" s="1"/>
+      <c r="H121" s="1" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5925,31 +6236,33 @@
         <v>150</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>151</v>
-      </c>
-      <c r="C122" s="1" t="s">
-        <v>5</v>
+        <v>129</v>
       </c>
       <c r="D122" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E122" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="F122" s="1"/>
+        <v>3</v>
+      </c>
+      <c r="F122" s="0" t="s">
+        <v>261</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D123" s="0" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F123" s="0" t="s">
-        <v>222</v>
+        <v>263</v>
+      </c>
+      <c r="H123" s="0" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5957,13 +6270,16 @@
         <v>150</v>
       </c>
       <c r="B124" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D124" s="0" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F124" s="0" t="s">
-        <v>223</v>
+        <v>132</v>
+      </c>
+      <c r="H124" s="0" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5971,13 +6287,16 @@
         <v>150</v>
       </c>
       <c r="B125" s="0" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="D125" s="0" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>132</v>
+        <v>268</v>
+      </c>
+      <c r="H125" s="0" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5985,16 +6304,16 @@
         <v>150</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>152</v>
+        <v>44</v>
       </c>
       <c r="D126" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="F126" s="0" t="s">
-        <v>224</v>
-      </c>
-      <c r="H126" s="0" t="s">
-        <v>225</v>
+        <v>7</v>
+      </c>
+      <c r="F126" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H126" s="1" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6002,13 +6321,16 @@
         <v>150</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D127" s="0" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F127" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
+      </c>
+      <c r="H127" s="1" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6016,81 +6338,98 @@
         <v>150</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D128" s="0" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F128" s="1" t="s">
-        <v>48</v>
+        <v>207</v>
+      </c>
+      <c r="G128" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="H128" s="1" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B129" s="0" t="s">
-        <v>49</v>
-      </c>
+      <c r="B129" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C129" s="1"/>
       <c r="D129" s="0" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F129" s="1" t="s">
-        <v>190</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="H129" s="1"/>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C130" s="1"/>
+        <v>53</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="D130" s="0" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F130" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="H130" s="1"/>
+        <v>54</v>
+      </c>
+      <c r="H130" s="1" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D131" s="0" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F131" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H131" s="1"/>
+        <v>211</v>
+      </c>
+      <c r="H131" s="0" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D132" s="0" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F132" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="H132" s="1" t="s">
-        <v>139</v>
+        <v>213</v>
+      </c>
+      <c r="G132" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="H132" s="0" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6098,201 +6437,219 @@
         <v>150</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D133" s="0" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F133" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="H133" s="1"/>
+        <v>215</v>
+      </c>
+      <c r="H133" s="0" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D134" s="0" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F134" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="H134" s="1"/>
+        <v>217</v>
+      </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C135" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D135" s="0" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F135" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="H135" s="1"/>
+        <v>64</v>
+      </c>
+      <c r="H135" s="1" t="s">
+        <v>218</v>
+      </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C136" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D136" s="0" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F136" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H136" s="1"/>
+        <v>66</v>
+      </c>
+      <c r="H136" s="1" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D137" s="0" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F137" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H137" s="1"/>
+        <v>68</v>
+      </c>
+      <c r="H137" s="1" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D138" s="0" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F138" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="H138" s="1"/>
+        <v>70</v>
+      </c>
+      <c r="H138" s="1" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C139" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D139" s="0" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F139" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="H139" s="1"/>
+        <v>72</v>
+      </c>
+      <c r="H139" s="1" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D140" s="0" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F140" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H140" s="1"/>
+        <v>74</v>
+      </c>
+      <c r="H140" s="1" t="s">
+        <v>223</v>
+      </c>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>73</v>
+        <v>140</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D141" s="0" t="n">
-        <v>21</v>
-      </c>
-      <c r="F141" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="H141" s="1"/>
+        <v>22</v>
+      </c>
+      <c r="E141" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="F141" s="1"/>
+      <c r="H141" s="1" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>140</v>
+        <v>226</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D142" s="0" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E142" s="0" t="s">
-        <v>195</v>
+        <v>227</v>
       </c>
       <c r="F142" s="1"/>
-      <c r="H142" s="1"/>
+      <c r="H142" s="1" t="s">
+        <v>266</v>
+      </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>197</v>
+        <v>229</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D143" s="0" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E143" s="0" t="s">
-        <v>198</v>
+        <v>230</v>
       </c>
       <c r="F143" s="1"/>
       <c r="H143" s="1" t="s">
-        <v>199</v>
+        <v>231</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6300,20 +6657,20 @@
         <v>150</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>200</v>
+        <v>232</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D144" s="0" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E144" s="0" t="s">
-        <v>201</v>
+        <v>233</v>
       </c>
       <c r="F144" s="1"/>
       <c r="H144" s="1" t="s">
-        <v>202</v>
+        <v>234</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6321,20 +6678,20 @@
         <v>150</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>203</v>
+        <v>235</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D145" s="0" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E145" s="0" t="s">
-        <v>204</v>
+        <v>236</v>
       </c>
       <c r="F145" s="1"/>
       <c r="H145" s="1" t="s">
-        <v>205</v>
+        <v>237</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6342,20 +6699,20 @@
         <v>150</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>206</v>
+        <v>238</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D146" s="0" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E146" s="0" t="s">
-        <v>207</v>
+        <v>239</v>
       </c>
       <c r="F146" s="1"/>
       <c r="H146" s="1" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6363,20 +6720,20 @@
         <v>150</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>209</v>
+        <v>241</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D147" s="0" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E147" s="0" t="s">
-        <v>210</v>
+        <v>242</v>
       </c>
       <c r="F147" s="1"/>
       <c r="H147" s="1" t="s">
-        <v>211</v>
+        <v>243</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6384,20 +6741,20 @@
         <v>150</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>212</v>
+        <v>244</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D148" s="0" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E148" s="0" t="s">
-        <v>213</v>
+        <v>245</v>
       </c>
       <c r="F148" s="1"/>
       <c r="H148" s="1" t="s">
-        <v>214</v>
+        <v>246</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6405,20 +6762,22 @@
         <v>150</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>215</v>
+        <v>247</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D149" s="0" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E149" s="0" t="s">
-        <v>216</v>
-      </c>
-      <c r="F149" s="1"/>
+        <v>248</v>
+      </c>
+      <c r="F149" s="1" t="s">
+        <v>249</v>
+      </c>
       <c r="H149" s="1" t="s">
-        <v>217</v>
+        <v>250</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6426,22 +6785,22 @@
         <v>150</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>218</v>
+        <v>82</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D150" s="0" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E150" s="0" t="s">
-        <v>219</v>
+        <v>83</v>
       </c>
       <c r="F150" s="1" t="s">
-        <v>220</v>
+        <v>84</v>
       </c>
       <c r="H150" s="1" t="s">
-        <v>221</v>
+        <v>251</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6449,53 +6808,57 @@
         <v>150</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="D151" s="0" t="n">
-        <v>31</v>
-      </c>
-      <c r="E151" s="0" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="F151" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="H151" s="1"/>
+        <v>86</v>
+      </c>
+      <c r="H151" s="1" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C152" s="1" t="s">
-        <v>19</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="C152" s="1"/>
       <c r="D152" s="0" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F152" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="H152" s="1"/>
+        <v>88</v>
+      </c>
+      <c r="H152" s="0" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C153" s="1"/>
+        <v>89</v>
+      </c>
+      <c r="C153" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="D153" s="0" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F153" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
+      </c>
+      <c r="H153" s="0" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6503,16 +6866,14 @@
         <v>150</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C154" s="1" t="s">
-        <v>19</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="C154" s="1"/>
       <c r="D154" s="0" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F154" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6520,14 +6881,19 @@
         <v>150</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C155" s="1"/>
+        <v>93</v>
+      </c>
+      <c r="C155" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="D155" s="0" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F155" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
+      </c>
+      <c r="H155" s="0" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6535,47 +6901,48 @@
         <v>150</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D156" s="0" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F156" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B157" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C157" s="1" t="s">
-        <v>2</v>
+      <c r="B157" s="0" t="s">
+        <v>144</v>
       </c>
       <c r="D157" s="0" t="n">
-        <v>37</v>
-      </c>
-      <c r="F157" s="1" t="s">
-        <v>96</v>
+        <v>38</v>
+      </c>
+      <c r="F157" s="0" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B158" s="0" t="s">
-        <v>144</v>
-      </c>
+      <c r="B158" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C158" s="1"/>
       <c r="D158" s="0" t="n">
-        <v>38</v>
-      </c>
-      <c r="F158" s="0" t="s">
-        <v>145</v>
+        <v>39</v>
+      </c>
+      <c r="F158" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="H158" s="0" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6583,14 +6950,16 @@
         <v>150</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C159" s="1"/>
+        <v>99</v>
+      </c>
+      <c r="C159" s="1" t="s">
+        <v>2</v>
+      </c>
       <c r="D159" s="0" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F159" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6598,16 +6967,16 @@
         <v>150</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D160" s="0" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F160" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6615,16 +6984,16 @@
         <v>150</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D161" s="0" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F161" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6632,16 +7001,16 @@
         <v>150</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D162" s="0" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F162" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6649,16 +7018,16 @@
         <v>150</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D163" s="0" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F163" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6666,16 +7035,16 @@
         <v>150</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D164" s="0" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F164" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6683,16 +7052,16 @@
         <v>150</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D165" s="0" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F165" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6700,16 +7069,16 @@
         <v>150</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D166" s="0" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F166" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6717,16 +7086,16 @@
         <v>150</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C167" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D167" s="0" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F167" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6734,16 +7103,14 @@
         <v>150</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C168" s="1" t="s">
-        <v>2</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="C168" s="1"/>
       <c r="D168" s="0" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F168" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6751,106 +7118,114 @@
         <v>150</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="C169" s="1"/>
+        <v>119</v>
+      </c>
+      <c r="C169" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="D169" s="0" t="n">
-        <v>49</v>
-      </c>
-      <c r="F169" s="1" t="s">
-        <v>118</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="F169" s="1"/>
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C170" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D170" s="0" t="n">
-        <v>50</v>
-      </c>
-      <c r="F170" s="1"/>
+        <v>51</v>
+      </c>
+      <c r="F170" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="H170" s="0" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C171" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D171" s="0" t="n">
-        <v>51</v>
-      </c>
-      <c r="F171" s="1" t="s">
-        <v>121</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="F171" s="1"/>
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D172" s="0" t="n">
-        <v>52</v>
-      </c>
-      <c r="F172" s="1"/>
+        <v>53</v>
+      </c>
+      <c r="F172" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="H172" s="0" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C173" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D173" s="0" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F173" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
+      </c>
+      <c r="H173" s="0" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B174" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C174" s="1" t="s">
-        <v>5</v>
+      <c r="B174" s="0" t="s">
+        <v>149</v>
       </c>
       <c r="D174" s="0" t="n">
-        <v>54</v>
-      </c>
-      <c r="F174" s="1" t="s">
-        <v>126</v>
+        <v>55</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B175" s="0" t="s">
-        <v>149</v>
+        <v>1</v>
       </c>
       <c r="D175" s="0" t="n">
-        <v>55</v>
+        <v>1</v>
+      </c>
+      <c r="E175" s="0" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6858,13 +7233,10 @@
         <v>153</v>
       </c>
       <c r="B176" s="0" t="s">
-        <v>1</v>
+        <v>154</v>
       </c>
       <c r="D176" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E176" s="0" t="s">
-        <v>188</v>
+        <v>2</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6872,10 +7244,13 @@
         <v>153</v>
       </c>
       <c r="B177" s="0" t="s">
-        <v>154</v>
+        <v>129</v>
       </c>
       <c r="D177" s="0" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="F177" s="0" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6883,13 +7258,13 @@
         <v>153</v>
       </c>
       <c r="B178" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D178" s="0" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F178" s="0" t="s">
-        <v>222</v>
+        <v>263</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6897,13 +7272,13 @@
         <v>153</v>
       </c>
       <c r="B179" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D179" s="0" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F179" s="0" t="s">
-        <v>223</v>
+        <v>132</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6911,41 +7286,38 @@
         <v>153</v>
       </c>
       <c r="B180" s="0" t="s">
-        <v>131</v>
+        <v>13</v>
       </c>
       <c r="D180" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="F180" s="0" t="s">
-        <v>132</v>
+        <v>6</v>
+      </c>
+      <c r="F180" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B181" s="0" t="s">
-        <v>13</v>
+      <c r="B181" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="D181" s="0" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F181" s="1" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B182" s="1" t="s">
-        <v>44</v>
+      <c r="B182" s="0" t="s">
+        <v>155</v>
       </c>
       <c r="D182" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="F182" s="1" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6953,10 +7325,10 @@
         <v>153</v>
       </c>
       <c r="B183" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D183" s="0" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6964,10 +7336,10 @@
         <v>153</v>
       </c>
       <c r="B184" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D184" s="0" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6975,10 +7347,10 @@
         <v>153</v>
       </c>
       <c r="B185" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D185" s="0" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6986,10 +7358,10 @@
         <v>153</v>
       </c>
       <c r="B186" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D186" s="0" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6997,10 +7369,10 @@
         <v>153</v>
       </c>
       <c r="B187" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D187" s="0" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7008,10 +7380,10 @@
         <v>153</v>
       </c>
       <c r="B188" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D188" s="0" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7019,10 +7391,10 @@
         <v>153</v>
       </c>
       <c r="B189" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D189" s="0" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7030,10 +7402,10 @@
         <v>153</v>
       </c>
       <c r="B190" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D190" s="0" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7041,34 +7413,23 @@
         <v>153</v>
       </c>
       <c r="B191" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D191" s="0" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A192" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="B192" s="0" t="s">
-        <v>164</v>
-      </c>
-      <c r="D192" s="0" t="n">
         <v>19</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" operator="between" prompt="The importer only looks at the trailing &quot;/ Number&quot; part of this text to match it with something in the database." promptTitle="Drop-down list" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C66 C71 C73:C95 C97:C102 C104:C119 C121:C122 C130:C157 C159:C174" type="list">
+    <dataValidation allowBlank="true" operator="between" prompt="The importer only looks at the trailing &quot;/ Number&quot; part of this text to match it with something in the database." promptTitle="Drop-down list" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C66 C71 C73:C94 C96:C101 C103:C118 C120:C121 C129:C156 C158:C173" type="list">
       <formula1>_Lists!$C$2:$C$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" prompt="The importer only looks at the trailing &quot;/ Number&quot; part of this text to match it with something in the database." promptTitle="Drop-down list" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G64 G74:G95 G97:G102 G104:G119 G130:G157 G159:G174" type="list">
+    <dataValidation allowBlank="true" operator="between" prompt="The importer only looks at the trailing &quot;/ Number&quot; part of this text to match it with something in the database." promptTitle="Drop-down list" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G64 G73:G94 G96:G101 G103:G118 G128:G156 G158:G173" type="list">
       <formula1>_Lists!$D$2:$D$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A192" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A191" type="list">
       <formula1>_Lists!$B$2:$B$7</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Added support for column behaviours and adding new values to multi-value columns.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@44957 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1462" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1462" uniqueCount="270">
   <si>
     <t xml:space="preserve">Outcrop / 2</t>
   </si>
@@ -643,6 +643,9 @@
   </si>
   <si>
     <t xml:space="preserve">What is the accuracy of the date?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLLECTOR_NAME</t>
   </si>
   <si>
     <t xml:space="preserve">#COLLECTOR$PERSON_ID$NAME</t>
@@ -4298,14 +4301,17 @@
       <c r="D20" s="0" t="n">
         <v>19</v>
       </c>
+      <c r="E20" s="0" t="s">
+        <v>207</v>
+      </c>
       <c r="F20" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G20" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4323,7 +4329,7 @@
         <v>52</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4343,7 +4349,7 @@
         <v>54</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4360,10 +4366,10 @@
         <v>22</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4380,13 +4386,13 @@
         <v>23</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G24" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4403,10 +4409,10 @@
         <v>24</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4423,7 +4429,7 @@
         <v>25</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4443,7 +4449,7 @@
         <v>64</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4463,7 +4469,7 @@
         <v>66</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4483,7 +4489,7 @@
         <v>68</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4503,7 +4509,7 @@
         <v>70</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4523,7 +4529,7 @@
         <v>72</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4543,7 +4549,7 @@
         <v>74</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4560,11 +4566,11 @@
         <v>32</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F33" s="1"/>
       <c r="H33" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4572,7 +4578,7 @@
         <v>0</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>2</v>
@@ -4581,11 +4587,11 @@
         <v>33</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F34" s="1"/>
       <c r="H34" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4593,7 +4599,7 @@
         <v>0</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>5</v>
@@ -4602,11 +4608,11 @@
         <v>34</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F35" s="1"/>
       <c r="H35" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4614,7 +4620,7 @@
         <v>0</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>2</v>
@@ -4623,11 +4629,11 @@
         <v>35</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F36" s="1"/>
       <c r="H36" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4635,7 +4641,7 @@
         <v>0</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>5</v>
@@ -4644,11 +4650,11 @@
         <v>36</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F37" s="1"/>
       <c r="H37" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4656,7 +4662,7 @@
         <v>0</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>2</v>
@@ -4665,11 +4671,11 @@
         <v>37</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F38" s="1"/>
       <c r="H38" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4677,7 +4683,7 @@
         <v>0</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>5</v>
@@ -4686,11 +4692,11 @@
         <v>38</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F39" s="1"/>
       <c r="H39" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4698,7 +4704,7 @@
         <v>0</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>2</v>
@@ -4707,11 +4713,11 @@
         <v>39</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F40" s="1"/>
       <c r="H40" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4719,7 +4725,7 @@
         <v>0</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>2</v>
@@ -4728,13 +4734,13 @@
         <v>40</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4757,7 +4763,7 @@
         <v>84</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4777,7 +4783,7 @@
         <v>86</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4795,7 +4801,7 @@
         <v>88</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4813,7 +4819,7 @@
         <v>90</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4848,7 +4854,7 @@
         <v>94</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4883,7 +4889,7 @@
         <v>98</v>
       </c>
       <c r="H49" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5046,9 +5052,7 @@
       <c r="B59" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C59" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="C59" s="1"/>
       <c r="D59" s="0" t="n">
         <v>58</v>
       </c>
@@ -5088,7 +5092,7 @@
         <v>121</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5123,7 +5127,7 @@
         <v>124</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5143,7 +5147,7 @@
         <v>126</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5184,7 +5188,7 @@
       </c>
       <c r="F66" s="1"/>
       <c r="H66" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5218,10 +5222,10 @@
         <v>4</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="H68" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5235,10 +5239,10 @@
         <v>5</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="H69" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5255,7 +5259,7 @@
         <v>132</v>
       </c>
       <c r="H70" s="0" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5309,13 +5313,13 @@
         <v>10</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G73" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5333,7 +5337,7 @@
         <v>52</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5353,7 +5357,7 @@
         <v>54</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5370,13 +5374,13 @@
         <v>13</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G76" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H76" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5393,13 +5397,13 @@
         <v>14</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G77" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H77" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5416,13 +5420,13 @@
         <v>15</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G78" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H78" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5439,7 +5443,7 @@
         <v>16</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G79" s="0" t="s">
         <v>176</v>
@@ -5462,7 +5466,7 @@
         <v>64</v>
       </c>
       <c r="H80" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5482,7 +5486,7 @@
         <v>66</v>
       </c>
       <c r="H81" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5502,7 +5506,7 @@
         <v>68</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5522,7 +5526,7 @@
         <v>70</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5542,7 +5546,7 @@
         <v>72</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5562,7 +5566,7 @@
         <v>74</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5579,11 +5583,11 @@
         <v>23</v>
       </c>
       <c r="E86" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F86" s="1"/>
       <c r="H86" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5591,7 +5595,7 @@
         <v>127</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>2</v>
@@ -5600,11 +5604,11 @@
         <v>24</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F87" s="1"/>
       <c r="H87" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5612,7 +5616,7 @@
         <v>127</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>5</v>
@@ -5621,11 +5625,11 @@
         <v>25</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F88" s="1"/>
       <c r="H88" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5633,7 +5637,7 @@
         <v>127</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>2</v>
@@ -5642,11 +5646,11 @@
         <v>26</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F89" s="1"/>
       <c r="H89" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5654,7 +5658,7 @@
         <v>127</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>5</v>
@@ -5663,11 +5667,11 @@
         <v>27</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F90" s="1"/>
       <c r="H90" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5675,7 +5679,7 @@
         <v>127</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>2</v>
@@ -5684,11 +5688,11 @@
         <v>28</v>
       </c>
       <c r="E91" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F91" s="1"/>
       <c r="H91" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5696,7 +5700,7 @@
         <v>127</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>5</v>
@@ -5705,11 +5709,11 @@
         <v>29</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F92" s="1"/>
       <c r="H92" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5717,7 +5721,7 @@
         <v>127</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>2</v>
@@ -5726,11 +5730,11 @@
         <v>30</v>
       </c>
       <c r="E93" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F93" s="1"/>
       <c r="H93" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5738,7 +5742,7 @@
         <v>127</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>2</v>
@@ -5747,13 +5751,13 @@
         <v>31</v>
       </c>
       <c r="E94" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H94" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5773,7 +5777,7 @@
         <v>84</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5793,7 +5797,7 @@
         <v>86</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5811,7 +5815,7 @@
         <v>88</v>
       </c>
       <c r="H97" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5831,7 +5835,7 @@
         <v>90</v>
       </c>
       <c r="H98" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5866,7 +5870,7 @@
         <v>94</v>
       </c>
       <c r="H100" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5915,7 +5919,7 @@
         <v>98</v>
       </c>
       <c r="H103" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6118,7 +6122,7 @@
         <v>121</v>
       </c>
       <c r="H115" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6153,7 +6157,7 @@
         <v>124</v>
       </c>
       <c r="H117" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6173,7 +6177,7 @@
         <v>126</v>
       </c>
       <c r="H118" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6187,7 +6191,7 @@
         <v>56</v>
       </c>
       <c r="H119" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6228,7 +6232,7 @@
       </c>
       <c r="F121" s="1"/>
       <c r="H121" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6242,7 +6246,7 @@
         <v>3</v>
       </c>
       <c r="F122" s="0" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="H122" s="1" t="s">
         <v>193</v>
@@ -6259,10 +6263,10 @@
         <v>4</v>
       </c>
       <c r="F123" s="0" t="s">
+        <v>264</v>
+      </c>
+      <c r="H123" s="0" t="s">
         <v>263</v>
-      </c>
-      <c r="H123" s="0" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6279,7 +6283,7 @@
         <v>132</v>
       </c>
       <c r="H124" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6293,10 +6297,10 @@
         <v>6</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H125" s="0" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6344,13 +6348,13 @@
         <v>9</v>
       </c>
       <c r="F128" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G128" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H128" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6386,7 +6390,7 @@
         <v>54</v>
       </c>
       <c r="H130" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6403,10 +6407,10 @@
         <v>12</v>
       </c>
       <c r="F131" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H131" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6423,13 +6427,13 @@
         <v>13</v>
       </c>
       <c r="F132" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G132" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H132" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6446,10 +6450,10 @@
         <v>14</v>
       </c>
       <c r="F133" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H133" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6466,7 +6470,7 @@
         <v>15</v>
       </c>
       <c r="F134" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6486,7 +6490,7 @@
         <v>64</v>
       </c>
       <c r="H135" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6506,7 +6510,7 @@
         <v>66</v>
       </c>
       <c r="H136" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6526,7 +6530,7 @@
         <v>68</v>
       </c>
       <c r="H137" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6546,7 +6550,7 @@
         <v>70</v>
       </c>
       <c r="H138" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6566,7 +6570,7 @@
         <v>72</v>
       </c>
       <c r="H139" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6586,7 +6590,7 @@
         <v>74</v>
       </c>
       <c r="H140" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6603,11 +6607,11 @@
         <v>22</v>
       </c>
       <c r="E141" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F141" s="1"/>
       <c r="H141" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6615,7 +6619,7 @@
         <v>150</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C142" s="1" t="s">
         <v>2</v>
@@ -6624,11 +6628,11 @@
         <v>23</v>
       </c>
       <c r="E142" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F142" s="1"/>
       <c r="H142" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6636,7 +6640,7 @@
         <v>150</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C143" s="1" t="s">
         <v>5</v>
@@ -6645,11 +6649,11 @@
         <v>24</v>
       </c>
       <c r="E143" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F143" s="1"/>
       <c r="H143" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6657,7 +6661,7 @@
         <v>150</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>2</v>
@@ -6666,11 +6670,11 @@
         <v>25</v>
       </c>
       <c r="E144" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F144" s="1"/>
       <c r="H144" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6678,7 +6682,7 @@
         <v>150</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>5</v>
@@ -6687,11 +6691,11 @@
         <v>26</v>
       </c>
       <c r="E145" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F145" s="1"/>
       <c r="H145" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6699,7 +6703,7 @@
         <v>150</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>2</v>
@@ -6708,11 +6712,11 @@
         <v>27</v>
       </c>
       <c r="E146" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F146" s="1"/>
       <c r="H146" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6720,7 +6724,7 @@
         <v>150</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>5</v>
@@ -6729,11 +6733,11 @@
         <v>28</v>
       </c>
       <c r="E147" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F147" s="1"/>
       <c r="H147" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6741,7 +6745,7 @@
         <v>150</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>2</v>
@@ -6750,11 +6754,11 @@
         <v>29</v>
       </c>
       <c r="E148" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F148" s="1"/>
       <c r="H148" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6762,7 +6766,7 @@
         <v>150</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>2</v>
@@ -6771,13 +6775,13 @@
         <v>30</v>
       </c>
       <c r="E149" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F149" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H149" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6800,7 +6804,7 @@
         <v>84</v>
       </c>
       <c r="H150" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6820,7 +6824,7 @@
         <v>86</v>
       </c>
       <c r="H151" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6838,7 +6842,7 @@
         <v>88</v>
       </c>
       <c r="H152" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6858,7 +6862,7 @@
         <v>90</v>
       </c>
       <c r="H153" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6893,7 +6897,7 @@
         <v>94</v>
       </c>
       <c r="H155" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6942,7 +6946,7 @@
         <v>98</v>
       </c>
       <c r="H158" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7145,7 +7149,7 @@
         <v>121</v>
       </c>
       <c r="H170" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7180,7 +7184,7 @@
         <v>124</v>
       </c>
       <c r="H172" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7200,7 +7204,7 @@
         <v>126</v>
       </c>
       <c r="H173" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7250,7 +7254,7 @@
         <v>3</v>
       </c>
       <c r="F177" s="0" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7264,7 +7268,7 @@
         <v>4</v>
       </c>
       <c r="F178" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Fix up the "Collector" columns.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@44958 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1462" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="271">
   <si>
     <t xml:space="preserve">Outcrop / 2</t>
   </si>
@@ -607,6 +607,9 @@
   </si>
   <si>
     <t xml:space="preserve">Choose the coordinate system you used to enter the following coordinates.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
   </si>
   <si>
     <t xml:space="preserve">Enter the easting or longitude coordinate.</t>
@@ -4048,8 +4051,8 @@
       <c r="A8" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>18</v>
+      <c r="B8" s="0" t="s">
+        <v>195</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>19</v>
@@ -4062,7 +4065,7 @@
       </c>
       <c r="F8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4083,7 +4086,7 @@
       </c>
       <c r="F9" s="1"/>
       <c r="H9" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4104,7 +4107,7 @@
       </c>
       <c r="F10" s="1"/>
       <c r="H10" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4122,7 +4125,7 @@
       </c>
       <c r="F11" s="1"/>
       <c r="H11" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4142,7 +4145,7 @@
         <v>30</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4163,7 +4166,7 @@
       </c>
       <c r="F13" s="1"/>
       <c r="H13" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4183,7 +4186,7 @@
         <v>35</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4206,7 +4209,7 @@
         <v>38</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4227,7 +4230,7 @@
       </c>
       <c r="F16" s="1"/>
       <c r="H16" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4245,7 +4248,7 @@
       </c>
       <c r="F17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4265,7 +4268,7 @@
         <v>46</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4285,7 +4288,7 @@
         <v>48</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4302,16 +4305,16 @@
         <v>19</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G20" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4329,7 +4332,7 @@
         <v>52</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4349,7 +4352,7 @@
         <v>54</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4366,10 +4369,10 @@
         <v>22</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4386,13 +4389,13 @@
         <v>23</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G24" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4409,10 +4412,10 @@
         <v>24</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4429,7 +4432,7 @@
         <v>25</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4449,7 +4452,7 @@
         <v>64</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4469,7 +4472,7 @@
         <v>66</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4489,7 +4492,7 @@
         <v>68</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4509,7 +4512,7 @@
         <v>70</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4529,7 +4532,7 @@
         <v>72</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4549,7 +4552,7 @@
         <v>74</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4566,11 +4569,11 @@
         <v>32</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F33" s="1"/>
       <c r="H33" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4578,7 +4581,7 @@
         <v>0</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>2</v>
@@ -4587,11 +4590,11 @@
         <v>33</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F34" s="1"/>
       <c r="H34" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4599,7 +4602,7 @@
         <v>0</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>5</v>
@@ -4608,11 +4611,11 @@
         <v>34</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F35" s="1"/>
       <c r="H35" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4620,7 +4623,7 @@
         <v>0</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>2</v>
@@ -4629,11 +4632,11 @@
         <v>35</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F36" s="1"/>
       <c r="H36" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4641,7 +4644,7 @@
         <v>0</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>5</v>
@@ -4650,11 +4653,11 @@
         <v>36</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F37" s="1"/>
       <c r="H37" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4662,7 +4665,7 @@
         <v>0</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>2</v>
@@ -4671,11 +4674,11 @@
         <v>37</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F38" s="1"/>
       <c r="H38" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4683,7 +4686,7 @@
         <v>0</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>5</v>
@@ -4692,11 +4695,11 @@
         <v>38</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F39" s="1"/>
       <c r="H39" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4704,7 +4707,7 @@
         <v>0</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>2</v>
@@ -4713,11 +4716,11 @@
         <v>39</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F40" s="1"/>
       <c r="H40" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4725,7 +4728,7 @@
         <v>0</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>2</v>
@@ -4734,13 +4737,13 @@
         <v>40</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4763,7 +4766,7 @@
         <v>84</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4783,7 +4786,7 @@
         <v>86</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4801,7 +4804,7 @@
         <v>88</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4819,7 +4822,7 @@
         <v>90</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4854,7 +4857,7 @@
         <v>94</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4889,7 +4892,7 @@
         <v>98</v>
       </c>
       <c r="H49" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5092,7 +5095,7 @@
         <v>121</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5127,7 +5130,7 @@
         <v>124</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5147,7 +5150,7 @@
         <v>126</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5188,7 +5191,7 @@
       </c>
       <c r="F66" s="1"/>
       <c r="H66" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5222,10 +5225,10 @@
         <v>4</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H68" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5239,10 +5242,10 @@
         <v>5</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H69" s="0" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5259,7 +5262,7 @@
         <v>132</v>
       </c>
       <c r="H70" s="0" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5279,7 +5282,7 @@
         <v>46</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5296,7 +5299,7 @@
         <v>48</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5312,14 +5315,17 @@
       <c r="D73" s="0" t="n">
         <v>10</v>
       </c>
+      <c r="E73" s="0" t="s">
+        <v>208</v>
+      </c>
       <c r="F73" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G73" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5337,7 +5343,7 @@
         <v>52</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5357,7 +5363,7 @@
         <v>54</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5374,13 +5380,13 @@
         <v>13</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G76" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H76" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5397,13 +5403,13 @@
         <v>14</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G77" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H77" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5420,13 +5426,13 @@
         <v>15</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G78" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H78" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5443,7 +5449,7 @@
         <v>16</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G79" s="0" t="s">
         <v>176</v>
@@ -5466,7 +5472,7 @@
         <v>64</v>
       </c>
       <c r="H80" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5486,7 +5492,7 @@
         <v>66</v>
       </c>
       <c r="H81" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5506,7 +5512,7 @@
         <v>68</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5526,7 +5532,7 @@
         <v>70</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5546,7 +5552,7 @@
         <v>72</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5566,7 +5572,7 @@
         <v>74</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5583,11 +5589,11 @@
         <v>23</v>
       </c>
       <c r="E86" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F86" s="1"/>
       <c r="H86" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5595,7 +5601,7 @@
         <v>127</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>2</v>
@@ -5604,11 +5610,11 @@
         <v>24</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F87" s="1"/>
       <c r="H87" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5616,7 +5622,7 @@
         <v>127</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>5</v>
@@ -5625,11 +5631,11 @@
         <v>25</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F88" s="1"/>
       <c r="H88" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5637,7 +5643,7 @@
         <v>127</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>2</v>
@@ -5646,11 +5652,11 @@
         <v>26</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F89" s="1"/>
       <c r="H89" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5658,7 +5664,7 @@
         <v>127</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>5</v>
@@ -5667,11 +5673,11 @@
         <v>27</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F90" s="1"/>
       <c r="H90" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5679,7 +5685,7 @@
         <v>127</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>2</v>
@@ -5688,11 +5694,11 @@
         <v>28</v>
       </c>
       <c r="E91" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F91" s="1"/>
       <c r="H91" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5700,7 +5706,7 @@
         <v>127</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>5</v>
@@ -5709,11 +5715,11 @@
         <v>29</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F92" s="1"/>
       <c r="H92" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5721,7 +5727,7 @@
         <v>127</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>2</v>
@@ -5730,11 +5736,11 @@
         <v>30</v>
       </c>
       <c r="E93" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F93" s="1"/>
       <c r="H93" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5742,7 +5748,7 @@
         <v>127</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>2</v>
@@ -5751,13 +5757,13 @@
         <v>31</v>
       </c>
       <c r="E94" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H94" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5777,7 +5783,7 @@
         <v>84</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5797,7 +5803,7 @@
         <v>86</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5815,7 +5821,7 @@
         <v>88</v>
       </c>
       <c r="H97" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5835,7 +5841,7 @@
         <v>90</v>
       </c>
       <c r="H98" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5870,7 +5876,7 @@
         <v>94</v>
       </c>
       <c r="H100" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5919,7 +5925,7 @@
         <v>98</v>
       </c>
       <c r="H103" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6122,7 +6128,7 @@
         <v>121</v>
       </c>
       <c r="H115" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6157,7 +6163,7 @@
         <v>124</v>
       </c>
       <c r="H117" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6177,7 +6183,7 @@
         <v>126</v>
       </c>
       <c r="H118" s="0" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6191,7 +6197,7 @@
         <v>56</v>
       </c>
       <c r="H119" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6232,7 +6238,7 @@
       </c>
       <c r="F121" s="1"/>
       <c r="H121" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6246,7 +6252,7 @@
         <v>3</v>
       </c>
       <c r="F122" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H122" s="1" t="s">
         <v>193</v>
@@ -6263,10 +6269,10 @@
         <v>4</v>
       </c>
       <c r="F123" s="0" t="s">
+        <v>265</v>
+      </c>
+      <c r="H123" s="0" t="s">
         <v>264</v>
-      </c>
-      <c r="H123" s="0" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6283,7 +6289,7 @@
         <v>132</v>
       </c>
       <c r="H124" s="0" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6297,10 +6303,10 @@
         <v>6</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="H125" s="0" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6317,7 +6323,7 @@
         <v>46</v>
       </c>
       <c r="H126" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6334,7 +6340,7 @@
         <v>48</v>
       </c>
       <c r="H127" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6347,14 +6353,17 @@
       <c r="D128" s="0" t="n">
         <v>9</v>
       </c>
+      <c r="E128" s="0" t="s">
+        <v>208</v>
+      </c>
       <c r="F128" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G128" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H128" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6390,7 +6399,7 @@
         <v>54</v>
       </c>
       <c r="H130" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6407,10 +6416,10 @@
         <v>12</v>
       </c>
       <c r="F131" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H131" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6427,13 +6436,13 @@
         <v>13</v>
       </c>
       <c r="F132" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G132" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H132" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6450,10 +6459,10 @@
         <v>14</v>
       </c>
       <c r="F133" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H133" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6470,7 +6479,7 @@
         <v>15</v>
       </c>
       <c r="F134" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6490,7 +6499,7 @@
         <v>64</v>
       </c>
       <c r="H135" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6510,7 +6519,7 @@
         <v>66</v>
       </c>
       <c r="H136" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6530,7 +6539,7 @@
         <v>68</v>
       </c>
       <c r="H137" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6550,7 +6559,7 @@
         <v>70</v>
       </c>
       <c r="H138" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6570,7 +6579,7 @@
         <v>72</v>
       </c>
       <c r="H139" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6590,7 +6599,7 @@
         <v>74</v>
       </c>
       <c r="H140" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6607,11 +6616,11 @@
         <v>22</v>
       </c>
       <c r="E141" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F141" s="1"/>
       <c r="H141" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6619,7 +6628,7 @@
         <v>150</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C142" s="1" t="s">
         <v>2</v>
@@ -6628,11 +6637,11 @@
         <v>23</v>
       </c>
       <c r="E142" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F142" s="1"/>
       <c r="H142" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6640,7 +6649,7 @@
         <v>150</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C143" s="1" t="s">
         <v>5</v>
@@ -6649,11 +6658,11 @@
         <v>24</v>
       </c>
       <c r="E143" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F143" s="1"/>
       <c r="H143" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6661,7 +6670,7 @@
         <v>150</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>2</v>
@@ -6670,11 +6679,11 @@
         <v>25</v>
       </c>
       <c r="E144" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F144" s="1"/>
       <c r="H144" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6682,7 +6691,7 @@
         <v>150</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>5</v>
@@ -6691,11 +6700,11 @@
         <v>26</v>
       </c>
       <c r="E145" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F145" s="1"/>
       <c r="H145" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6703,7 +6712,7 @@
         <v>150</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>2</v>
@@ -6712,11 +6721,11 @@
         <v>27</v>
       </c>
       <c r="E146" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F146" s="1"/>
       <c r="H146" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6724,7 +6733,7 @@
         <v>150</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>5</v>
@@ -6733,11 +6742,11 @@
         <v>28</v>
       </c>
       <c r="E147" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F147" s="1"/>
       <c r="H147" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6745,7 +6754,7 @@
         <v>150</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>2</v>
@@ -6754,11 +6763,11 @@
         <v>29</v>
       </c>
       <c r="E148" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F148" s="1"/>
       <c r="H148" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6766,7 +6775,7 @@
         <v>150</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>2</v>
@@ -6775,13 +6784,13 @@
         <v>30</v>
       </c>
       <c r="E149" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F149" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H149" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6804,7 +6813,7 @@
         <v>84</v>
       </c>
       <c r="H150" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6824,7 +6833,7 @@
         <v>86</v>
       </c>
       <c r="H151" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6842,7 +6851,7 @@
         <v>88</v>
       </c>
       <c r="H152" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6862,7 +6871,7 @@
         <v>90</v>
       </c>
       <c r="H153" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6897,7 +6906,7 @@
         <v>94</v>
       </c>
       <c r="H155" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6946,7 +6955,7 @@
         <v>98</v>
       </c>
       <c r="H158" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7149,7 +7158,7 @@
         <v>121</v>
       </c>
       <c r="H170" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7184,7 +7193,7 @@
         <v>124</v>
       </c>
       <c r="H172" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7204,7 +7213,7 @@
         <v>126</v>
       </c>
       <c r="H173" s="0" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7254,7 +7263,7 @@
         <v>3</v>
       </c>
       <c r="F177" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7268,7 +7277,7 @@
         <v>4</v>
       </c>
       <c r="F178" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Integrate FRED import into FRED. PDP-202.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45013 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="270">
   <si>
     <t xml:space="preserve">Outcrop / 2</t>
   </si>
@@ -607,9 +607,6 @@
   </si>
   <si>
     <t xml:space="preserve">Choose the coordinate system you used to enter the following coordinates.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C</t>
   </si>
   <si>
     <t xml:space="preserve">Enter the easting or longitude coordinate.</t>
@@ -4052,7 +4049,7 @@
         <v>0</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>195</v>
+        <v>18</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>19</v>
@@ -4065,7 +4062,7 @@
       </c>
       <c r="F8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4086,7 +4083,7 @@
       </c>
       <c r="F9" s="1"/>
       <c r="H9" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4107,7 +4104,7 @@
       </c>
       <c r="F10" s="1"/>
       <c r="H10" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4125,7 +4122,7 @@
       </c>
       <c r="F11" s="1"/>
       <c r="H11" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4145,7 +4142,7 @@
         <v>30</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4166,7 +4163,7 @@
       </c>
       <c r="F13" s="1"/>
       <c r="H13" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4186,7 +4183,7 @@
         <v>35</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4209,7 +4206,7 @@
         <v>38</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4230,7 +4227,7 @@
       </c>
       <c r="F16" s="1"/>
       <c r="H16" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4248,7 +4245,7 @@
       </c>
       <c r="F17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4268,7 +4265,7 @@
         <v>46</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4288,7 +4285,7 @@
         <v>48</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4305,16 +4302,16 @@
         <v>19</v>
       </c>
       <c r="E20" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>208</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>209</v>
       </c>
       <c r="G20" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4332,7 +4329,7 @@
         <v>52</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4352,7 +4349,7 @@
         <v>54</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4369,10 +4366,10 @@
         <v>22</v>
       </c>
       <c r="F23" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="H23" s="0" t="s">
         <v>213</v>
-      </c>
-      <c r="H23" s="0" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4389,13 +4386,13 @@
         <v>23</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G24" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4412,10 +4409,10 @@
         <v>24</v>
       </c>
       <c r="F25" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="H25" s="0" t="s">
         <v>217</v>
-      </c>
-      <c r="H25" s="0" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4432,7 +4429,7 @@
         <v>25</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4452,7 +4449,7 @@
         <v>64</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4472,7 +4469,7 @@
         <v>66</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4492,7 +4489,7 @@
         <v>68</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4512,7 +4509,7 @@
         <v>70</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4532,7 +4529,7 @@
         <v>72</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4552,7 +4549,7 @@
         <v>74</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4569,11 +4566,11 @@
         <v>32</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F33" s="1"/>
       <c r="H33" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4581,7 +4578,7 @@
         <v>0</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>2</v>
@@ -4590,11 +4587,11 @@
         <v>33</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F34" s="1"/>
       <c r="H34" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4602,7 +4599,7 @@
         <v>0</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>5</v>
@@ -4611,11 +4608,11 @@
         <v>34</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F35" s="1"/>
       <c r="H35" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4623,7 +4620,7 @@
         <v>0</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>2</v>
@@ -4632,11 +4629,11 @@
         <v>35</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F36" s="1"/>
       <c r="H36" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4644,7 +4641,7 @@
         <v>0</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>5</v>
@@ -4653,11 +4650,11 @@
         <v>36</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F37" s="1"/>
       <c r="H37" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4665,7 +4662,7 @@
         <v>0</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>2</v>
@@ -4674,11 +4671,11 @@
         <v>37</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F38" s="1"/>
       <c r="H38" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4686,7 +4683,7 @@
         <v>0</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>5</v>
@@ -4695,11 +4692,11 @@
         <v>38</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F39" s="1"/>
       <c r="H39" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4707,7 +4704,7 @@
         <v>0</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>2</v>
@@ -4716,11 +4713,11 @@
         <v>39</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F40" s="1"/>
       <c r="H40" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4728,7 +4725,7 @@
         <v>0</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>2</v>
@@ -4737,13 +4734,13 @@
         <v>40</v>
       </c>
       <c r="E41" s="0" t="s">
+        <v>249</v>
+      </c>
+      <c r="F41" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="H41" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="H41" s="1" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4766,7 +4763,7 @@
         <v>84</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4786,7 +4783,7 @@
         <v>86</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4804,7 +4801,7 @@
         <v>88</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4822,7 +4819,7 @@
         <v>90</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4857,7 +4854,7 @@
         <v>94</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4892,7 +4889,7 @@
         <v>98</v>
       </c>
       <c r="H49" s="0" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5095,7 +5092,7 @@
         <v>121</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5130,7 +5127,7 @@
         <v>124</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5150,7 +5147,7 @@
         <v>126</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5191,7 +5188,7 @@
       </c>
       <c r="F66" s="1"/>
       <c r="H66" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5225,10 +5222,10 @@
         <v>4</v>
       </c>
       <c r="F68" s="0" t="s">
+        <v>262</v>
+      </c>
+      <c r="H68" s="0" t="s">
         <v>263</v>
-      </c>
-      <c r="H68" s="0" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5242,10 +5239,10 @@
         <v>5</v>
       </c>
       <c r="F69" s="0" t="s">
+        <v>264</v>
+      </c>
+      <c r="H69" s="0" t="s">
         <v>265</v>
-      </c>
-      <c r="H69" s="0" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5262,7 +5259,7 @@
         <v>132</v>
       </c>
       <c r="H70" s="0" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5282,7 +5279,7 @@
         <v>46</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5299,7 +5296,7 @@
         <v>48</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5316,16 +5313,16 @@
         <v>10</v>
       </c>
       <c r="E73" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="F73" s="1" t="s">
         <v>208</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>209</v>
       </c>
       <c r="G73" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5343,7 +5340,7 @@
         <v>52</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5363,7 +5360,7 @@
         <v>54</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5380,13 +5377,13 @@
         <v>13</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G76" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H76" s="0" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5403,13 +5400,13 @@
         <v>14</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G77" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H77" s="0" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5426,13 +5423,13 @@
         <v>15</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G78" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H78" s="0" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5449,7 +5446,7 @@
         <v>16</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G79" s="0" t="s">
         <v>176</v>
@@ -5472,7 +5469,7 @@
         <v>64</v>
       </c>
       <c r="H80" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5492,7 +5489,7 @@
         <v>66</v>
       </c>
       <c r="H81" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5512,7 +5509,7 @@
         <v>68</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5532,7 +5529,7 @@
         <v>70</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5552,7 +5549,7 @@
         <v>72</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5572,7 +5569,7 @@
         <v>74</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5589,11 +5586,11 @@
         <v>23</v>
       </c>
       <c r="E86" s="0" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F86" s="1"/>
       <c r="H86" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5601,7 +5598,7 @@
         <v>127</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>2</v>
@@ -5610,11 +5607,11 @@
         <v>24</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F87" s="1"/>
       <c r="H87" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5622,7 +5619,7 @@
         <v>127</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>5</v>
@@ -5631,11 +5628,11 @@
         <v>25</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F88" s="1"/>
       <c r="H88" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5643,7 +5640,7 @@
         <v>127</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>2</v>
@@ -5652,11 +5649,11 @@
         <v>26</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F89" s="1"/>
       <c r="H89" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5664,7 +5661,7 @@
         <v>127</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>5</v>
@@ -5673,11 +5670,11 @@
         <v>27</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F90" s="1"/>
       <c r="H90" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5685,7 +5682,7 @@
         <v>127</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>2</v>
@@ -5694,11 +5691,11 @@
         <v>28</v>
       </c>
       <c r="E91" s="0" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F91" s="1"/>
       <c r="H91" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5706,7 +5703,7 @@
         <v>127</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>5</v>
@@ -5715,11 +5712,11 @@
         <v>29</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F92" s="1"/>
       <c r="H92" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5727,7 +5724,7 @@
         <v>127</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>2</v>
@@ -5736,11 +5733,11 @@
         <v>30</v>
       </c>
       <c r="E93" s="0" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F93" s="1"/>
       <c r="H93" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5748,7 +5745,7 @@
         <v>127</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>2</v>
@@ -5757,13 +5754,13 @@
         <v>31</v>
       </c>
       <c r="E94" s="0" t="s">
+        <v>249</v>
+      </c>
+      <c r="F94" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="F94" s="1" t="s">
+      <c r="H94" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="H94" s="1" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5783,7 +5780,7 @@
         <v>84</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5803,7 +5800,7 @@
         <v>86</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5821,7 +5818,7 @@
         <v>88</v>
       </c>
       <c r="H97" s="0" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5841,7 +5838,7 @@
         <v>90</v>
       </c>
       <c r="H98" s="0" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5876,7 +5873,7 @@
         <v>94</v>
       </c>
       <c r="H100" s="0" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5925,7 +5922,7 @@
         <v>98</v>
       </c>
       <c r="H103" s="0" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6128,7 +6125,7 @@
         <v>121</v>
       </c>
       <c r="H115" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6163,7 +6160,7 @@
         <v>124</v>
       </c>
       <c r="H117" s="0" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6183,7 +6180,7 @@
         <v>126</v>
       </c>
       <c r="H118" s="0" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6197,7 +6194,7 @@
         <v>56</v>
       </c>
       <c r="H119" s="0" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6238,7 +6235,7 @@
       </c>
       <c r="F121" s="1"/>
       <c r="H121" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6252,7 +6249,7 @@
         <v>3</v>
       </c>
       <c r="F122" s="0" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H122" s="1" t="s">
         <v>193</v>
@@ -6269,10 +6266,10 @@
         <v>4</v>
       </c>
       <c r="F123" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="H123" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6289,7 +6286,7 @@
         <v>132</v>
       </c>
       <c r="H124" s="0" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6303,10 +6300,10 @@
         <v>6</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="H125" s="0" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6323,7 +6320,7 @@
         <v>46</v>
       </c>
       <c r="H126" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6340,7 +6337,7 @@
         <v>48</v>
       </c>
       <c r="H127" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6354,16 +6351,16 @@
         <v>9</v>
       </c>
       <c r="E128" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="F128" s="1" t="s">
         <v>208</v>
-      </c>
-      <c r="F128" s="1" t="s">
-        <v>209</v>
       </c>
       <c r="G128" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H128" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6399,7 +6396,7 @@
         <v>54</v>
       </c>
       <c r="H130" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6416,10 +6413,10 @@
         <v>12</v>
       </c>
       <c r="F131" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="H131" s="0" t="s">
         <v>213</v>
-      </c>
-      <c r="H131" s="0" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6436,13 +6433,13 @@
         <v>13</v>
       </c>
       <c r="F132" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G132" s="0" t="s">
         <v>176</v>
       </c>
       <c r="H132" s="0" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6459,10 +6456,10 @@
         <v>14</v>
       </c>
       <c r="F133" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="H133" s="0" t="s">
         <v>217</v>
-      </c>
-      <c r="H133" s="0" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6479,7 +6476,7 @@
         <v>15</v>
       </c>
       <c r="F134" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6499,7 +6496,7 @@
         <v>64</v>
       </c>
       <c r="H135" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6519,7 +6516,7 @@
         <v>66</v>
       </c>
       <c r="H136" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6539,7 +6536,7 @@
         <v>68</v>
       </c>
       <c r="H137" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6559,7 +6556,7 @@
         <v>70</v>
       </c>
       <c r="H138" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6579,7 +6576,7 @@
         <v>72</v>
       </c>
       <c r="H139" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6599,7 +6596,7 @@
         <v>74</v>
       </c>
       <c r="H140" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6616,11 +6613,11 @@
         <v>22</v>
       </c>
       <c r="E141" s="0" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F141" s="1"/>
       <c r="H141" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6628,7 +6625,7 @@
         <v>150</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C142" s="1" t="s">
         <v>2</v>
@@ -6637,11 +6634,11 @@
         <v>23</v>
       </c>
       <c r="E142" s="0" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F142" s="1"/>
       <c r="H142" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6649,7 +6646,7 @@
         <v>150</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C143" s="1" t="s">
         <v>5</v>
@@ -6658,11 +6655,11 @@
         <v>24</v>
       </c>
       <c r="E143" s="0" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F143" s="1"/>
       <c r="H143" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6670,7 +6667,7 @@
         <v>150</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>2</v>
@@ -6679,11 +6676,11 @@
         <v>25</v>
       </c>
       <c r="E144" s="0" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F144" s="1"/>
       <c r="H144" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6691,7 +6688,7 @@
         <v>150</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>5</v>
@@ -6700,11 +6697,11 @@
         <v>26</v>
       </c>
       <c r="E145" s="0" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F145" s="1"/>
       <c r="H145" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6712,7 +6709,7 @@
         <v>150</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>2</v>
@@ -6721,11 +6718,11 @@
         <v>27</v>
       </c>
       <c r="E146" s="0" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F146" s="1"/>
       <c r="H146" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6733,7 +6730,7 @@
         <v>150</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>5</v>
@@ -6742,11 +6739,11 @@
         <v>28</v>
       </c>
       <c r="E147" s="0" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F147" s="1"/>
       <c r="H147" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6754,7 +6751,7 @@
         <v>150</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>2</v>
@@ -6763,11 +6760,11 @@
         <v>29</v>
       </c>
       <c r="E148" s="0" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F148" s="1"/>
       <c r="H148" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6775,7 +6772,7 @@
         <v>150</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>2</v>
@@ -6784,13 +6781,13 @@
         <v>30</v>
       </c>
       <c r="E149" s="0" t="s">
+        <v>249</v>
+      </c>
+      <c r="F149" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="F149" s="1" t="s">
+      <c r="H149" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="H149" s="1" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6813,7 +6810,7 @@
         <v>84</v>
       </c>
       <c r="H150" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6833,7 +6830,7 @@
         <v>86</v>
       </c>
       <c r="H151" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6851,7 +6848,7 @@
         <v>88</v>
       </c>
       <c r="H152" s="0" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6871,7 +6868,7 @@
         <v>90</v>
       </c>
       <c r="H153" s="0" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6906,7 +6903,7 @@
         <v>94</v>
       </c>
       <c r="H155" s="0" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6955,7 +6952,7 @@
         <v>98</v>
       </c>
       <c r="H158" s="0" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7158,7 +7155,7 @@
         <v>121</v>
       </c>
       <c r="H170" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7193,7 +7190,7 @@
         <v>124</v>
       </c>
       <c r="H172" s="0" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7213,7 +7210,7 @@
         <v>126</v>
       </c>
       <c r="H173" s="0" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7263,7 +7260,7 @@
         <v>3</v>
       </c>
       <c r="F177" s="0" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7277,7 +7274,7 @@
         <v>4</v>
       </c>
       <c r="F178" s="0" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Change "Collection Date" to be dates rather than timestamps. PDB-204
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45310 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -9,7 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="_Cover sheet" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="_Lists" sheetId="2" state="hidden" r:id="rId3"/>
+    <sheet name="_Lists" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="Metaimporter" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="239">
   <si>
     <t xml:space="preserve">testExportMetaTemplate</t>
   </si>
@@ -85,6 +85,9 @@
   </si>
   <si>
     <t xml:space="preserve">Auto-increment ID / 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date / 10</t>
   </si>
   <si>
     <t xml:space="preserve">Sheet template</t>
@@ -750,6 +753,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -897,7 +901,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="1" style="0" width="16"/>
@@ -982,6 +986,11 @@
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="0" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C11" s="0" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1003,7 +1012,9 @@
   <dimension ref="A1:I191"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="76.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="11" style="0" width="8.67"/>
@@ -1011,39 +1022,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>17</v>
@@ -1052,18 +1063,18 @@
         <v>1</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>14</v>
@@ -1072,18 +1083,18 @@
         <v>2</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>17</v>
@@ -1092,18 +1103,18 @@
         <v>3</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>14</v>
@@ -1112,15 +1123,15 @@
         <v>4</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>14</v>
@@ -1129,18 +1140,18 @@
         <v>5</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>17</v>
@@ -1149,21 +1160,21 @@
         <v>6</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>11</v>
@@ -1172,18 +1183,18 @@
         <v>7</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>11</v>
@@ -1192,18 +1203,18 @@
         <v>8</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>17</v>
@@ -1212,18 +1223,18 @@
         <v>9</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I10" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>14</v>
@@ -1232,15 +1243,15 @@
         <v>10</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>7</v>
@@ -1249,18 +1260,18 @@
         <v>11</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>7</v>
@@ -1269,18 +1280,18 @@
         <v>12</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>14</v>
@@ -1289,18 +1300,18 @@
         <v>13</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>14</v>
@@ -1309,21 +1320,21 @@
         <v>14</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>17</v>
@@ -1332,18 +1343,18 @@
         <v>15</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>14</v>
@@ -1352,35 +1363,35 @@
         <v>16</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D18" s="0" t="n">
         <v>17</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>17</v>
@@ -1389,18 +1400,18 @@
         <v>18</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I19" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>17</v>
@@ -1409,42 +1420,42 @@
         <v>19</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G20" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I20" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="0" t="n">
         <v>20</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I21" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>14</v>
@@ -1453,18 +1464,18 @@
         <v>21</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>17</v>
@@ -1473,18 +1484,18 @@
         <v>22</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>17</v>
@@ -1493,21 +1504,21 @@
         <v>23</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>17</v>
@@ -1516,18 +1527,18 @@
         <v>24</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>14</v>
@@ -1536,15 +1547,15 @@
         <v>25</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>14</v>
@@ -1553,18 +1564,18 @@
         <v>26</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>14</v>
@@ -1573,18 +1584,18 @@
         <v>27</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>17</v>
@@ -1593,18 +1604,18 @@
         <v>28</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I29" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>17</v>
@@ -1613,18 +1624,18 @@
         <v>29</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>17</v>
@@ -1633,18 +1644,18 @@
         <v>30</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>17</v>
@@ -1653,18 +1664,18 @@
         <v>31</v>
       </c>
       <c r="F32" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I32" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>14</v>
@@ -1673,21 +1684,21 @@
         <v>32</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H33" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I33" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>17</v>
@@ -1696,21 +1707,21 @@
         <v>33</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H34" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>14</v>
@@ -1719,21 +1730,21 @@
         <v>34</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H35" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>17</v>
@@ -1742,21 +1753,21 @@
         <v>35</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H36" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>14</v>
@@ -1765,21 +1776,21 @@
         <v>36</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H37" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>17</v>
@@ -1788,21 +1799,21 @@
         <v>37</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H38" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>14</v>
@@ -1811,21 +1822,21 @@
         <v>38</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H39" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I39" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>17</v>
@@ -1834,21 +1845,21 @@
         <v>39</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H40" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>17</v>
@@ -1857,27 +1868,27 @@
         <v>40</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H41" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>14</v>
@@ -1886,21 +1897,21 @@
         <v>41</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I42" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>11</v>
@@ -1909,69 +1920,69 @@
         <v>42</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="0" t="n">
         <v>43</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="0" t="n">
         <v>44</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="0" t="n">
         <v>45</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>14</v>
@@ -1980,18 +1991,18 @@
         <v>46</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I47" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>17</v>
@@ -2000,33 +2011,33 @@
         <v>47</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="0" t="n">
         <v>48</v>
       </c>
       <c r="F49" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I49" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>17</v>
@@ -2035,15 +2046,15 @@
         <v>49</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>17</v>
@@ -2052,15 +2063,15 @@
         <v>50</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>17</v>
@@ -2069,15 +2080,15 @@
         <v>51</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>17</v>
@@ -2086,15 +2097,15 @@
         <v>52</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>17</v>
@@ -2103,15 +2114,15 @@
         <v>53</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>17</v>
@@ -2120,15 +2131,15 @@
         <v>54</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>17</v>
@@ -2137,15 +2148,15 @@
         <v>55</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>17</v>
@@ -2154,15 +2165,15 @@
         <v>56</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>17</v>
@@ -2171,30 +2182,30 @@
         <v>57</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" s="0" t="n">
         <v>58</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>14</v>
@@ -2205,10 +2216,10 @@
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>14</v>
@@ -2217,18 +2228,18 @@
         <v>60</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>14</v>
@@ -2239,10 +2250,10 @@
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>14</v>
@@ -2251,18 +2262,18 @@
         <v>62</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>14</v>
@@ -2271,18 +2282,18 @@
         <v>63</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>14</v>
@@ -2291,18 +2302,18 @@
         <v>1</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I65" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>14</v>
@@ -2311,18 +2322,18 @@
         <v>2</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I66" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>14</v>
@@ -2331,110 +2342,110 @@
         <v>3</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" s="0" t="n">
         <v>4</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I68" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B69" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" s="0" t="n">
         <v>5</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="I69" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B70" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" s="0" t="n">
         <v>6</v>
       </c>
       <c r="F70" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="I70" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B71" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D71" s="0" t="n">
         <v>7</v>
       </c>
       <c r="F71" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I71" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B72" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" s="0" t="n">
         <v>8</v>
       </c>
       <c r="F72" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I72" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B73" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C73" s="2" t="s">
         <v>17</v>
@@ -2443,42 +2454,42 @@
         <v>9</v>
       </c>
       <c r="E73" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F73" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G73" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I73" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B74" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" s="0" t="n">
         <v>10</v>
       </c>
       <c r="F74" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I74" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C75" s="2" t="s">
         <v>14</v>
@@ -2487,18 +2498,18 @@
         <v>11</v>
       </c>
       <c r="F75" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I75" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>17</v>
@@ -2507,21 +2518,21 @@
         <v>12</v>
       </c>
       <c r="F76" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G76" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I76" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B77" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>17</v>
@@ -2530,21 +2541,21 @@
         <v>13</v>
       </c>
       <c r="F77" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G77" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I77" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B78" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>17</v>
@@ -2553,21 +2564,21 @@
         <v>14</v>
       </c>
       <c r="F78" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G78" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I78" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B79" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>14</v>
@@ -2576,18 +2587,18 @@
         <v>15</v>
       </c>
       <c r="F79" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G79" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B80" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>14</v>
@@ -2596,18 +2607,18 @@
         <v>16</v>
       </c>
       <c r="F80" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I80" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B81" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>14</v>
@@ -2616,18 +2627,18 @@
         <v>17</v>
       </c>
       <c r="F81" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I81" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B82" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>17</v>
@@ -2636,18 +2647,18 @@
         <v>18</v>
       </c>
       <c r="F82" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I82" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B83" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>17</v>
@@ -2656,18 +2667,18 @@
         <v>19</v>
       </c>
       <c r="F83" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I83" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B84" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>17</v>
@@ -2676,18 +2687,18 @@
         <v>20</v>
       </c>
       <c r="F84" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I84" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B85" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C85" s="2" t="s">
         <v>17</v>
@@ -2696,18 +2707,18 @@
         <v>21</v>
       </c>
       <c r="F85" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I85" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B86" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C86" s="2" t="s">
         <v>14</v>
@@ -2716,21 +2727,21 @@
         <v>22</v>
       </c>
       <c r="E86" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H86" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I86" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B87" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C87" s="2" t="s">
         <v>17</v>
@@ -2739,21 +2750,21 @@
         <v>23</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H87" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I87" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>14</v>
@@ -2762,21 +2773,21 @@
         <v>24</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H88" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I88" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B89" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C89" s="2" t="s">
         <v>17</v>
@@ -2785,21 +2796,21 @@
         <v>25</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H89" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I89" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B90" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C90" s="2" t="s">
         <v>14</v>
@@ -2808,21 +2819,21 @@
         <v>26</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H90" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I90" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B91" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C91" s="2" t="s">
         <v>17</v>
@@ -2831,21 +2842,21 @@
         <v>27</v>
       </c>
       <c r="E91" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H91" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I91" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C92" s="2" t="s">
         <v>14</v>
@@ -2854,21 +2865,21 @@
         <v>28</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H92" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I92" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C93" s="2" t="s">
         <v>17</v>
@@ -2877,21 +2888,21 @@
         <v>29</v>
       </c>
       <c r="E93" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H93" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I93" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C94" s="2" t="s">
         <v>17</v>
@@ -2900,48 +2911,48 @@
         <v>30</v>
       </c>
       <c r="E94" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F94" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G94" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H94" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I94" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" s="0" t="n">
         <v>31</v>
       </c>
       <c r="E95" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F95" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I95" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B96" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C96" s="2" t="s">
         <v>11</v>
@@ -2950,36 +2961,36 @@
         <v>32</v>
       </c>
       <c r="F96" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I96" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B97" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" s="0" t="n">
         <v>33</v>
       </c>
       <c r="F97" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I97" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C98" s="2" t="s">
         <v>11</v>
@@ -2988,33 +2999,33 @@
         <v>34</v>
       </c>
       <c r="F98" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I98" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B99" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" s="0" t="n">
         <v>35</v>
       </c>
       <c r="F99" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B100" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C100" s="2" t="s">
         <v>14</v>
@@ -3023,18 +3034,18 @@
         <v>36</v>
       </c>
       <c r="F100" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I100" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B101" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C101" s="2" t="s">
         <v>17</v>
@@ -3043,48 +3054,48 @@
         <v>37</v>
       </c>
       <c r="F101" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B102" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" s="0" t="n">
         <v>38</v>
       </c>
       <c r="F102" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B103" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" s="0" t="n">
         <v>39</v>
       </c>
       <c r="F103" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I103" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B104" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C104" s="2" t="s">
         <v>17</v>
@@ -3093,15 +3104,15 @@
         <v>40</v>
       </c>
       <c r="F104" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B105" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C105" s="2" t="s">
         <v>17</v>
@@ -3110,15 +3121,15 @@
         <v>41</v>
       </c>
       <c r="F105" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B106" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C106" s="2" t="s">
         <v>17</v>
@@ -3127,15 +3138,15 @@
         <v>42</v>
       </c>
       <c r="F106" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B107" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C107" s="2" t="s">
         <v>17</v>
@@ -3144,15 +3155,15 @@
         <v>43</v>
       </c>
       <c r="F107" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C108" s="2" t="s">
         <v>17</v>
@@ -3161,15 +3172,15 @@
         <v>44</v>
       </c>
       <c r="F108" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B109" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C109" s="2" t="s">
         <v>17</v>
@@ -3178,15 +3189,15 @@
         <v>45</v>
       </c>
       <c r="F109" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B110" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C110" s="2" t="s">
         <v>17</v>
@@ -3195,15 +3206,15 @@
         <v>46</v>
       </c>
       <c r="F110" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B111" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C111" s="2" t="s">
         <v>17</v>
@@ -3212,15 +3223,15 @@
         <v>47</v>
       </c>
       <c r="F111" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B112" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C112" s="2" t="s">
         <v>17</v>
@@ -3229,30 +3240,30 @@
         <v>48</v>
       </c>
       <c r="F112" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B113" s="0" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" s="0" t="n">
         <v>49</v>
       </c>
       <c r="F113" s="0" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B114" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C114" s="2" t="s">
         <v>14</v>
@@ -3263,10 +3274,10 @@
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C115" s="2" t="s">
         <v>14</v>
@@ -3275,18 +3286,18 @@
         <v>51</v>
       </c>
       <c r="F115" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I115" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B116" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C116" s="2" t="s">
         <v>14</v>
@@ -3297,10 +3308,10 @@
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B117" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C117" s="2" t="s">
         <v>14</v>
@@ -3309,18 +3320,18 @@
         <v>53</v>
       </c>
       <c r="F117" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I117" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B118" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C118" s="2" t="s">
         <v>14</v>
@@ -3329,33 +3340,33 @@
         <v>54</v>
       </c>
       <c r="F118" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I118" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C119" s="2"/>
       <c r="D119" s="0" t="n">
         <v>55</v>
       </c>
       <c r="I119" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B120" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C120" s="2" t="s">
         <v>14</v>
@@ -3364,18 +3375,18 @@
         <v>1</v>
       </c>
       <c r="E120" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I120" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C121" s="2" t="s">
         <v>14</v>
@@ -3384,165 +3395,167 @@
         <v>2</v>
       </c>
       <c r="E121" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I121" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" s="0" t="n">
         <v>3</v>
       </c>
       <c r="F122" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I122" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" s="0" t="n">
         <v>4</v>
       </c>
       <c r="F123" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="I123" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B124" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" s="0" t="n">
         <v>5</v>
       </c>
       <c r="F124" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="I124" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B125" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" s="0" t="n">
         <v>6</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I125" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="C126" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D126" s="0" t="n">
         <v>7</v>
       </c>
       <c r="F126" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I126" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" s="0" t="n">
         <v>8</v>
       </c>
       <c r="F127" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I127" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C128" s="2"/>
       <c r="D128" s="0" t="n">
         <v>9</v>
       </c>
       <c r="E128" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F128" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G128" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I128" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C129" s="2"/>
       <c r="D129" s="0" t="n">
         <v>10</v>
       </c>
       <c r="F129" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B130" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C130" s="2" t="s">
         <v>14</v>
@@ -3551,18 +3564,18 @@
         <v>11</v>
       </c>
       <c r="F130" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I130" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B131" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C131" s="2" t="s">
         <v>17</v>
@@ -3571,18 +3584,18 @@
         <v>12</v>
       </c>
       <c r="F131" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I131" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B132" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C132" s="2" t="s">
         <v>17</v>
@@ -3591,21 +3604,21 @@
         <v>13</v>
       </c>
       <c r="F132" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G132" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I132" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B133" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C133" s="2" t="s">
         <v>17</v>
@@ -3614,18 +3627,18 @@
         <v>14</v>
       </c>
       <c r="F133" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I133" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B134" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C134" s="2" t="s">
         <v>14</v>
@@ -3634,15 +3647,15 @@
         <v>15</v>
       </c>
       <c r="F134" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B135" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C135" s="2" t="s">
         <v>14</v>
@@ -3651,18 +3664,18 @@
         <v>16</v>
       </c>
       <c r="F135" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I135" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B136" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C136" s="2" t="s">
         <v>14</v>
@@ -3671,18 +3684,18 @@
         <v>17</v>
       </c>
       <c r="F136" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I136" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B137" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C137" s="2" t="s">
         <v>17</v>
@@ -3691,18 +3704,18 @@
         <v>18</v>
       </c>
       <c r="F137" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I137" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B138" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C138" s="2" t="s">
         <v>17</v>
@@ -3711,18 +3724,18 @@
         <v>19</v>
       </c>
       <c r="F138" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I138" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B139" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C139" s="2" t="s">
         <v>17</v>
@@ -3731,18 +3744,18 @@
         <v>20</v>
       </c>
       <c r="F139" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I139" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B140" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C140" s="2" t="s">
         <v>17</v>
@@ -3751,18 +3764,18 @@
         <v>21</v>
       </c>
       <c r="F140" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I140" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B141" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C141" s="2" t="s">
         <v>14</v>
@@ -3771,21 +3784,21 @@
         <v>22</v>
       </c>
       <c r="E141" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H141" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I141" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B142" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C142" s="2" t="s">
         <v>17</v>
@@ -3794,21 +3807,21 @@
         <v>23</v>
       </c>
       <c r="E142" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H142" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I142" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B143" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C143" s="2" t="s">
         <v>14</v>
@@ -3817,21 +3830,21 @@
         <v>24</v>
       </c>
       <c r="E143" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H143" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I143" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B144" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C144" s="2" t="s">
         <v>17</v>
@@ -3840,21 +3853,21 @@
         <v>25</v>
       </c>
       <c r="E144" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H144" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I144" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B145" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C145" s="2" t="s">
         <v>14</v>
@@ -3863,21 +3876,21 @@
         <v>26</v>
       </c>
       <c r="E145" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H145" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I145" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B146" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C146" s="2" t="s">
         <v>17</v>
@@ -3886,21 +3899,21 @@
         <v>27</v>
       </c>
       <c r="E146" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H146" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I146" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B147" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C147" s="2" t="s">
         <v>14</v>
@@ -3909,21 +3922,21 @@
         <v>28</v>
       </c>
       <c r="E147" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H147" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I147" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B148" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C148" s="2" t="s">
         <v>17</v>
@@ -3932,21 +3945,21 @@
         <v>29</v>
       </c>
       <c r="E148" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H148" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I148" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B149" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C149" s="2" t="s">
         <v>17</v>
@@ -3955,27 +3968,27 @@
         <v>30</v>
       </c>
       <c r="E149" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F149" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G149" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H149" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I149" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B150" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C150" s="2" t="s">
         <v>14</v>
@@ -3984,21 +3997,21 @@
         <v>31</v>
       </c>
       <c r="E150" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F150" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I150" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B151" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C151" s="2" t="s">
         <v>11</v>
@@ -4007,36 +4020,36 @@
         <v>32</v>
       </c>
       <c r="F151" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I151" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B152" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C152" s="2"/>
       <c r="D152" s="0" t="n">
         <v>33</v>
       </c>
       <c r="F152" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I152" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B153" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C153" s="2" t="s">
         <v>11</v>
@@ -4045,33 +4058,33 @@
         <v>34</v>
       </c>
       <c r="F153" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I153" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B154" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C154" s="2"/>
       <c r="D154" s="0" t="n">
         <v>35</v>
       </c>
       <c r="F154" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B155" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C155" s="2" t="s">
         <v>14</v>
@@ -4080,18 +4093,18 @@
         <v>36</v>
       </c>
       <c r="F155" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I155" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B156" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C156" s="2" t="s">
         <v>17</v>
@@ -4100,48 +4113,48 @@
         <v>37</v>
       </c>
       <c r="F156" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B157" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C157" s="2"/>
       <c r="D157" s="0" t="n">
         <v>38</v>
       </c>
       <c r="F157" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B158" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C158" s="2"/>
       <c r="D158" s="0" t="n">
         <v>39</v>
       </c>
       <c r="F158" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I158" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B159" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C159" s="2" t="s">
         <v>17</v>
@@ -4150,15 +4163,15 @@
         <v>40</v>
       </c>
       <c r="F159" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B160" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C160" s="2" t="s">
         <v>17</v>
@@ -4167,15 +4180,15 @@
         <v>41</v>
       </c>
       <c r="F160" s="0" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B161" s="0" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C161" s="2" t="s">
         <v>17</v>
@@ -4184,15 +4197,15 @@
         <v>42</v>
       </c>
       <c r="F161" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B162" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C162" s="2" t="s">
         <v>17</v>
@@ -4201,15 +4214,15 @@
         <v>43</v>
       </c>
       <c r="F162" s="0" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B163" s="0" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C163" s="2" t="s">
         <v>17</v>
@@ -4218,15 +4231,15 @@
         <v>44</v>
       </c>
       <c r="F163" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B164" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C164" s="2" t="s">
         <v>17</v>
@@ -4235,15 +4248,15 @@
         <v>45</v>
       </c>
       <c r="F164" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B165" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C165" s="2" t="s">
         <v>17</v>
@@ -4252,15 +4265,15 @@
         <v>46</v>
       </c>
       <c r="F165" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B166" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C166" s="2" t="s">
         <v>17</v>
@@ -4269,15 +4282,15 @@
         <v>47</v>
       </c>
       <c r="F166" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B167" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C167" s="2" t="s">
         <v>17</v>
@@ -4286,30 +4299,30 @@
         <v>48</v>
       </c>
       <c r="F167" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B168" s="0" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C168" s="2"/>
       <c r="D168" s="0" t="n">
         <v>49</v>
       </c>
       <c r="F168" s="0" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B169" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C169" s="2" t="s">
         <v>14</v>
@@ -4320,10 +4333,10 @@
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B170" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C170" s="2" t="s">
         <v>14</v>
@@ -4332,18 +4345,18 @@
         <v>51</v>
       </c>
       <c r="F170" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I170" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B171" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C171" s="2" t="s">
         <v>14</v>
@@ -4354,10 +4367,10 @@
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B172" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C172" s="2" t="s">
         <v>14</v>
@@ -4366,18 +4379,18 @@
         <v>53</v>
       </c>
       <c r="F172" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I172" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B173" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C173" s="2" t="s">
         <v>14</v>
@@ -4386,18 +4399,18 @@
         <v>54</v>
       </c>
       <c r="F173" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I173" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B174" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C174" s="2"/>
       <c r="D174" s="0" t="n">
@@ -4406,25 +4419,25 @@
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B175" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C175" s="2"/>
       <c r="D175" s="0" t="n">
         <v>1</v>
       </c>
       <c r="E175" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B176" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C176" s="2"/>
       <c r="D176" s="0" t="n">
@@ -4433,85 +4446,87 @@
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B177" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C177" s="2"/>
       <c r="D177" s="0" t="n">
         <v>3</v>
       </c>
       <c r="F177" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B178" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C178" s="2"/>
       <c r="D178" s="0" t="n">
         <v>4</v>
       </c>
       <c r="F178" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B179" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C179" s="2"/>
       <c r="D179" s="0" t="n">
         <v>5</v>
       </c>
       <c r="F179" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B180" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C180" s="2"/>
       <c r="D180" s="0" t="n">
         <v>6</v>
       </c>
       <c r="F180" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B181" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="C181" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D181" s="0" t="n">
         <v>7</v>
       </c>
       <c r="F181" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B182" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C182" s="2"/>
       <c r="D182" s="0" t="n">
@@ -4520,10 +4535,10 @@
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B183" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" s="0" t="n">
@@ -4532,10 +4547,10 @@
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B184" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" s="0" t="n">
@@ -4544,10 +4559,10 @@
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B185" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" s="0" t="n">
@@ -4556,10 +4571,10 @@
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B186" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C186" s="2"/>
       <c r="D186" s="0" t="n">
@@ -4568,10 +4583,10 @@
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B187" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C187" s="2"/>
       <c r="D187" s="0" t="n">
@@ -4580,10 +4595,10 @@
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B188" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C188" s="2"/>
       <c r="D188" s="0" t="n">
@@ -4592,10 +4607,10 @@
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B189" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C189" s="2"/>
       <c r="D189" s="0" t="n">
@@ -4604,10 +4619,10 @@
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B190" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C190" s="2"/>
       <c r="D190" s="0" t="n">
@@ -4616,10 +4631,10 @@
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B191" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C191" s="2"/>
       <c r="D191" s="0" t="n">

</xml_diff>

<commit_message>
PDB-207: Inferred Environment is an option select box.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45311 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="906" uniqueCount="240">
   <si>
     <t xml:space="preserve">testExportMetaTemplate</t>
   </si>
@@ -540,6 +540,12 @@
     <t xml:space="preserve">PRIMARY_GRAINSIZE_ID$NAME</t>
   </si>
   <si>
+    <t xml:space="preserve">Grain Size (secondary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SECONDARY_GRAINSIZE_ID$NAME</t>
+  </si>
+  <si>
     <t xml:space="preserve">Comparator Used</t>
   </si>
   <si>
@@ -615,10 +621,13 @@
     <t xml:space="preserve">Inferred Environment</t>
   </si>
   <si>
+    <t xml:space="preserve">INFERRED_ENVIRONMENT</t>
+  </si>
+  <si>
     <t xml:space="preserve">DEPOSITION_ENV</t>
   </si>
   <si>
-    <t xml:space="preserve">Enter one of “marine” or “non-marine”</t>
+    <t xml:space="preserve">Enter one of “Marine” or “Non Marine”</t>
   </si>
   <si>
     <t xml:space="preserve">Environmental Features</t>
@@ -679,12 +688,6 @@
   </si>
   <si>
     <t xml:space="preserve">For a Sample Relationship, “c.” or “?”. TODO: what do these mean?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grain Size (secondary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SECONDARY_GRAINSIZE_ID$NAME</t>
   </si>
   <si>
     <t xml:space="preserve">Confidential</t>
@@ -1009,7 +1012,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I191"/>
+  <dimension ref="A1:I192"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -2021,31 +2024,31 @@
       <c r="B49" s="0" t="s">
         <v>172</v>
       </c>
-      <c r="C49" s="2"/>
+      <c r="C49" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D49" s="0" t="n">
         <v>48</v>
       </c>
       <c r="F49" s="0" t="s">
         <v>173</v>
       </c>
-      <c r="I49" s="0" t="s">
-        <v>174</v>
-      </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="C50" s="2"/>
       <c r="D50" s="0" t="n">
         <v>49</v>
       </c>
       <c r="F50" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="I50" s="0" t="s">
         <v>176</v>
       </c>
     </row>
@@ -2192,7 +2195,9 @@
       <c r="B59" s="0" t="s">
         <v>193</v>
       </c>
-      <c r="C59" s="2"/>
+      <c r="C59" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D59" s="0" t="n">
         <v>58</v>
       </c>
@@ -2207,19 +2212,20 @@
       <c r="B60" s="0" t="s">
         <v>195</v>
       </c>
-      <c r="C60" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="C60" s="2"/>
       <c r="D60" s="0" t="n">
         <v>59</v>
       </c>
+      <c r="F60" s="0" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>14</v>
@@ -2227,19 +2233,13 @@
       <c r="D61" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="F61" s="0" t="s">
-        <v>197</v>
-      </c>
-      <c r="I61" s="0" t="s">
-        <v>198</v>
-      </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>14</v>
@@ -2247,13 +2247,25 @@
       <c r="D62" s="0" t="n">
         <v>61</v>
       </c>
+      <c r="E62" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="F62" s="0" t="s">
+        <v>200</v>
+      </c>
+      <c r="G62" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I62" s="0" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>14</v>
@@ -2261,12 +2273,6 @@
       <c r="D63" s="0" t="n">
         <v>62</v>
       </c>
-      <c r="F63" s="0" t="s">
-        <v>201</v>
-      </c>
-      <c r="I63" s="0" t="s">
-        <v>202</v>
-      </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
@@ -2290,92 +2296,94 @@
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B65" s="0" t="s">
         <v>206</v>
       </c>
-      <c r="B65" s="0" t="s">
-        <v>31</v>
-      </c>
       <c r="C65" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D65" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E65" s="0" t="s">
-        <v>32</v>
+        <v>64</v>
+      </c>
+      <c r="F65" s="0" t="s">
+        <v>207</v>
       </c>
       <c r="I65" s="0" t="s">
-        <v>33</v>
+        <v>208</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>207</v>
+        <v>31</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D66" s="0" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I66" s="0" t="s">
-        <v>208</v>
+        <v>33</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>42</v>
+        <v>210</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D67" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="F67" s="0" t="s">
-        <v>43</v>
+        <v>2</v>
+      </c>
+      <c r="E67" s="0" t="s">
+        <v>35</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>44</v>
+        <v>211</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>209</v>
-      </c>
-      <c r="C68" s="2"/>
+        <v>42</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D68" s="0" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>210</v>
+        <v>43</v>
       </c>
       <c r="I68" s="0" t="s">
-        <v>211</v>
+        <v>44</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B69" s="0" t="s">
         <v>212</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" s="0" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F69" s="0" t="s">
         <v>213</v>
@@ -2386,14 +2394,14 @@
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B70" s="0" t="s">
         <v>215</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" s="0" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F70" s="0" t="s">
         <v>216</v>
@@ -2404,712 +2412,713 @@
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B71" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>218</v>
+      </c>
+      <c r="C71" s="2"/>
       <c r="D71" s="0" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F71" s="0" t="s">
-        <v>79</v>
+        <v>219</v>
       </c>
       <c r="I71" s="0" t="s">
-        <v>80</v>
+        <v>220</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B72" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="C72" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D72" s="0" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F72" s="0" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I72" s="0" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B73" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="C73" s="2"/>
       <c r="D73" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E73" s="0" t="s">
-        <v>85</v>
+        <v>8</v>
       </c>
       <c r="F73" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="G73" s="0" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="I73" s="0" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B74" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="C74" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D74" s="0" t="n">
-        <v>10</v>
+        <v>9</v>
+      </c>
+      <c r="E74" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="F74" s="0" t="s">
-        <v>90</v>
+        <v>86</v>
+      </c>
+      <c r="G74" s="0" t="s">
+        <v>87</v>
       </c>
       <c r="I74" s="0" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="C75" s="2"/>
       <c r="D75" s="0" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F75" s="0" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I75" s="0" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D76" s="0" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F76" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="G76" s="0" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="I76" s="0" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B77" s="0" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D77" s="0" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F77" s="0" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G77" s="0" t="s">
         <v>87</v>
       </c>
       <c r="I77" s="0" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B78" s="0" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D78" s="0" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F78" s="0" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G78" s="0" t="s">
         <v>87</v>
       </c>
       <c r="I78" s="0" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B79" s="0" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D79" s="0" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F79" s="0" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G79" s="0" t="s">
         <v>87</v>
       </c>
+      <c r="I79" s="0" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B80" s="0" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D80" s="0" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F80" s="0" t="s">
-        <v>107</v>
-      </c>
-      <c r="I80" s="0" t="s">
-        <v>108</v>
+        <v>105</v>
+      </c>
+      <c r="G80" s="0" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B81" s="0" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D81" s="0" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F81" s="0" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I81" s="0" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B82" s="0" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D82" s="0" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F82" s="0" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I82" s="0" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B83" s="0" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D83" s="0" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F83" s="0" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="I83" s="0" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B84" s="0" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D84" s="0" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F84" s="0" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I84" s="0" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B85" s="0" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C85" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D85" s="0" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F85" s="0" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I85" s="0" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B86" s="0" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D86" s="0" t="n">
-        <v>22</v>
-      </c>
-      <c r="E86" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="H86" s="0" t="s">
-        <v>5</v>
+        <v>21</v>
+      </c>
+      <c r="F86" s="0" t="s">
+        <v>122</v>
       </c>
       <c r="I86" s="0" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B87" s="0" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D87" s="0" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="H87" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I87" s="0" t="s">
-        <v>218</v>
+        <v>126</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D88" s="0" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="H88" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I88" s="0" t="s">
-        <v>132</v>
+        <v>221</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B89" s="0" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D89" s="0" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="H89" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I89" s="0" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B90" s="0" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D90" s="0" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="H90" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I90" s="0" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B91" s="0" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D91" s="0" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E91" s="0" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H91" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I91" s="0" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D92" s="0" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="H92" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I92" s="0" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D93" s="0" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E93" s="0" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H93" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I93" s="0" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C94" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D94" s="0" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E94" s="0" t="s">
-        <v>149</v>
-      </c>
-      <c r="F94" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="G94" s="0" t="s">
-        <v>87</v>
+        <v>146</v>
       </c>
       <c r="H94" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I94" s="0" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="C95" s="2"/>
+        <v>148</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D95" s="0" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E95" s="0" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="F95" s="0" t="s">
-        <v>154</v>
+        <v>150</v>
+      </c>
+      <c r="G95" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="H95" s="0" t="s">
+        <v>5</v>
       </c>
       <c r="I95" s="0" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B96" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="C96" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="C96" s="2"/>
       <c r="D96" s="0" t="n">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="E96" s="0" t="s">
+        <v>153</v>
       </c>
       <c r="F96" s="0" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="I96" s="0" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B97" s="0" t="s">
-        <v>159</v>
-      </c>
-      <c r="C97" s="2"/>
+        <v>156</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D97" s="0" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F97" s="0" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="I97" s="0" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>162</v>
-      </c>
-      <c r="C98" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="C98" s="2"/>
       <c r="D98" s="0" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F98" s="0" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I98" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B99" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="C99" s="2"/>
+        <v>162</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D99" s="0" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F99" s="0" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+      <c r="I99" s="0" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B100" s="0" t="s">
-        <v>167</v>
-      </c>
-      <c r="C100" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="C100" s="2"/>
       <c r="D100" s="0" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F100" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="I100" s="0" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B101" s="0" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D101" s="0" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F101" s="0" t="s">
-        <v>171</v>
+        <v>168</v>
+      </c>
+      <c r="I101" s="0" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B102" s="0" t="s">
-        <v>219</v>
-      </c>
-      <c r="C102" s="2"/>
+        <v>170</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D102" s="0" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F102" s="0" t="s">
-        <v>220</v>
+        <v>171</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B103" s="0" t="s">
         <v>172</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" s="0" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F103" s="0" t="s">
         <v>173</v>
       </c>
-      <c r="I103" s="0" t="s">
-        <v>174</v>
-      </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B104" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="C104" s="2"/>
+      <c r="D104" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="F104" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="C104" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D104" s="0" t="n">
-        <v>40</v>
-      </c>
-      <c r="F104" s="0" t="s">
+      <c r="I104" s="0" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B105" s="0" t="s">
         <v>177</v>
@@ -3118,7 +3127,7 @@
         <v>17</v>
       </c>
       <c r="D105" s="0" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F105" s="0" t="s">
         <v>178</v>
@@ -3126,7 +3135,7 @@
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B106" s="0" t="s">
         <v>179</v>
@@ -3135,7 +3144,7 @@
         <v>17</v>
       </c>
       <c r="D106" s="0" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F106" s="0" t="s">
         <v>180</v>
@@ -3143,7 +3152,7 @@
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B107" s="0" t="s">
         <v>181</v>
@@ -3152,7 +3161,7 @@
         <v>17</v>
       </c>
       <c r="D107" s="0" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F107" s="0" t="s">
         <v>182</v>
@@ -3160,7 +3169,7 @@
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B108" s="0" t="s">
         <v>183</v>
@@ -3169,7 +3178,7 @@
         <v>17</v>
       </c>
       <c r="D108" s="0" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F108" s="0" t="s">
         <v>184</v>
@@ -3177,7 +3186,7 @@
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B109" s="0" t="s">
         <v>185</v>
@@ -3186,7 +3195,7 @@
         <v>17</v>
       </c>
       <c r="D109" s="0" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F109" s="0" t="s">
         <v>186</v>
@@ -3194,7 +3203,7 @@
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B110" s="0" t="s">
         <v>187</v>
@@ -3203,7 +3212,7 @@
         <v>17</v>
       </c>
       <c r="D110" s="0" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F110" s="0" t="s">
         <v>188</v>
@@ -3211,7 +3220,7 @@
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B111" s="0" t="s">
         <v>189</v>
@@ -3220,7 +3229,7 @@
         <v>17</v>
       </c>
       <c r="D111" s="0" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F111" s="0" t="s">
         <v>190</v>
@@ -3228,7 +3237,7 @@
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B112" s="0" t="s">
         <v>191</v>
@@ -3237,7 +3246,7 @@
         <v>17</v>
       </c>
       <c r="D112" s="0" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F112" s="0" t="s">
         <v>192</v>
@@ -3245,14 +3254,16 @@
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B113" s="0" t="s">
         <v>193</v>
       </c>
-      <c r="C113" s="2"/>
+      <c r="C113" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D113" s="0" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F113" s="0" t="s">
         <v>194</v>
@@ -3260,75 +3271,76 @@
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B114" s="0" t="s">
         <v>195</v>
       </c>
-      <c r="C114" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="C114" s="2"/>
       <c r="D114" s="0" t="n">
-        <v>50</v>
+        <v>49</v>
+      </c>
+      <c r="F114" s="0" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C115" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D115" s="0" t="n">
-        <v>51</v>
-      </c>
-      <c r="F115" s="0" t="s">
-        <v>197</v>
-      </c>
-      <c r="I115" s="0" t="s">
-        <v>198</v>
+        <v>50</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B116" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D116" s="0" t="n">
+        <v>51</v>
+      </c>
+      <c r="E116" s="0" t="s">
         <v>199</v>
       </c>
-      <c r="C116" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D116" s="0" t="n">
-        <v>52</v>
+      <c r="F116" s="0" t="s">
+        <v>200</v>
+      </c>
+      <c r="G116" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I116" s="0" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B117" s="0" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C117" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D117" s="0" t="n">
-        <v>53</v>
-      </c>
-      <c r="F117" s="0" t="s">
-        <v>201</v>
-      </c>
-      <c r="I117" s="0" t="s">
-        <v>202</v>
+        <v>52</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B118" s="0" t="s">
         <v>203</v>
@@ -3337,7 +3349,7 @@
         <v>14</v>
       </c>
       <c r="D118" s="0" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F118" s="0" t="s">
         <v>204</v>
@@ -3348,105 +3360,107 @@
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B119" s="0" t="s">
         <v>206</v>
       </c>
-      <c r="B119" s="0" t="s">
-        <v>221</v>
-      </c>
-      <c r="C119" s="2"/>
+      <c r="C119" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D119" s="0" t="n">
-        <v>55</v>
+        <v>54</v>
+      </c>
+      <c r="F119" s="0" t="s">
+        <v>207</v>
       </c>
       <c r="I119" s="0" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B120" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="C120" s="2"/>
+      <c r="D120" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="I120" s="0" t="s">
         <v>223</v>
-      </c>
-      <c r="B120" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="C120" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D120" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E120" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="I120" s="0" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>224</v>
+        <v>31</v>
       </c>
       <c r="C121" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D121" s="0" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E121" s="0" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I121" s="0" t="s">
-        <v>208</v>
+        <v>33</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>209</v>
-      </c>
-      <c r="C122" s="2"/>
+        <v>225</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D122" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="F122" s="0" t="s">
-        <v>210</v>
+        <v>2</v>
+      </c>
+      <c r="E122" s="0" t="s">
+        <v>35</v>
       </c>
       <c r="I122" s="0" t="s">
-        <v>44</v>
+        <v>211</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B123" s="0" t="s">
         <v>212</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" s="0" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F123" s="0" t="s">
         <v>213</v>
       </c>
       <c r="I123" s="0" t="s">
-        <v>211</v>
+        <v>44</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B124" s="0" t="s">
         <v>215</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" s="0" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F124" s="0" t="s">
         <v>216</v>
@@ -3457,17 +3471,17 @@
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B125" s="0" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" s="0" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="I125" s="0" t="s">
         <v>217</v>
@@ -3475,700 +3489,701 @@
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>226</v>
+      </c>
+      <c r="C126" s="2"/>
       <c r="D126" s="0" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F126" s="0" t="s">
-        <v>79</v>
+        <v>227</v>
       </c>
       <c r="I126" s="0" t="s">
-        <v>80</v>
+        <v>220</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="C127" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D127" s="0" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F127" s="0" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I127" s="0" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C128" s="2"/>
       <c r="D128" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E128" s="0" t="s">
-        <v>85</v>
+        <v>8</v>
       </c>
       <c r="F128" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="G128" s="0" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="I128" s="0" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C129" s="2"/>
       <c r="D129" s="0" t="n">
-        <v>10</v>
+        <v>9</v>
+      </c>
+      <c r="E129" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="F129" s="0" t="s">
-        <v>90</v>
+        <v>86</v>
+      </c>
+      <c r="G129" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="I129" s="0" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B130" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="C130" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="C130" s="2"/>
       <c r="D130" s="0" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F130" s="0" t="s">
-        <v>93</v>
-      </c>
-      <c r="I130" s="0" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B131" s="0" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D131" s="0" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F131" s="0" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="I131" s="0" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B132" s="0" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C132" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D132" s="0" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F132" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="G132" s="0" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="I132" s="0" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B133" s="0" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C133" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D133" s="0" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F133" s="0" t="s">
-        <v>102</v>
+        <v>99</v>
+      </c>
+      <c r="G133" s="0" t="s">
+        <v>87</v>
       </c>
       <c r="I133" s="0" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B134" s="0" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D134" s="0" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F134" s="0" t="s">
-        <v>105</v>
+        <v>102</v>
+      </c>
+      <c r="I134" s="0" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B135" s="0" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C135" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D135" s="0" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F135" s="0" t="s">
-        <v>107</v>
-      </c>
-      <c r="I135" s="0" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B136" s="0" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C136" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D136" s="0" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F136" s="0" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I136" s="0" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B137" s="0" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D137" s="0" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F137" s="0" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I137" s="0" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B138" s="0" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C138" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D138" s="0" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F138" s="0" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="I138" s="0" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B139" s="0" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C139" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D139" s="0" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F139" s="0" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I139" s="0" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B140" s="0" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C140" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D140" s="0" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F140" s="0" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I140" s="0" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B141" s="0" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D141" s="0" t="n">
-        <v>22</v>
-      </c>
-      <c r="E141" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="H141" s="0" t="s">
-        <v>5</v>
+        <v>21</v>
+      </c>
+      <c r="F141" s="0" t="s">
+        <v>122</v>
       </c>
       <c r="I141" s="0" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B142" s="0" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D142" s="0" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E142" s="0" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="H142" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I142" s="0" t="s">
-        <v>218</v>
+        <v>126</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B143" s="0" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D143" s="0" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E143" s="0" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="H143" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I143" s="0" t="s">
-        <v>132</v>
+        <v>221</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B144" s="0" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D144" s="0" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E144" s="0" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="H144" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I144" s="0" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B145" s="0" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D145" s="0" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E145" s="0" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="H145" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I145" s="0" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B146" s="0" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D146" s="0" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E146" s="0" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H146" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I146" s="0" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B147" s="0" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D147" s="0" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E147" s="0" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="H147" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I147" s="0" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B148" s="0" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D148" s="0" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E148" s="0" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H148" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I148" s="0" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B149" s="0" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C149" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D149" s="0" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E149" s="0" t="s">
-        <v>149</v>
-      </c>
-      <c r="F149" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="G149" s="0" t="s">
-        <v>87</v>
+        <v>146</v>
       </c>
       <c r="H149" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I149" s="0" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B150" s="0" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D150" s="0" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E150" s="0" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="F150" s="0" t="s">
-        <v>154</v>
+        <v>150</v>
+      </c>
+      <c r="G150" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="H150" s="0" t="s">
+        <v>5</v>
       </c>
       <c r="I150" s="0" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B151" s="0" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D151" s="0" t="n">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="E151" s="0" t="s">
+        <v>153</v>
       </c>
       <c r="F151" s="0" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="I151" s="0" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B152" s="0" t="s">
-        <v>159</v>
-      </c>
-      <c r="C152" s="2"/>
+        <v>156</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D152" s="0" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F152" s="0" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="I152" s="0" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B153" s="0" t="s">
-        <v>162</v>
-      </c>
-      <c r="C153" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="C153" s="2"/>
       <c r="D153" s="0" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F153" s="0" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I153" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B154" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="C154" s="2"/>
+        <v>162</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D154" s="0" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F154" s="0" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+      <c r="I154" s="0" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B155" s="0" t="s">
-        <v>167</v>
-      </c>
-      <c r="C155" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="C155" s="2"/>
       <c r="D155" s="0" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F155" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="I155" s="0" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B156" s="0" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D156" s="0" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F156" s="0" t="s">
-        <v>171</v>
+        <v>168</v>
+      </c>
+      <c r="I156" s="0" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B157" s="0" t="s">
-        <v>219</v>
-      </c>
-      <c r="C157" s="2"/>
+        <v>170</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D157" s="0" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F157" s="0" t="s">
-        <v>220</v>
+        <v>171</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B158" s="0" t="s">
         <v>172</v>
       </c>
       <c r="C158" s="2"/>
       <c r="D158" s="0" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F158" s="0" t="s">
         <v>173</v>
       </c>
-      <c r="I158" s="0" t="s">
-        <v>174</v>
-      </c>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B159" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="C159" s="2"/>
+      <c r="D159" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="F159" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="C159" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D159" s="0" t="n">
-        <v>40</v>
-      </c>
-      <c r="F159" s="0" t="s">
+      <c r="I159" s="0" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B160" s="0" t="s">
         <v>177</v>
@@ -4177,7 +4192,7 @@
         <v>17</v>
       </c>
       <c r="D160" s="0" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F160" s="0" t="s">
         <v>178</v>
@@ -4185,7 +4200,7 @@
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B161" s="0" t="s">
         <v>179</v>
@@ -4194,7 +4209,7 @@
         <v>17</v>
       </c>
       <c r="D161" s="0" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F161" s="0" t="s">
         <v>180</v>
@@ -4202,7 +4217,7 @@
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B162" s="0" t="s">
         <v>181</v>
@@ -4211,7 +4226,7 @@
         <v>17</v>
       </c>
       <c r="D162" s="0" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F162" s="0" t="s">
         <v>182</v>
@@ -4219,7 +4234,7 @@
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B163" s="0" t="s">
         <v>183</v>
@@ -4228,7 +4243,7 @@
         <v>17</v>
       </c>
       <c r="D163" s="0" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F163" s="0" t="s">
         <v>184</v>
@@ -4236,7 +4251,7 @@
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B164" s="0" t="s">
         <v>185</v>
@@ -4245,7 +4260,7 @@
         <v>17</v>
       </c>
       <c r="D164" s="0" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F164" s="0" t="s">
         <v>186</v>
@@ -4253,7 +4268,7 @@
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B165" s="0" t="s">
         <v>187</v>
@@ -4262,7 +4277,7 @@
         <v>17</v>
       </c>
       <c r="D165" s="0" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F165" s="0" t="s">
         <v>188</v>
@@ -4270,7 +4285,7 @@
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B166" s="0" t="s">
         <v>189</v>
@@ -4279,7 +4294,7 @@
         <v>17</v>
       </c>
       <c r="D166" s="0" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F166" s="0" t="s">
         <v>190</v>
@@ -4287,7 +4302,7 @@
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B167" s="0" t="s">
         <v>191</v>
@@ -4296,7 +4311,7 @@
         <v>17</v>
       </c>
       <c r="D167" s="0" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F167" s="0" t="s">
         <v>192</v>
@@ -4304,14 +4319,16 @@
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B168" s="0" t="s">
         <v>193</v>
       </c>
-      <c r="C168" s="2"/>
+      <c r="C168" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D168" s="0" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F168" s="0" t="s">
         <v>194</v>
@@ -4319,75 +4336,76 @@
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B169" s="0" t="s">
         <v>195</v>
       </c>
-      <c r="C169" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="C169" s="2"/>
       <c r="D169" s="0" t="n">
-        <v>50</v>
+        <v>49</v>
+      </c>
+      <c r="F169" s="0" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B170" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C170" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D170" s="0" t="n">
-        <v>51</v>
-      </c>
-      <c r="F170" s="0" t="s">
-        <v>197</v>
-      </c>
-      <c r="I170" s="0" t="s">
-        <v>198</v>
+        <v>50</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B171" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="C171" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D171" s="0" t="n">
+        <v>51</v>
+      </c>
+      <c r="E171" s="0" t="s">
         <v>199</v>
       </c>
-      <c r="C171" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D171" s="0" t="n">
-        <v>52</v>
+      <c r="F171" s="0" t="s">
+        <v>200</v>
+      </c>
+      <c r="G171" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I171" s="0" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B172" s="0" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C172" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D172" s="0" t="n">
-        <v>53</v>
-      </c>
-      <c r="F172" s="0" t="s">
-        <v>201</v>
-      </c>
-      <c r="I172" s="0" t="s">
-        <v>202</v>
+        <v>52</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B173" s="0" t="s">
         <v>203</v>
@@ -4396,7 +4414,7 @@
         <v>14</v>
       </c>
       <c r="D173" s="0" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F173" s="0" t="s">
         <v>204</v>
@@ -4407,68 +4425,73 @@
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B174" s="0" t="s">
-        <v>221</v>
-      </c>
-      <c r="C174" s="2"/>
+        <v>206</v>
+      </c>
+      <c r="C174" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D174" s="0" t="n">
-        <v>55</v>
+        <v>54</v>
+      </c>
+      <c r="F174" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="I174" s="0" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="B175" s="0" t="s">
-        <v>31</v>
+        <v>222</v>
       </c>
       <c r="C175" s="2"/>
       <c r="D175" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E175" s="0" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B176" s="0" t="s">
-        <v>228</v>
+        <v>31</v>
       </c>
       <c r="C176" s="2"/>
       <c r="D176" s="0" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="E176" s="0" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B177" s="0" t="s">
-        <v>209</v>
+        <v>229</v>
       </c>
       <c r="C177" s="2"/>
       <c r="D177" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="F177" s="0" t="s">
-        <v>210</v>
+        <v>2</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B178" s="0" t="s">
         <v>212</v>
       </c>
       <c r="C178" s="2"/>
       <c r="D178" s="0" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F178" s="0" t="s">
         <v>213</v>
@@ -4476,14 +4499,14 @@
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B179" s="0" t="s">
         <v>215</v>
       </c>
       <c r="C179" s="2"/>
       <c r="D179" s="0" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F179" s="0" t="s">
         <v>216</v>
@@ -4491,153 +4514,168 @@
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B180" s="0" t="s">
-        <v>42</v>
+        <v>218</v>
       </c>
       <c r="C180" s="2"/>
       <c r="D180" s="0" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F180" s="0" t="s">
-        <v>43</v>
+        <v>219</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B181" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C181" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="C181" s="2"/>
       <c r="D181" s="0" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F181" s="0" t="s">
-        <v>79</v>
+        <v>43</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B182" s="0" t="s">
-        <v>229</v>
-      </c>
-      <c r="C182" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="C182" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D182" s="0" t="n">
-        <v>8</v>
+        <v>7</v>
+      </c>
+      <c r="F182" s="0" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B183" s="0" t="s">
         <v>230</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" s="0" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B184" s="0" t="s">
         <v>231</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" s="0" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B185" s="0" t="s">
         <v>232</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" s="0" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B186" s="0" t="s">
         <v>233</v>
       </c>
       <c r="C186" s="2"/>
       <c r="D186" s="0" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B187" s="0" t="s">
         <v>234</v>
       </c>
       <c r="C187" s="2"/>
       <c r="D187" s="0" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B188" s="0" t="s">
         <v>235</v>
       </c>
       <c r="C188" s="2"/>
       <c r="D188" s="0" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B189" s="0" t="s">
         <v>236</v>
       </c>
       <c r="C189" s="2"/>
       <c r="D189" s="0" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B190" s="0" t="s">
         <v>237</v>
       </c>
       <c r="C190" s="2"/>
       <c r="D190" s="0" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B191" s="0" t="s">
         <v>238</v>
       </c>
       <c r="C191" s="2"/>
       <c r="D191" s="0" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B192" s="0" t="s">
+        <v>239</v>
+      </c>
+      <c r="C192" s="2"/>
+      <c r="D192" s="0" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4647,7 +4685,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A191" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A192" type="list">
       <formula1>_Lists!$B$2:$B$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4659,7 +4697,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C191" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C192" type="list">
       <formula1>_Lists!$C$2:$C$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4667,7 +4705,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D191" type="whole">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D192" type="whole">
       <formula1>-2000000000</formula1>
       <formula2>2000000000</formula2>
     </dataValidation>
@@ -4683,7 +4721,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G191" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G192" type="list">
       <formula1>_Lists!$D$2:$D$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4695,7 +4733,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" prompt="The only valid values here are no value, &quot;yes&quot; or &quot;no&quot;" promptTitle="Boolean value" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="H2:H191" type="list">
+    <dataValidation allowBlank="true" operator="between" prompt="The only valid values here are no value, &quot;yes&quot; or &quot;no&quot;" promptTitle="Boolean value" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="H2:H192" type="list">
       <formula1>_Lists!$A$2:$A$4</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
PDB-197: Remove map scale.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45313 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="906" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="902" uniqueCount="238">
   <si>
     <t xml:space="preserve">testExportMetaTemplate</t>
   </si>
@@ -196,12 +196,6 @@
   </si>
   <si>
     <t xml:space="preserve">Enter how this coordinate was found.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Map Scale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If using a map, what was the scale on that map?</t>
   </si>
   <si>
     <t xml:space="preserve">Map Year</t>
@@ -1012,7 +1006,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I192"/>
+  <dimension ref="A1:I191"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -1240,13 +1234,16 @@
         <v>58</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D11" s="0" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="F11" s="0" t="s">
+        <v>59</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1254,19 +1251,19 @@
         <v>30</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D12" s="0" t="n">
-        <v>11</v>
-      </c>
-      <c r="F12" s="0" t="s">
-        <v>61</v>
+        <v>12</v>
+      </c>
+      <c r="E12" s="0" t="s">
+        <v>62</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1274,19 +1271,19 @@
         <v>30</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D13" s="0" t="n">
-        <v>12</v>
-      </c>
-      <c r="E13" s="0" t="s">
-        <v>64</v>
+        <v>13</v>
+      </c>
+      <c r="F13" s="0" t="s">
+        <v>65</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1294,19 +1291,22 @@
         <v>30</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D14" s="0" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="E14" s="0" t="s">
+        <v>68</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1314,22 +1314,19 @@
         <v>30</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D15" s="0" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="F15" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1337,16 +1334,13 @@
         <v>30</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D16" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="E16" s="0" t="s">
-        <v>74</v>
+        <v>16</v>
       </c>
       <c r="I16" s="0" t="s">
         <v>75</v>
@@ -1360,13 +1354,16 @@
         <v>76</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D17" s="0" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="F17" s="0" t="s">
+        <v>77</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1374,19 +1371,19 @@
         <v>30</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D18" s="0" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1394,19 +1391,25 @@
         <v>30</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D19" s="0" t="n">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="E19" s="0" t="s">
+        <v>83</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
+      </c>
+      <c r="G19" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="I19" s="0" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1414,25 +1417,17 @@
         <v>30</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="C20" s="2"/>
       <c r="D20" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="E20" s="0" t="s">
-        <v>85</v>
+        <v>20</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="G20" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I20" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1440,17 +1435,19 @@
         <v>30</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="C21" s="2"/>
+        <v>90</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D21" s="0" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I21" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1458,19 +1455,19 @@
         <v>30</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D22" s="0" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1478,19 +1475,22 @@
         <v>30</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="0" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
+      </c>
+      <c r="G23" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1498,22 +1498,19 @@
         <v>30</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D24" s="0" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="G24" s="0" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1521,18 +1518,15 @@
         <v>30</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D25" s="0" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="I25" s="0" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1547,30 +1541,33 @@
         <v>14</v>
       </c>
       <c r="D26" s="0" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F26" s="0" t="s">
         <v>105</v>
       </c>
+      <c r="I26" s="0" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D27" s="0" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1578,19 +1575,19 @@
         <v>30</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D28" s="0" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1598,19 +1595,19 @@
         <v>30</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D29" s="0" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I29" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1618,19 +1615,19 @@
         <v>30</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D30" s="0" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1638,19 +1635,19 @@
         <v>30</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D31" s="0" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1658,19 +1655,22 @@
         <v>30</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D32" s="0" t="n">
-        <v>31</v>
-      </c>
-      <c r="F32" s="0" t="s">
-        <v>122</v>
+        <v>32</v>
+      </c>
+      <c r="E32" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="H32" s="0" t="s">
+        <v>5</v>
       </c>
       <c r="I32" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1678,22 +1678,22 @@
         <v>30</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D33" s="0" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H33" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I33" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1701,22 +1701,22 @@
         <v>30</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D34" s="0" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H34" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1724,22 +1724,22 @@
         <v>30</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D35" s="0" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H35" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1747,22 +1747,22 @@
         <v>30</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D36" s="0" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H36" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1770,22 +1770,22 @@
         <v>30</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D37" s="0" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H37" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1793,22 +1793,22 @@
         <v>30</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D38" s="0" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H38" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1816,22 +1816,22 @@
         <v>30</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D39" s="0" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H39" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I39" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1839,22 +1839,28 @@
         <v>30</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D40" s="0" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
+      </c>
+      <c r="F40" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="G40" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="H40" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1862,28 +1868,22 @@
         <v>30</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D41" s="0" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="G41" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="H41" s="0" t="s">
-        <v>5</v>
+        <v>152</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1891,22 +1891,19 @@
         <v>30</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D42" s="0" t="n">
-        <v>41</v>
-      </c>
-      <c r="E42" s="0" t="s">
-        <v>153</v>
+        <v>42</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I42" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1914,19 +1911,17 @@
         <v>30</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="C43" s="2"/>
       <c r="D43" s="0" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1934,17 +1929,17 @@
         <v>30</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="0" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1952,16 +1947,13 @@
         <v>30</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="0" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="I45" s="0" t="s">
         <v>164</v>
       </c>
     </row>
@@ -1972,31 +1964,33 @@
       <c r="B46" s="0" t="s">
         <v>165</v>
       </c>
-      <c r="C46" s="2"/>
+      <c r="C46" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D46" s="0" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F46" s="0" t="s">
         <v>166</v>
       </c>
+      <c r="I46" s="0" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D47" s="0" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="I47" s="0" t="s">
         <v>169</v>
       </c>
     </row>
@@ -2011,7 +2005,7 @@
         <v>17</v>
       </c>
       <c r="D48" s="0" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F48" s="0" t="s">
         <v>171</v>
@@ -2024,31 +2018,31 @@
       <c r="B49" s="0" t="s">
         <v>172</v>
       </c>
-      <c r="C49" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="C49" s="2"/>
       <c r="D49" s="0" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F49" s="0" t="s">
         <v>173</v>
       </c>
+      <c r="I49" s="0" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="C50" s="2"/>
+        <v>175</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D50" s="0" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="I50" s="0" t="s">
         <v>176</v>
       </c>
     </row>
@@ -2063,7 +2057,7 @@
         <v>17</v>
       </c>
       <c r="D51" s="0" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F51" s="0" t="s">
         <v>178</v>
@@ -2080,7 +2074,7 @@
         <v>17</v>
       </c>
       <c r="D52" s="0" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F52" s="0" t="s">
         <v>180</v>
@@ -2097,7 +2091,7 @@
         <v>17</v>
       </c>
       <c r="D53" s="0" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F53" s="0" t="s">
         <v>182</v>
@@ -2114,7 +2108,7 @@
         <v>17</v>
       </c>
       <c r="D54" s="0" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F54" s="0" t="s">
         <v>184</v>
@@ -2131,7 +2125,7 @@
         <v>17</v>
       </c>
       <c r="D55" s="0" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F55" s="0" t="s">
         <v>186</v>
@@ -2148,7 +2142,7 @@
         <v>17</v>
       </c>
       <c r="D56" s="0" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F56" s="0" t="s">
         <v>188</v>
@@ -2165,7 +2159,7 @@
         <v>17</v>
       </c>
       <c r="D57" s="0" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F57" s="0" t="s">
         <v>190</v>
@@ -2182,7 +2176,7 @@
         <v>17</v>
       </c>
       <c r="D58" s="0" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F58" s="0" t="s">
         <v>192</v>
@@ -2195,11 +2189,9 @@
       <c r="B59" s="0" t="s">
         <v>193</v>
       </c>
-      <c r="C59" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="C59" s="2"/>
       <c r="D59" s="0" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F59" s="0" t="s">
         <v>194</v>
@@ -2212,12 +2204,11 @@
       <c r="B60" s="0" t="s">
         <v>195</v>
       </c>
-      <c r="C60" s="2"/>
+      <c r="C60" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D60" s="0" t="n">
-        <v>59</v>
-      </c>
-      <c r="F60" s="0" t="s">
-        <v>196</v>
+        <v>60</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2225,13 +2216,25 @@
         <v>30</v>
       </c>
       <c r="B61" s="0" t="s">
+        <v>196</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D61" s="0" t="n">
+        <v>61</v>
+      </c>
+      <c r="E61" s="0" t="s">
         <v>197</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D61" s="0" t="n">
-        <v>60</v>
+      <c r="F61" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="G61" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I61" s="0" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2239,25 +2242,13 @@
         <v>30</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D62" s="0" t="n">
-        <v>61</v>
-      </c>
-      <c r="E62" s="0" t="s">
-        <v>199</v>
-      </c>
-      <c r="F62" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="G62" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="I62" s="0" t="s">
-        <v>201</v>
+        <v>62</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2265,13 +2256,19 @@
         <v>30</v>
       </c>
       <c r="B63" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D63" s="0" t="n">
+        <v>63</v>
+      </c>
+      <c r="F63" s="0" t="s">
         <v>202</v>
       </c>
-      <c r="C63" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D63" s="0" t="n">
-        <v>62</v>
+      <c r="I63" s="0" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2279,329 +2276,329 @@
         <v>30</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D64" s="0" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>30</v>
+        <v>207</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>206</v>
+        <v>31</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D65" s="0" t="n">
-        <v>64</v>
-      </c>
-      <c r="F65" s="0" t="s">
-        <v>207</v>
+        <v>1</v>
+      </c>
+      <c r="E65" s="0" t="s">
+        <v>32</v>
       </c>
       <c r="I65" s="0" t="s">
-        <v>208</v>
+        <v>33</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B66" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D66" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="I66" s="0" t="s">
         <v>209</v>
-      </c>
-      <c r="B66" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D66" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E66" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="I66" s="0" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>210</v>
+        <v>42</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D67" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E67" s="0" t="s">
-        <v>35</v>
+        <v>3</v>
+      </c>
+      <c r="F67" s="0" t="s">
+        <v>43</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>211</v>
+        <v>44</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="C68" s="2"/>
       <c r="D68" s="0" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>43</v>
+        <v>211</v>
       </c>
       <c r="I68" s="0" t="s">
-        <v>44</v>
+        <v>212</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B69" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" s="0" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I69" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B70" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" s="0" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F70" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="I70" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B71" s="0" t="s">
-        <v>218</v>
-      </c>
-      <c r="C71" s="2"/>
+        <v>76</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D71" s="0" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F71" s="0" t="s">
-        <v>219</v>
+        <v>77</v>
       </c>
       <c r="I71" s="0" t="s">
-        <v>220</v>
+        <v>78</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B72" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="C72" s="2"/>
       <c r="D72" s="0" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F72" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I72" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B73" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="C73" s="2"/>
+        <v>82</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D73" s="0" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="E73" s="0" t="s">
+        <v>83</v>
       </c>
       <c r="F73" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
+      </c>
+      <c r="G73" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="I73" s="0" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B74" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="C74" s="2"/>
       <c r="D74" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E74" s="0" t="s">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="F74" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="G74" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I74" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="C75" s="2"/>
+        <v>90</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D75" s="0" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F75" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I75" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D76" s="0" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F76" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
+      </c>
+      <c r="G76" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="I76" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B77" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D77" s="0" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F77" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G77" s="0" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="I77" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B78" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D78" s="0" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F78" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G78" s="0" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="I78" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B79" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D79" s="0" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F79" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G79" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="I79" s="0" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B80" s="0" t="s">
         <v>104</v>
@@ -2610,474 +2607,469 @@
         <v>14</v>
       </c>
       <c r="D80" s="0" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F80" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="G80" s="0" t="s">
-        <v>87</v>
+      <c r="I80" s="0" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B81" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D81" s="0" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F81" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I81" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B82" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D82" s="0" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F82" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I82" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B83" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D83" s="0" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F83" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I83" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B84" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D84" s="0" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F84" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I84" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B85" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C85" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D85" s="0" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F85" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I85" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B86" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D86" s="0" t="n">
-        <v>21</v>
-      </c>
-      <c r="F86" s="0" t="s">
-        <v>122</v>
+        <v>22</v>
+      </c>
+      <c r="E86" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="H86" s="0" t="s">
+        <v>5</v>
       </c>
       <c r="I86" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B87" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D87" s="0" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H87" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I87" s="0" t="s">
-        <v>126</v>
+        <v>219</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D88" s="0" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H88" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I88" s="0" t="s">
-        <v>221</v>
+        <v>130</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B89" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D89" s="0" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H89" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I89" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B90" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D90" s="0" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H90" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I90" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B91" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D91" s="0" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E91" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H91" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I91" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D92" s="0" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H92" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I92" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D93" s="0" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E93" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H93" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I93" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C94" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D94" s="0" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E94" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
+      </c>
+      <c r="F94" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="G94" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="H94" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I94" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="C95" s="2"/>
       <c r="D95" s="0" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E95" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F95" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="G95" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="H95" s="0" t="s">
-        <v>5</v>
+        <v>152</v>
       </c>
       <c r="I95" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B96" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="C96" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D96" s="0" t="n">
-        <v>31</v>
-      </c>
-      <c r="E96" s="0" t="s">
-        <v>153</v>
+        <v>32</v>
       </c>
       <c r="F96" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I96" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B97" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="C97" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="C97" s="2"/>
       <c r="D97" s="0" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F97" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I97" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>159</v>
-      </c>
-      <c r="C98" s="2"/>
+        <v>160</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D98" s="0" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F98" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I98" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B99" s="0" t="s">
-        <v>162</v>
-      </c>
-      <c r="C99" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="C99" s="2"/>
       <c r="D99" s="0" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F99" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="I99" s="0" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B100" s="0" t="s">
         <v>165</v>
       </c>
-      <c r="C100" s="2"/>
+      <c r="C100" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D100" s="0" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F100" s="0" t="s">
         <v>166</v>
       </c>
+      <c r="I100" s="0" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B101" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D101" s="0" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F101" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="I101" s="0" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B102" s="0" t="s">
         <v>170</v>
       </c>
-      <c r="C102" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="C102" s="2"/>
       <c r="D102" s="0" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F102" s="0" t="s">
         <v>171</v>
@@ -3085,40 +3077,42 @@
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B103" s="0" t="s">
         <v>172</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" s="0" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F103" s="0" t="s">
         <v>173</v>
       </c>
+      <c r="I103" s="0" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B104" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="C104" s="2"/>
+        <v>175</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D104" s="0" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F104" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="I104" s="0" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B105" s="0" t="s">
         <v>177</v>
@@ -3127,7 +3121,7 @@
         <v>17</v>
       </c>
       <c r="D105" s="0" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F105" s="0" t="s">
         <v>178</v>
@@ -3135,7 +3129,7 @@
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B106" s="0" t="s">
         <v>179</v>
@@ -3144,7 +3138,7 @@
         <v>17</v>
       </c>
       <c r="D106" s="0" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F106" s="0" t="s">
         <v>180</v>
@@ -3152,7 +3146,7 @@
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B107" s="0" t="s">
         <v>181</v>
@@ -3161,7 +3155,7 @@
         <v>17</v>
       </c>
       <c r="D107" s="0" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F107" s="0" t="s">
         <v>182</v>
@@ -3169,7 +3163,7 @@
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B108" s="0" t="s">
         <v>183</v>
@@ -3178,7 +3172,7 @@
         <v>17</v>
       </c>
       <c r="D108" s="0" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F108" s="0" t="s">
         <v>184</v>
@@ -3186,7 +3180,7 @@
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B109" s="0" t="s">
         <v>185</v>
@@ -3195,7 +3189,7 @@
         <v>17</v>
       </c>
       <c r="D109" s="0" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F109" s="0" t="s">
         <v>186</v>
@@ -3203,7 +3197,7 @@
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B110" s="0" t="s">
         <v>187</v>
@@ -3212,7 +3206,7 @@
         <v>17</v>
       </c>
       <c r="D110" s="0" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F110" s="0" t="s">
         <v>188</v>
@@ -3220,7 +3214,7 @@
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B111" s="0" t="s">
         <v>189</v>
@@ -3229,7 +3223,7 @@
         <v>17</v>
       </c>
       <c r="D111" s="0" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F111" s="0" t="s">
         <v>190</v>
@@ -3237,7 +3231,7 @@
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B112" s="0" t="s">
         <v>191</v>
@@ -3246,7 +3240,7 @@
         <v>17</v>
       </c>
       <c r="D112" s="0" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F112" s="0" t="s">
         <v>192</v>
@@ -3254,16 +3248,14 @@
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B113" s="0" t="s">
         <v>193</v>
       </c>
-      <c r="C113" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="C113" s="2"/>
       <c r="D113" s="0" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F113" s="0" t="s">
         <v>194</v>
@@ -3271,403 +3263,405 @@
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B114" s="0" t="s">
         <v>195</v>
       </c>
-      <c r="C114" s="2"/>
+      <c r="C114" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D114" s="0" t="n">
-        <v>49</v>
-      </c>
-      <c r="F114" s="0" t="s">
-        <v>196</v>
+        <v>50</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B115" s="0" t="s">
+        <v>196</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D115" s="0" t="n">
+        <v>51</v>
+      </c>
+      <c r="E115" s="0" t="s">
         <v>197</v>
       </c>
-      <c r="C115" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D115" s="0" t="n">
-        <v>50</v>
+      <c r="F115" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="G115" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I115" s="0" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B116" s="0" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C116" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D116" s="0" t="n">
-        <v>51</v>
-      </c>
-      <c r="E116" s="0" t="s">
-        <v>199</v>
-      </c>
-      <c r="F116" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="G116" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="I116" s="0" t="s">
-        <v>201</v>
+        <v>52</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B117" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D117" s="0" t="n">
+        <v>53</v>
+      </c>
+      <c r="F117" s="0" t="s">
         <v>202</v>
       </c>
-      <c r="C117" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D117" s="0" t="n">
-        <v>52</v>
+      <c r="I117" s="0" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B118" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C118" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D118" s="0" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F118" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="I118" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>206</v>
-      </c>
-      <c r="C119" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>220</v>
+      </c>
+      <c r="C119" s="2"/>
       <c r="D119" s="0" t="n">
-        <v>54</v>
-      </c>
-      <c r="F119" s="0" t="s">
-        <v>207</v>
+        <v>55</v>
       </c>
       <c r="I119" s="0" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="2" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="B120" s="0" t="s">
-        <v>222</v>
-      </c>
-      <c r="C120" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D120" s="0" t="n">
-        <v>55</v>
+        <v>1</v>
+      </c>
+      <c r="E120" s="0" t="s">
+        <v>32</v>
       </c>
       <c r="I120" s="0" t="s">
-        <v>223</v>
+        <v>33</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>31</v>
+        <v>223</v>
       </c>
       <c r="C121" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D121" s="0" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E121" s="0" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="I121" s="0" t="s">
-        <v>33</v>
+        <v>209</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>225</v>
-      </c>
-      <c r="C122" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="C122" s="2"/>
       <c r="D122" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E122" s="0" t="s">
-        <v>35</v>
+        <v>3</v>
+      </c>
+      <c r="F122" s="0" t="s">
+        <v>211</v>
       </c>
       <c r="I122" s="0" t="s">
-        <v>211</v>
+        <v>44</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" s="0" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F123" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I123" s="0" t="s">
-        <v>44</v>
+        <v>212</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B124" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" s="0" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F124" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="I124" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B125" s="0" t="s">
         <v>224</v>
-      </c>
-      <c r="B125" s="0" t="s">
-        <v>218</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" s="0" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="I125" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>226</v>
-      </c>
-      <c r="C126" s="2"/>
+        <v>76</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D126" s="0" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F126" s="0" t="s">
-        <v>227</v>
+        <v>77</v>
       </c>
       <c r="I126" s="0" t="s">
-        <v>220</v>
+        <v>78</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C127" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="C127" s="2"/>
       <c r="D127" s="0" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F127" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I127" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C128" s="2"/>
       <c r="D128" s="0" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="E128" s="0" t="s">
+        <v>83</v>
       </c>
       <c r="F128" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
+      </c>
+      <c r="G128" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="I128" s="0" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C129" s="2"/>
       <c r="D129" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E129" s="0" t="s">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="F129" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="G129" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="I129" s="0" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B130" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="C130" s="2"/>
+        <v>90</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D130" s="0" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F130" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
+      </c>
+      <c r="I130" s="0" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B131" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D131" s="0" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F131" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I131" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B132" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C132" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D132" s="0" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F132" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
+      </c>
+      <c r="G132" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="I132" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B133" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C133" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D133" s="0" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F133" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="G133" s="0" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="I133" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B134" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D134" s="0" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F134" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="I134" s="0" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B135" s="0" t="s">
         <v>104</v>
@@ -3676,473 +3670,471 @@
         <v>14</v>
       </c>
       <c r="D135" s="0" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F135" s="0" t="s">
         <v>105</v>
       </c>
+      <c r="I135" s="0" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B136" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C136" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D136" s="0" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F136" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I136" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B137" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D137" s="0" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F137" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I137" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B138" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C138" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D138" s="0" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F138" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I138" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B139" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C139" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D139" s="0" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F139" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I139" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B140" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C140" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D140" s="0" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F140" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I140" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B141" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D141" s="0" t="n">
-        <v>21</v>
-      </c>
-      <c r="F141" s="0" t="s">
-        <v>122</v>
+        <v>22</v>
+      </c>
+      <c r="E141" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="H141" s="0" t="s">
+        <v>5</v>
       </c>
       <c r="I141" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B142" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D142" s="0" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E142" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H142" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I142" s="0" t="s">
-        <v>126</v>
+        <v>219</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B143" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D143" s="0" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E143" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H143" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I143" s="0" t="s">
-        <v>221</v>
+        <v>130</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B144" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D144" s="0" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E144" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H144" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I144" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B145" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D145" s="0" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E145" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H145" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I145" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B146" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D146" s="0" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E146" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H146" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I146" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B147" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D147" s="0" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E147" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H147" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I147" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B148" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D148" s="0" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E148" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H148" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I148" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B149" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C149" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D149" s="0" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E149" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
+      </c>
+      <c r="F149" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="G149" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="H149" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I149" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B150" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D150" s="0" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E150" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F150" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="G150" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="H150" s="0" t="s">
-        <v>5</v>
+        <v>152</v>
       </c>
       <c r="I150" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B151" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D151" s="0" t="n">
-        <v>31</v>
-      </c>
-      <c r="E151" s="0" t="s">
-        <v>153</v>
+        <v>32</v>
       </c>
       <c r="F151" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I151" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B152" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="C152" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="C152" s="2"/>
       <c r="D152" s="0" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F152" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I152" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B153" s="0" t="s">
-        <v>159</v>
-      </c>
-      <c r="C153" s="2"/>
+        <v>160</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D153" s="0" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F153" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I153" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B154" s="0" t="s">
-        <v>162</v>
-      </c>
-      <c r="C154" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="C154" s="2"/>
       <c r="D154" s="0" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F154" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="I154" s="0" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B155" s="0" t="s">
         <v>165</v>
       </c>
-      <c r="C155" s="2"/>
+      <c r="C155" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D155" s="0" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F155" s="0" t="s">
         <v>166</v>
       </c>
+      <c r="I155" s="0" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B156" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D156" s="0" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F156" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="I156" s="0" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B157" s="0" t="s">
         <v>170</v>
       </c>
-      <c r="C157" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="C157" s="2"/>
       <c r="D157" s="0" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F157" s="0" t="s">
         <v>171</v>
@@ -4150,40 +4142,42 @@
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B158" s="0" t="s">
         <v>172</v>
       </c>
       <c r="C158" s="2"/>
       <c r="D158" s="0" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F158" s="0" t="s">
         <v>173</v>
       </c>
+      <c r="I158" s="0" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B159" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="C159" s="2"/>
+        <v>175</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D159" s="0" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F159" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="I159" s="0" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B160" s="0" t="s">
         <v>177</v>
@@ -4192,7 +4186,7 @@
         <v>17</v>
       </c>
       <c r="D160" s="0" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F160" s="0" t="s">
         <v>178</v>
@@ -4200,7 +4194,7 @@
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B161" s="0" t="s">
         <v>179</v>
@@ -4209,7 +4203,7 @@
         <v>17</v>
       </c>
       <c r="D161" s="0" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F161" s="0" t="s">
         <v>180</v>
@@ -4217,7 +4211,7 @@
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B162" s="0" t="s">
         <v>181</v>
@@ -4226,7 +4220,7 @@
         <v>17</v>
       </c>
       <c r="D162" s="0" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F162" s="0" t="s">
         <v>182</v>
@@ -4234,7 +4228,7 @@
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B163" s="0" t="s">
         <v>183</v>
@@ -4243,7 +4237,7 @@
         <v>17</v>
       </c>
       <c r="D163" s="0" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F163" s="0" t="s">
         <v>184</v>
@@ -4251,7 +4245,7 @@
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B164" s="0" t="s">
         <v>185</v>
@@ -4260,7 +4254,7 @@
         <v>17</v>
       </c>
       <c r="D164" s="0" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F164" s="0" t="s">
         <v>186</v>
@@ -4268,7 +4262,7 @@
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B165" s="0" t="s">
         <v>187</v>
@@ -4277,7 +4271,7 @@
         <v>17</v>
       </c>
       <c r="D165" s="0" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F165" s="0" t="s">
         <v>188</v>
@@ -4285,7 +4279,7 @@
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B166" s="0" t="s">
         <v>189</v>
@@ -4294,7 +4288,7 @@
         <v>17</v>
       </c>
       <c r="D166" s="0" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F166" s="0" t="s">
         <v>190</v>
@@ -4302,7 +4296,7 @@
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B167" s="0" t="s">
         <v>191</v>
@@ -4311,7 +4305,7 @@
         <v>17</v>
       </c>
       <c r="D167" s="0" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F167" s="0" t="s">
         <v>192</v>
@@ -4319,16 +4313,14 @@
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B168" s="0" t="s">
         <v>193</v>
       </c>
-      <c r="C168" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="C168" s="2"/>
       <c r="D168" s="0" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F168" s="0" t="s">
         <v>194</v>
@@ -4336,346 +4328,331 @@
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B169" s="0" t="s">
         <v>195</v>
       </c>
-      <c r="C169" s="2"/>
+      <c r="C169" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D169" s="0" t="n">
-        <v>49</v>
-      </c>
-      <c r="F169" s="0" t="s">
-        <v>196</v>
+        <v>50</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B170" s="0" t="s">
+        <v>196</v>
+      </c>
+      <c r="C170" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D170" s="0" t="n">
+        <v>51</v>
+      </c>
+      <c r="E170" s="0" t="s">
         <v>197</v>
       </c>
-      <c r="C170" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D170" s="0" t="n">
-        <v>50</v>
+      <c r="F170" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="G170" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I170" s="0" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B171" s="0" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C171" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D171" s="0" t="n">
-        <v>51</v>
-      </c>
-      <c r="E171" s="0" t="s">
-        <v>199</v>
-      </c>
-      <c r="F171" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="G171" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="I171" s="0" t="s">
-        <v>201</v>
+        <v>52</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B172" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="C172" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D172" s="0" t="n">
+        <v>53</v>
+      </c>
+      <c r="F172" s="0" t="s">
         <v>202</v>
       </c>
-      <c r="C172" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D172" s="0" t="n">
-        <v>52</v>
+      <c r="I172" s="0" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B173" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C173" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D173" s="0" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F173" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="I173" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B174" s="0" t="s">
-        <v>206</v>
-      </c>
-      <c r="C174" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>220</v>
+      </c>
+      <c r="C174" s="2"/>
       <c r="D174" s="0" t="n">
-        <v>54</v>
-      </c>
-      <c r="F174" s="0" t="s">
-        <v>207</v>
-      </c>
-      <c r="I174" s="0" t="s">
-        <v>208</v>
+        <v>55</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B175" s="0" t="s">
-        <v>222</v>
+        <v>31</v>
       </c>
       <c r="C175" s="2"/>
       <c r="D175" s="0" t="n">
-        <v>55</v>
+        <v>1</v>
+      </c>
+      <c r="E175" s="0" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B176" s="0" t="s">
-        <v>31</v>
+        <v>227</v>
       </c>
       <c r="C176" s="2"/>
       <c r="D176" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E176" s="0" t="s">
-        <v>32</v>
+        <v>2</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B177" s="0" t="s">
-        <v>229</v>
+        <v>210</v>
       </c>
       <c r="C177" s="2"/>
       <c r="D177" s="0" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="F177" s="0" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B178" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C178" s="2"/>
       <c r="D178" s="0" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F178" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B179" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C179" s="2"/>
       <c r="D179" s="0" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F179" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B180" s="0" t="s">
-        <v>218</v>
+        <v>42</v>
       </c>
       <c r="C180" s="2"/>
       <c r="D180" s="0" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F180" s="0" t="s">
-        <v>219</v>
+        <v>43</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B181" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="C181" s="2"/>
+        <v>76</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D181" s="0" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F181" s="0" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B182" s="0" t="s">
         <v>228</v>
       </c>
-      <c r="B182" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C182" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="C182" s="2"/>
       <c r="D182" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="F182" s="0" t="s">
-        <v>79</v>
+        <v>8</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B183" s="0" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" s="0" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B184" s="0" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" s="0" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B185" s="0" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" s="0" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B186" s="0" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C186" s="2"/>
       <c r="D186" s="0" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B187" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C187" s="2"/>
       <c r="D187" s="0" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B188" s="0" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C188" s="2"/>
       <c r="D188" s="0" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B189" s="0" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C189" s="2"/>
       <c r="D189" s="0" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B190" s="0" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C190" s="2"/>
       <c r="D190" s="0" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B191" s="0" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C191" s="2"/>
       <c r="D191" s="0" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A192" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="B192" s="0" t="s">
-        <v>239</v>
-      </c>
-      <c r="C192" s="2"/>
-      <c r="D192" s="0" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4685,7 +4662,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A192" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A191" type="list">
       <formula1>_Lists!$B$2:$B$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4697,7 +4674,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C192" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C191" type="list">
       <formula1>_Lists!$C$2:$C$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4705,7 +4682,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D192" type="whole">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D191" type="whole">
       <formula1>-2000000000</formula1>
       <formula2>2000000000</formula2>
     </dataValidation>
@@ -4721,7 +4698,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G192" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G191" type="list">
       <formula1>_Lists!$D$2:$D$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4733,7 +4710,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" prompt="The only valid values here are no value, &quot;yes&quot; or &quot;no&quot;" promptTitle="Boolean value" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="H2:H192" type="list">
+    <dataValidation allowBlank="true" operator="between" prompt="The only valid values here are no value, &quot;yes&quot; or &quot;no&quot;" promptTitle="Boolean value" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="H2:H191" type="list">
       <formula1>_Lists!$A$2:$A$4</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Do most of PDB-196.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45314 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -90,7 +90,7 @@
     <t xml:space="preserve">Date / 10</t>
   </si>
   <si>
-    <t xml:space="preserve">Sheet template</t>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t xml:space="preserve">Column name</t>
@@ -549,19 +549,19 @@
     <t xml:space="preserve">Was a comparator used?</t>
   </si>
   <si>
-    <t xml:space="preserve">Stratification Thickness</t>
+    <t xml:space="preserve">Stratification – Bed Thickness</t>
   </si>
   <si>
     <t xml:space="preserve">BED_THICK_ID$NAME</t>
   </si>
   <si>
-    <t xml:space="preserve">Stratification Features (Primary)</t>
+    <t xml:space="preserve">Stratification – Internal Features Primary</t>
   </si>
   <si>
     <t xml:space="preserve">PRIMARY_BEDDING_ID$NAME</t>
   </si>
   <si>
-    <t xml:space="preserve">Stratification Features (Secondary)</t>
+    <t xml:space="preserve">Stratification - Internal Features Secondary</t>
   </si>
   <si>
     <t xml:space="preserve">SECONDARY_BEDDING_ID$NAME</t>

</xml_diff>

<commit_message>
Add commit support for RowProcessors.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45509 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="242">
   <si>
     <t xml:space="preserve">testExportMetaTemplate</t>
   </si>
@@ -549,7 +549,7 @@
     <t xml:space="preserve">Comparator Used</t>
   </si>
   <si>
-    <t xml:space="preserve">COMPARATOR_USED$CODE</t>
+    <t xml:space="preserve">COMPARATOR_USED</t>
   </si>
   <si>
     <t xml:space="preserve">Was a comparator used?</t>
@@ -1685,7 +1685,7 @@
         <v>125</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I32" s="0" t="s">
         <v>126</v>
@@ -2040,6 +2040,9 @@
       <c r="D49" s="0" t="n">
         <v>49</v>
       </c>
+      <c r="E49" s="0" t="s">
+        <v>175</v>
+      </c>
       <c r="F49" s="0" t="s">
         <v>175</v>
       </c>
@@ -2223,7 +2226,7 @@
         <v>197</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D60" s="0" t="n">
         <v>60</v>
@@ -3107,6 +3110,9 @@
       <c r="D103" s="0" t="n">
         <v>39</v>
       </c>
+      <c r="E103" s="0" t="s">
+        <v>175</v>
+      </c>
       <c r="F103" s="0" t="s">
         <v>175</v>
       </c>
@@ -3290,7 +3296,7 @@
         <v>197</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D114" s="0" t="n">
         <v>50</v>
@@ -4175,6 +4181,9 @@
       <c r="D158" s="0" t="n">
         <v>39</v>
       </c>
+      <c r="E158" s="0" t="s">
+        <v>175</v>
+      </c>
       <c r="F158" s="0" t="s">
         <v>175</v>
       </c>
@@ -4358,7 +4367,7 @@
         <v>197</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D169" s="0" t="n">
         <v>50</v>

</xml_diff>

<commit_message>
Do stages manually. PDB-216.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45590 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -363,7 +363,7 @@
     <t xml:space="preserve">Known Stage Limits – From</t>
   </si>
   <si>
-    <t xml:space="preserve">KNOWN_STAGE_ID$AGE_LOWER_ID$NAME</t>
+    <t xml:space="preserve">KNOWN_STAGE_LOWER</t>
   </si>
   <si>
     <t xml:space="preserve">Enter the lower bound for the known stage.</t>
@@ -372,7 +372,7 @@
     <t xml:space="preserve">Known Stage Limits – To</t>
   </si>
   <si>
-    <t xml:space="preserve">KNOWN_STAGE_ID$AGE_UPPER_ID$NAME</t>
+    <t xml:space="preserve">KNOWN_STAGE_UPPER</t>
   </si>
   <si>
     <t xml:space="preserve">Enter the upport bound for the known stage.</t>
@@ -381,7 +381,7 @@
     <t xml:space="preserve">Inferred Stage Limits – From</t>
   </si>
   <si>
-    <t xml:space="preserve">INFERRED_STAGE_ID$AGE_LOWER_ID$NAME</t>
+    <t xml:space="preserve">INFERRED_STAGE_LOWER</t>
   </si>
   <si>
     <t xml:space="preserve">Enter the lower bound for the inferred stage.</t>
@@ -390,7 +390,7 @@
     <t xml:space="preserve">Inferred Stage Limits – To</t>
   </si>
   <si>
-    <t xml:space="preserve">INFERRED_STAGE_ID$AGE_UPPER_ID$NAME</t>
+    <t xml:space="preserve">INFERRED_STAGE_UPPER</t>
   </si>
   <si>
     <t xml:space="preserve">Enter the upper bound for the inferred stage.</t>
@@ -1601,7 +1601,7 @@
       <c r="D28" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="F28" s="0" t="s">
+      <c r="E28" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I28" s="0" t="s">
@@ -1621,7 +1621,7 @@
       <c r="D29" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="F29" s="0" t="s">
+      <c r="E29" s="0" t="s">
         <v>116</v>
       </c>
       <c r="I29" s="0" t="s">
@@ -1641,7 +1641,7 @@
       <c r="D30" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="F30" s="0" t="s">
+      <c r="E30" s="0" t="s">
         <v>119</v>
       </c>
       <c r="I30" s="0" t="s">
@@ -1661,7 +1661,7 @@
       <c r="D31" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="F31" s="0" t="s">
+      <c r="E31" s="0" t="s">
         <v>122</v>
       </c>
       <c r="I31" s="0" t="s">
@@ -2673,7 +2673,7 @@
       <c r="D82" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="F82" s="0" t="s">
+      <c r="E82" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I82" s="0" t="s">
@@ -2693,7 +2693,7 @@
       <c r="D83" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="F83" s="0" t="s">
+      <c r="E83" s="0" t="s">
         <v>116</v>
       </c>
       <c r="I83" s="0" t="s">
@@ -2713,7 +2713,7 @@
       <c r="D84" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="F84" s="0" t="s">
+      <c r="E84" s="0" t="s">
         <v>119</v>
       </c>
       <c r="I84" s="0" t="s">
@@ -2733,7 +2733,7 @@
       <c r="D85" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="F85" s="0" t="s">
+      <c r="E85" s="0" t="s">
         <v>122</v>
       </c>
       <c r="I85" s="0" t="s">
@@ -3742,7 +3742,7 @@
       <c r="D137" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="F137" s="0" t="s">
+      <c r="E137" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I137" s="0" t="s">
@@ -3762,7 +3762,7 @@
       <c r="D138" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="F138" s="0" t="s">
+      <c r="E138" s="0" t="s">
         <v>116</v>
       </c>
       <c r="I138" s="0" t="s">
@@ -3782,7 +3782,7 @@
       <c r="D139" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="F139" s="0" t="s">
+      <c r="E139" s="0" t="s">
         <v>119</v>
       </c>
       <c r="I139" s="0" t="s">
@@ -3802,7 +3802,7 @@
       <c r="D140" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="F140" s="0" t="s">
+      <c r="E140" s="0" t="s">
         <v>122</v>
       </c>
       <c r="I140" s="0" t="s">

</xml_diff>

<commit_message>
PDB-217: Do the audit stuff manually.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45591 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="241">
   <si>
     <t xml:space="preserve">testExportMetaTemplate</t>
   </si>
@@ -661,9 +661,6 @@
   </si>
   <si>
     <t xml:space="preserve">Enter the name of a previously entered and approved vertical section.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUDIT_ID$WORKING_COMMENTS</t>
   </si>
   <si>
     <t xml:space="preserve">Bottom Depth</t>
@@ -2368,8 +2365,8 @@
       <c r="D67" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F67" s="0" t="s">
-        <v>213</v>
+      <c r="E67" s="0" t="s">
+        <v>44</v>
       </c>
       <c r="I67" s="0" t="s">
         <v>45</v>
@@ -2380,17 +2377,17 @@
         <v>210</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" s="0" t="n">
         <v>4</v>
       </c>
       <c r="F68" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="I68" s="0" t="s">
         <v>215</v>
-      </c>
-      <c r="I68" s="0" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2398,17 +2395,17 @@
         <v>210</v>
       </c>
       <c r="B69" s="0" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" s="0" t="n">
         <v>5</v>
       </c>
       <c r="F69" s="0" t="s">
+        <v>217</v>
+      </c>
+      <c r="I69" s="0" t="s">
         <v>218</v>
-      </c>
-      <c r="I69" s="0" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2416,17 +2413,17 @@
         <v>210</v>
       </c>
       <c r="B70" s="0" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" s="0" t="n">
         <v>6</v>
       </c>
       <c r="F70" s="0" t="s">
+        <v>220</v>
+      </c>
+      <c r="I70" s="0" t="s">
         <v>221</v>
-      </c>
-      <c r="I70" s="0" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2783,7 +2780,7 @@
         <v>5</v>
       </c>
       <c r="I87" s="0" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3390,19 +3387,19 @@
         <v>210</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C119" s="2"/>
       <c r="D119" s="0" t="n">
         <v>55</v>
       </c>
       <c r="I119" s="0" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B120" s="0" t="s">
         <v>31</v>
@@ -3422,10 +3419,10 @@
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B121" s="0" t="s">
         <v>226</v>
-      </c>
-      <c r="B121" s="0" t="s">
-        <v>227</v>
       </c>
       <c r="C121" s="2" t="s">
         <v>14</v>
@@ -3442,79 +3439,76 @@
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" s="0" t="n">
         <v>3</v>
       </c>
       <c r="F122" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="I122" s="0" t="s">
         <v>215</v>
-      </c>
-      <c r="I122" s="0" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" s="0" t="n">
         <v>4</v>
       </c>
       <c r="F123" s="0" t="s">
+        <v>217</v>
+      </c>
+      <c r="I123" s="0" t="s">
         <v>218</v>
-      </c>
-      <c r="I123" s="0" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B124" s="0" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" s="0" t="n">
         <v>5</v>
       </c>
       <c r="F124" s="0" t="s">
+        <v>220</v>
+      </c>
+      <c r="I124" s="0" t="s">
         <v>221</v>
-      </c>
-      <c r="I124" s="0" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B125" s="0" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" s="0" t="n">
         <v>6</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>229</v>
-      </c>
-      <c r="I125" s="0" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B126" s="0" t="s">
         <v>78</v>
@@ -3534,7 +3528,7 @@
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B127" s="0" t="s">
         <v>81</v>
@@ -3552,7 +3546,7 @@
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B128" s="0" t="s">
         <v>84</v>
@@ -3576,7 +3570,7 @@
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B129" s="0" t="s">
         <v>89</v>
@@ -3591,7 +3585,7 @@
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B130" s="0" t="s">
         <v>92</v>
@@ -3611,7 +3605,7 @@
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B131" s="0" t="s">
         <v>95</v>
@@ -3631,7 +3625,7 @@
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B132" s="0" t="s">
         <v>98</v>
@@ -3654,7 +3648,7 @@
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B133" s="0" t="s">
         <v>101</v>
@@ -3674,7 +3668,7 @@
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B134" s="0" t="s">
         <v>104</v>
@@ -3691,7 +3685,7 @@
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B135" s="0" t="s">
         <v>106</v>
@@ -3711,7 +3705,7 @@
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B136" s="0" t="s">
         <v>109</v>
@@ -3731,7 +3725,7 @@
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B137" s="0" t="s">
         <v>112</v>
@@ -3751,7 +3745,7 @@
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B138" s="0" t="s">
         <v>115</v>
@@ -3771,7 +3765,7 @@
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B139" s="0" t="s">
         <v>118</v>
@@ -3791,7 +3785,7 @@
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B140" s="0" t="s">
         <v>121</v>
@@ -3811,7 +3805,7 @@
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B141" s="0" t="s">
         <v>124</v>
@@ -3834,7 +3828,7 @@
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B142" s="0" t="s">
         <v>127</v>
@@ -3852,12 +3846,12 @@
         <v>5</v>
       </c>
       <c r="I142" s="0" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B143" s="0" t="s">
         <v>130</v>
@@ -3880,7 +3874,7 @@
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B144" s="0" t="s">
         <v>133</v>
@@ -3903,7 +3897,7 @@
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B145" s="0" t="s">
         <v>136</v>
@@ -3926,7 +3920,7 @@
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B146" s="0" t="s">
         <v>139</v>
@@ -3949,7 +3943,7 @@
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B147" s="0" t="s">
         <v>142</v>
@@ -3972,7 +3966,7 @@
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B148" s="0" t="s">
         <v>145</v>
@@ -3995,7 +3989,7 @@
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B149" s="0" t="s">
         <v>148</v>
@@ -4024,7 +4018,7 @@
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B150" s="0" t="s">
         <v>152</v>
@@ -4047,7 +4041,7 @@
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B151" s="0" t="s">
         <v>156</v>
@@ -4067,7 +4061,7 @@
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B152" s="0" t="s">
         <v>159</v>
@@ -4085,7 +4079,7 @@
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B153" s="0" t="s">
         <v>162</v>
@@ -4105,7 +4099,7 @@
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B154" s="0" t="s">
         <v>165</v>
@@ -4120,7 +4114,7 @@
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B155" s="0" t="s">
         <v>167</v>
@@ -4140,7 +4134,7 @@
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B156" s="0" t="s">
         <v>170</v>
@@ -4157,7 +4151,7 @@
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B157" s="0" t="s">
         <v>172</v>
@@ -4172,7 +4166,7 @@
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B158" s="0" t="s">
         <v>174</v>
@@ -4193,7 +4187,7 @@
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B159" s="0" t="s">
         <v>177</v>
@@ -4210,7 +4204,7 @@
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B160" s="0" t="s">
         <v>179</v>
@@ -4227,7 +4221,7 @@
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B161" s="0" t="s">
         <v>181</v>
@@ -4244,7 +4238,7 @@
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B162" s="0" t="s">
         <v>183</v>
@@ -4261,7 +4255,7 @@
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B163" s="0" t="s">
         <v>185</v>
@@ -4278,7 +4272,7 @@
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B164" s="0" t="s">
         <v>187</v>
@@ -4295,7 +4289,7 @@
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B165" s="0" t="s">
         <v>189</v>
@@ -4312,7 +4306,7 @@
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B166" s="0" t="s">
         <v>191</v>
@@ -4329,7 +4323,7 @@
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B167" s="0" t="s">
         <v>193</v>
@@ -4346,7 +4340,7 @@
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B168" s="0" t="s">
         <v>195</v>
@@ -4361,7 +4355,7 @@
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B169" s="0" t="s">
         <v>197</v>
@@ -4378,7 +4372,7 @@
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B170" s="0" t="s">
         <v>199</v>
@@ -4404,7 +4398,7 @@
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B171" s="0" t="s">
         <v>203</v>
@@ -4418,7 +4412,7 @@
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B172" s="0" t="s">
         <v>204</v>
@@ -4438,7 +4432,7 @@
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B173" s="0" t="s">
         <v>207</v>
@@ -4458,10 +4452,10 @@
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B174" s="0" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C174" s="2"/>
       <c r="D174" s="0" t="n">
@@ -4470,7 +4464,7 @@
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B175" s="0" t="s">
         <v>31</v>
@@ -4485,10 +4479,10 @@
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B176" s="0" t="s">
         <v>230</v>
-      </c>
-      <c r="B176" s="0" t="s">
-        <v>231</v>
       </c>
       <c r="C176" s="2"/>
       <c r="D176" s="0" t="n">
@@ -4497,52 +4491,52 @@
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B177" s="0" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C177" s="2"/>
       <c r="D177" s="0" t="n">
         <v>3</v>
       </c>
       <c r="F177" s="0" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B178" s="0" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C178" s="2"/>
       <c r="D178" s="0" t="n">
         <v>4</v>
       </c>
       <c r="F178" s="0" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B179" s="0" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C179" s="2"/>
       <c r="D179" s="0" t="n">
         <v>5</v>
       </c>
       <c r="F179" s="0" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B180" s="0" t="s">
         <v>43</v>
@@ -4551,13 +4545,13 @@
       <c r="D180" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F180" s="0" t="s">
-        <v>213</v>
+      <c r="E180" s="0" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B181" s="0" t="s">
         <v>78</v>
@@ -4574,10 +4568,10 @@
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B182" s="0" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C182" s="2"/>
       <c r="D182" s="0" t="n">
@@ -4586,10 +4580,10 @@
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B183" s="0" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" s="0" t="n">
@@ -4598,10 +4592,10 @@
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B184" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" s="0" t="n">
@@ -4610,10 +4604,10 @@
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B185" s="0" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" s="0" t="n">
@@ -4622,10 +4616,10 @@
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B186" s="0" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C186" s="2"/>
       <c r="D186" s="0" t="n">
@@ -4634,10 +4628,10 @@
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B187" s="0" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C187" s="2"/>
       <c r="D187" s="0" t="n">
@@ -4646,10 +4640,10 @@
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B188" s="0" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C188" s="2"/>
       <c r="D188" s="0" t="n">
@@ -4658,10 +4652,10 @@
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B189" s="0" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C189" s="2"/>
       <c r="D189" s="0" t="n">
@@ -4670,10 +4664,10 @@
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B190" s="0" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C190" s="2"/>
       <c r="D190" s="0" t="n">
@@ -4682,10 +4676,10 @@
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B191" s="0" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C191" s="2"/>
       <c r="D191" s="0" t="n">

</xml_diff>

<commit_message>
Remove confidential field. Make "WORKING COMMENTS" optional.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45593 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="241">
   <si>
     <t xml:space="preserve">testExportMetaTemplate</t>
   </si>
@@ -1015,7 +1015,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I191"/>
+  <dimension ref="A1:I190"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -4452,14 +4452,17 @@
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="2" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B174" s="0" t="s">
-        <v>223</v>
+        <v>31</v>
       </c>
       <c r="C174" s="2"/>
       <c r="D174" s="0" t="n">
-        <v>55</v>
+        <v>1</v>
+      </c>
+      <c r="E174" s="0" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4467,14 +4470,11 @@
         <v>229</v>
       </c>
       <c r="B175" s="0" t="s">
-        <v>31</v>
+        <v>230</v>
       </c>
       <c r="C175" s="2"/>
       <c r="D175" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E175" s="0" t="s">
-        <v>32</v>
+        <v>2</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4482,11 +4482,14 @@
         <v>229</v>
       </c>
       <c r="B176" s="0" t="s">
-        <v>230</v>
+        <v>213</v>
       </c>
       <c r="C176" s="2"/>
       <c r="D176" s="0" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="F176" s="0" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4494,14 +4497,14 @@
         <v>229</v>
       </c>
       <c r="B177" s="0" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="C177" s="2"/>
       <c r="D177" s="0" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F177" s="0" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4509,14 +4512,14 @@
         <v>229</v>
       </c>
       <c r="B178" s="0" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="C178" s="2"/>
       <c r="D178" s="0" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F178" s="0" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4524,14 +4527,14 @@
         <v>229</v>
       </c>
       <c r="B179" s="0" t="s">
-        <v>219</v>
+        <v>43</v>
       </c>
       <c r="C179" s="2"/>
       <c r="D179" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="F179" s="0" t="s">
-        <v>220</v>
+        <v>6</v>
+      </c>
+      <c r="E179" s="0" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4539,14 +4542,16 @@
         <v>229</v>
       </c>
       <c r="B180" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="C180" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="C180" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D180" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="E180" s="0" t="s">
-        <v>44</v>
+        <v>7</v>
+      </c>
+      <c r="F180" s="0" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4554,16 +4559,11 @@
         <v>229</v>
       </c>
       <c r="B181" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C181" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>231</v>
+      </c>
+      <c r="C181" s="2"/>
       <c r="D181" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="F181" s="0" t="s">
-        <v>79</v>
+        <v>8</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4571,11 +4571,11 @@
         <v>229</v>
       </c>
       <c r="B182" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C182" s="2"/>
       <c r="D182" s="0" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4583,11 +4583,11 @@
         <v>229</v>
       </c>
       <c r="B183" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" s="0" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4595,11 +4595,11 @@
         <v>229</v>
       </c>
       <c r="B184" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" s="0" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4607,11 +4607,11 @@
         <v>229</v>
       </c>
       <c r="B185" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" s="0" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4619,11 +4619,11 @@
         <v>229</v>
       </c>
       <c r="B186" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C186" s="2"/>
       <c r="D186" s="0" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4631,11 +4631,11 @@
         <v>229</v>
       </c>
       <c r="B187" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C187" s="2"/>
       <c r="D187" s="0" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4643,11 +4643,11 @@
         <v>229</v>
       </c>
       <c r="B188" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C188" s="2"/>
       <c r="D188" s="0" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4655,11 +4655,11 @@
         <v>229</v>
       </c>
       <c r="B189" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C189" s="2"/>
       <c r="D189" s="0" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4667,22 +4667,10 @@
         <v>229</v>
       </c>
       <c r="B190" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C190" s="2"/>
       <c r="D190" s="0" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A191" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="B191" s="0" t="s">
-        <v>240</v>
-      </c>
-      <c r="C191" s="2"/>
-      <c r="D191" s="0" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4692,7 +4680,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A191" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A190" type="list">
       <formula1>_Lists!$B$2:$B$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4704,7 +4692,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C191" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C190" type="list">
       <formula1>_Lists!$C$2:$C$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4712,7 +4700,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D191" type="whole">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D190" type="whole">
       <formula1>-2000000000</formula1>
       <formula2>2000000000</formula2>
     </dataValidation>
@@ -4728,7 +4716,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G191" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G190" type="list">
       <formula1>_Lists!$D$2:$D$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4740,7 +4728,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" prompt="The only valid values here are no value, &quot;yes&quot; or &quot;no&quot;" promptTitle="Boolean value" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="H2:H191" type="list">
+    <dataValidation allowBlank="true" operator="between" prompt="The only valid values here are no value, &quot;yes&quot; or &quot;no&quot;" promptTitle="Boolean value" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="H2:H190" type="list">
       <formula1>_Lists!$A$2:$A$4</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Remove columns that we don't know what to do with.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45594 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="895" uniqueCount="238">
   <si>
     <t xml:space="preserve">testExportMetaTemplate</t>
   </si>
@@ -633,9 +633,6 @@
     <t xml:space="preserve">Enter one of “Marine” or “Non Marine”</t>
   </si>
   <si>
-    <t xml:space="preserve">Environmental Features</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nature of Rock Unit</t>
   </si>
   <si>
@@ -691,12 +688,6 @@
   </si>
   <si>
     <t xml:space="preserve">For a Sample Relationship, “c.” or “?”. TODO: what do these mean?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confidential</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TODO: What does this column do?</t>
   </si>
   <si>
     <t xml:space="preserve">Drill Hole / 4</t>
@@ -1015,7 +1006,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I190"/>
+  <dimension ref="A1:I186"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -2269,7 +2260,13 @@
         <v>14</v>
       </c>
       <c r="D62" s="0" t="n">
-        <v>62</v>
+        <v>63</v>
+      </c>
+      <c r="F62" s="0" t="s">
+        <v>204</v>
+      </c>
+      <c r="I62" s="0" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2277,2400 +2274,2337 @@
         <v>30</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D63" s="0" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>30</v>
+        <v>209</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>207</v>
+        <v>31</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D64" s="0" t="n">
-        <v>64</v>
-      </c>
-      <c r="F64" s="0" t="s">
-        <v>208</v>
+        <v>1</v>
+      </c>
+      <c r="E64" s="0" t="s">
+        <v>32</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>209</v>
+        <v>33</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B65" s="0" t="s">
         <v>210</v>
       </c>
-      <c r="B65" s="0" t="s">
-        <v>31</v>
-      </c>
       <c r="C65" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D65" s="0" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="I65" s="0" t="s">
-        <v>33</v>
+        <v>211</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>211</v>
+        <v>43</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D66" s="0" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="I66" s="0" t="s">
-        <v>212</v>
+        <v>45</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>212</v>
+      </c>
+      <c r="C67" s="2"/>
       <c r="D67" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="E67" s="0" t="s">
-        <v>44</v>
+        <v>4</v>
+      </c>
+      <c r="F67" s="0" t="s">
+        <v>213</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>45</v>
+        <v>214</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" s="0" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="I68" s="0" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B69" s="0" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" s="0" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I69" s="0" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B70" s="0" t="s">
-        <v>219</v>
-      </c>
-      <c r="C70" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D70" s="0" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F70" s="0" t="s">
-        <v>220</v>
+        <v>79</v>
       </c>
       <c r="I70" s="0" t="s">
-        <v>221</v>
+        <v>80</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B71" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="C71" s="2"/>
       <c r="D71" s="0" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F71" s="0" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="I71" s="0" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B72" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="C72" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D72" s="0" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="E72" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="F72" s="0" t="s">
-        <v>82</v>
+        <v>86</v>
+      </c>
+      <c r="G72" s="0" t="s">
+        <v>87</v>
       </c>
       <c r="I72" s="0" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B73" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="C73" s="2"/>
       <c r="D73" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E73" s="0" t="s">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="F73" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="G73" s="0" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="I73" s="0" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B74" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="C74" s="2"/>
+        <v>92</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D74" s="0" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F74" s="0" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="I74" s="0" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D75" s="0" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F75" s="0" t="s">
-        <v>93</v>
+        <v>96</v>
+      </c>
+      <c r="G75" s="0" t="s">
+        <v>87</v>
       </c>
       <c r="I75" s="0" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D76" s="0" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F76" s="0" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="G76" s="0" t="s">
         <v>87</v>
       </c>
       <c r="I76" s="0" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B77" s="0" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D77" s="0" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F77" s="0" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="G77" s="0" t="s">
         <v>87</v>
       </c>
       <c r="I77" s="0" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B78" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D78" s="0" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F78" s="0" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G78" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="I78" s="0" t="s">
-        <v>103</v>
-      </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B79" s="0" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D79" s="0" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F79" s="0" t="s">
-        <v>105</v>
-      </c>
-      <c r="G79" s="0" t="s">
-        <v>87</v>
+        <v>107</v>
+      </c>
+      <c r="I79" s="0" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B80" s="0" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D80" s="0" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F80" s="0" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I80" s="0" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B81" s="0" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D81" s="0" t="n">
-        <v>17</v>
-      </c>
-      <c r="F81" s="0" t="s">
-        <v>110</v>
+        <v>18</v>
+      </c>
+      <c r="E81" s="0" t="s">
+        <v>113</v>
       </c>
       <c r="I81" s="0" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B82" s="0" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D82" s="0" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E82" s="0" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="I82" s="0" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B83" s="0" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D83" s="0" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E83" s="0" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="I83" s="0" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B84" s="0" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D84" s="0" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E84" s="0" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="I84" s="0" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B85" s="0" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D85" s="0" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E85" s="0" t="s">
-        <v>122</v>
+        <v>125</v>
+      </c>
+      <c r="H85" s="0" t="s">
+        <v>5</v>
       </c>
       <c r="I85" s="0" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B86" s="0" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D86" s="0" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E86" s="0" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="H86" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I86" s="0" t="s">
-        <v>126</v>
+        <v>221</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B87" s="0" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D87" s="0" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="H87" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I87" s="0" t="s">
-        <v>222</v>
+        <v>132</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D88" s="0" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="H88" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I88" s="0" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B89" s="0" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D89" s="0" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="H89" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I89" s="0" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B90" s="0" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D90" s="0" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="H90" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I90" s="0" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B91" s="0" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D91" s="0" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E91" s="0" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="H91" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I91" s="0" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D92" s="0" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="H92" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I92" s="0" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C93" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D93" s="0" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E93" s="0" t="s">
-        <v>146</v>
+        <v>149</v>
+      </c>
+      <c r="F93" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="G93" s="0" t="s">
+        <v>87</v>
       </c>
       <c r="H93" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I93" s="0" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="C94" s="2"/>
       <c r="D94" s="0" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E94" s="0" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F94" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="G94" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="H94" s="0" t="s">
-        <v>5</v>
+        <v>154</v>
       </c>
       <c r="I94" s="0" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="C95" s="2"/>
+        <v>156</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D95" s="0" t="n">
-        <v>31</v>
-      </c>
-      <c r="E95" s="0" t="s">
-        <v>153</v>
+        <v>32</v>
       </c>
       <c r="F95" s="0" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="I95" s="0" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B96" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="C96" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="C96" s="2"/>
       <c r="D96" s="0" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F96" s="0" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I96" s="0" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B97" s="0" t="s">
-        <v>159</v>
-      </c>
-      <c r="C97" s="2"/>
+        <v>162</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D97" s="0" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F97" s="0" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="I97" s="0" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>162</v>
-      </c>
-      <c r="C98" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="C98" s="2"/>
       <c r="D98" s="0" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F98" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="I98" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B99" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="C99" s="2"/>
+        <v>167</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D99" s="0" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F99" s="0" t="s">
-        <v>166</v>
+        <v>168</v>
+      </c>
+      <c r="I99" s="0" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B100" s="0" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D100" s="0" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F100" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="I100" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B101" s="0" t="s">
-        <v>170</v>
-      </c>
-      <c r="C101" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="C101" s="2"/>
       <c r="D101" s="0" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F101" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B102" s="0" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" s="0" t="n">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="E102" s="0" t="s">
+        <v>175</v>
       </c>
       <c r="F102" s="0" t="s">
-        <v>173</v>
+        <v>175</v>
+      </c>
+      <c r="I102" s="0" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B103" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="C103" s="2"/>
+        <v>177</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D103" s="0" t="n">
-        <v>39</v>
-      </c>
-      <c r="E103" s="0" t="s">
-        <v>175</v>
+        <v>40</v>
       </c>
       <c r="F103" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="I103" s="0" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B104" s="0" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C104" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D104" s="0" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F104" s="0" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B105" s="0" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C105" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D105" s="0" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F105" s="0" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B106" s="0" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C106" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D106" s="0" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F106" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B107" s="0" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C107" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D107" s="0" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F107" s="0" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C108" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D108" s="0" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F108" s="0" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B109" s="0" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C109" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D109" s="0" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F109" s="0" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B110" s="0" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C110" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D110" s="0" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F110" s="0" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B111" s="0" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C111" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D111" s="0" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F111" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B112" s="0" t="s">
-        <v>193</v>
-      </c>
-      <c r="C112" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>195</v>
+      </c>
+      <c r="C112" s="2"/>
       <c r="D112" s="0" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F112" s="0" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B113" s="0" t="s">
-        <v>195</v>
-      </c>
-      <c r="C113" s="2"/>
+        <v>197</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D113" s="0" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F113" s="0" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B114" s="0" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D114" s="0" t="n">
-        <v>50</v>
+        <v>51</v>
+      </c>
+      <c r="E114" s="0" t="s">
+        <v>200</v>
       </c>
       <c r="F114" s="0" t="s">
-        <v>198</v>
+        <v>201</v>
+      </c>
+      <c r="G114" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I114" s="0" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C115" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D115" s="0" t="n">
-        <v>51</v>
-      </c>
-      <c r="E115" s="0" t="s">
-        <v>200</v>
+        <v>53</v>
       </c>
       <c r="F115" s="0" t="s">
-        <v>201</v>
-      </c>
-      <c r="G115" s="0" t="s">
-        <v>12</v>
+        <v>204</v>
       </c>
       <c r="I115" s="0" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B116" s="0" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C116" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D116" s="0" t="n">
-        <v>52</v>
+        <v>54</v>
+      </c>
+      <c r="F116" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="I116" s="0" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="2" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="B117" s="0" t="s">
-        <v>204</v>
+        <v>31</v>
       </c>
       <c r="C117" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D117" s="0" t="n">
-        <v>53</v>
-      </c>
-      <c r="F117" s="0" t="s">
-        <v>205</v>
+        <v>1</v>
+      </c>
+      <c r="E117" s="0" t="s">
+        <v>32</v>
       </c>
       <c r="I117" s="0" t="s">
-        <v>206</v>
+        <v>33</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="2" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="B118" s="0" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
       <c r="C118" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D118" s="0" t="n">
-        <v>54</v>
-      </c>
-      <c r="F118" s="0" t="s">
-        <v>208</v>
+        <v>2</v>
+      </c>
+      <c r="E118" s="0" t="s">
+        <v>35</v>
       </c>
       <c r="I118" s="0" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="2" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="C119" s="2"/>
       <c r="D119" s="0" t="n">
-        <v>55</v>
+        <v>3</v>
+      </c>
+      <c r="F119" s="0" t="s">
+        <v>213</v>
       </c>
       <c r="I119" s="0" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B120" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="C120" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>215</v>
+      </c>
+      <c r="C120" s="2"/>
       <c r="D120" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E120" s="0" t="s">
-        <v>32</v>
+        <v>4</v>
+      </c>
+      <c r="F120" s="0" t="s">
+        <v>216</v>
       </c>
       <c r="I120" s="0" t="s">
-        <v>33</v>
+        <v>217</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>226</v>
-      </c>
-      <c r="C121" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>218</v>
+      </c>
+      <c r="C121" s="2"/>
       <c r="D121" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E121" s="0" t="s">
-        <v>35</v>
+        <v>5</v>
+      </c>
+      <c r="F121" s="0" t="s">
+        <v>219</v>
       </c>
       <c r="I121" s="0" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" s="0" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F122" s="0" t="s">
-        <v>214</v>
-      </c>
-      <c r="I122" s="0" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>216</v>
-      </c>
-      <c r="C123" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D123" s="0" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F123" s="0" t="s">
-        <v>217</v>
+        <v>79</v>
       </c>
       <c r="I123" s="0" t="s">
-        <v>218</v>
+        <v>80</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B124" s="0" t="s">
-        <v>219</v>
+        <v>81</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" s="0" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F124" s="0" t="s">
-        <v>220</v>
+        <v>82</v>
       </c>
       <c r="I124" s="0" t="s">
-        <v>221</v>
+        <v>83</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B125" s="0" t="s">
-        <v>227</v>
+        <v>84</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" s="0" t="n">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="E125" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>228</v>
+        <v>86</v>
+      </c>
+      <c r="G125" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="I125" s="0" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="C126" s="2"/>
       <c r="D126" s="0" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F126" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="I126" s="0" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="C127" s="2"/>
+        <v>92</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D127" s="0" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F127" s="0" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="I127" s="0" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="C128" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D128" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E128" s="0" t="s">
-        <v>85</v>
+        <v>12</v>
       </c>
       <c r="F128" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="G128" s="0" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="I128" s="0" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="C129" s="2"/>
+        <v>98</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D129" s="0" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F129" s="0" t="s">
-        <v>90</v>
+        <v>99</v>
+      </c>
+      <c r="G129" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="I129" s="0" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B130" s="0" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D130" s="0" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F130" s="0" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="I130" s="0" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B131" s="0" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D131" s="0" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F131" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="I131" s="0" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B132" s="0" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D132" s="0" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F132" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="G132" s="0" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="I132" s="0" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B133" s="0" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D133" s="0" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F133" s="0" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="I133" s="0" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B134" s="0" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D134" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="F134" s="0" t="s">
-        <v>105</v>
+        <v>18</v>
+      </c>
+      <c r="E134" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="I134" s="0" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B135" s="0" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D135" s="0" t="n">
-        <v>16</v>
-      </c>
-      <c r="F135" s="0" t="s">
-        <v>107</v>
+        <v>19</v>
+      </c>
+      <c r="E135" s="0" t="s">
+        <v>116</v>
       </c>
       <c r="I135" s="0" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B136" s="0" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D136" s="0" t="n">
-        <v>17</v>
-      </c>
-      <c r="F136" s="0" t="s">
-        <v>110</v>
+        <v>20</v>
+      </c>
+      <c r="E136" s="0" t="s">
+        <v>119</v>
       </c>
       <c r="I136" s="0" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B137" s="0" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="C137" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D137" s="0" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E137" s="0" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="I137" s="0" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B138" s="0" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D138" s="0" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E138" s="0" t="s">
-        <v>116</v>
+        <v>125</v>
+      </c>
+      <c r="H138" s="0" t="s">
+        <v>5</v>
       </c>
       <c r="I138" s="0" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B139" s="0" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="C139" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D139" s="0" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E139" s="0" t="s">
-        <v>119</v>
+        <v>128</v>
+      </c>
+      <c r="H139" s="0" t="s">
+        <v>5</v>
       </c>
       <c r="I139" s="0" t="s">
-        <v>120</v>
+        <v>221</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B140" s="0" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D140" s="0" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E140" s="0" t="s">
-        <v>122</v>
+        <v>131</v>
+      </c>
+      <c r="H140" s="0" t="s">
+        <v>5</v>
       </c>
       <c r="I140" s="0" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B141" s="0" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D141" s="0" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E141" s="0" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="H141" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I141" s="0" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B142" s="0" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D142" s="0" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E142" s="0" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="H142" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I142" s="0" t="s">
-        <v>222</v>
+        <v>138</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B143" s="0" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D143" s="0" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E143" s="0" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="H143" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I143" s="0" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B144" s="0" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D144" s="0" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E144" s="0" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H144" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I144" s="0" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B145" s="0" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D145" s="0" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E145" s="0" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="H145" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I145" s="0" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B146" s="0" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="C146" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D146" s="0" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E146" s="0" t="s">
-        <v>140</v>
+        <v>149</v>
+      </c>
+      <c r="F146" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="G146" s="0" t="s">
+        <v>87</v>
       </c>
       <c r="H146" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I146" s="0" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B147" s="0" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="C147" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D147" s="0" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E147" s="0" t="s">
-        <v>143</v>
-      </c>
-      <c r="H147" s="0" t="s">
-        <v>5</v>
+        <v>153</v>
+      </c>
+      <c r="F147" s="0" t="s">
+        <v>154</v>
       </c>
       <c r="I147" s="0" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B148" s="0" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D148" s="0" t="n">
-        <v>29</v>
-      </c>
-      <c r="E148" s="0" t="s">
-        <v>146</v>
-      </c>
-      <c r="H148" s="0" t="s">
-        <v>5</v>
+        <v>32</v>
+      </c>
+      <c r="F148" s="0" t="s">
+        <v>157</v>
       </c>
       <c r="I148" s="0" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B149" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="C149" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="C149" s="2"/>
       <c r="D149" s="0" t="n">
-        <v>30</v>
-      </c>
-      <c r="E149" s="0" t="s">
-        <v>149</v>
+        <v>33</v>
       </c>
       <c r="F149" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="G149" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="H149" s="0" t="s">
-        <v>5</v>
+        <v>160</v>
       </c>
       <c r="I149" s="0" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B150" s="0" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D150" s="0" t="n">
-        <v>31</v>
-      </c>
-      <c r="E150" s="0" t="s">
-        <v>153</v>
+        <v>34</v>
       </c>
       <c r="F150" s="0" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="I150" s="0" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B151" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="C151" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="C151" s="2"/>
       <c r="D151" s="0" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F151" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="I151" s="0" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B152" s="0" t="s">
-        <v>159</v>
-      </c>
-      <c r="C152" s="2"/>
+        <v>167</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D152" s="0" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F152" s="0" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="I152" s="0" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B153" s="0" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D153" s="0" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F153" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="I153" s="0" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B154" s="0" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C154" s="2"/>
       <c r="D154" s="0" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F154" s="0" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B155" s="0" t="s">
-        <v>167</v>
-      </c>
-      <c r="C155" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="C155" s="2"/>
       <c r="D155" s="0" t="n">
-        <v>36</v>
+        <v>39</v>
+      </c>
+      <c r="E155" s="0" t="s">
+        <v>175</v>
       </c>
       <c r="F155" s="0" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I155" s="0" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B156" s="0" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C156" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D156" s="0" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F156" s="0" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B157" s="0" t="s">
-        <v>172</v>
-      </c>
-      <c r="C157" s="2"/>
+        <v>179</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D157" s="0" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F157" s="0" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B158" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="C158" s="2"/>
+        <v>181</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D158" s="0" t="n">
-        <v>39</v>
-      </c>
-      <c r="E158" s="0" t="s">
-        <v>175</v>
+        <v>42</v>
       </c>
       <c r="F158" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="I158" s="0" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B159" s="0" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="C159" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D159" s="0" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F159" s="0" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B160" s="0" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C160" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D160" s="0" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F160" s="0" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B161" s="0" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C161" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D161" s="0" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F161" s="0" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B162" s="0" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C162" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D162" s="0" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F162" s="0" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B163" s="0" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C163" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D163" s="0" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F163" s="0" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B164" s="0" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="C164" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D164" s="0" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F164" s="0" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B165" s="0" t="s">
-        <v>189</v>
-      </c>
-      <c r="C165" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>195</v>
+      </c>
+      <c r="C165" s="2"/>
       <c r="D165" s="0" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F165" s="0" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B166" s="0" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="C166" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D166" s="0" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F166" s="0" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B167" s="0" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D167" s="0" t="n">
-        <v>48</v>
+        <v>51</v>
+      </c>
+      <c r="E167" s="0" t="s">
+        <v>200</v>
       </c>
       <c r="F167" s="0" t="s">
-        <v>194</v>
+        <v>201</v>
+      </c>
+      <c r="G167" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I167" s="0" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B168" s="0" t="s">
-        <v>195</v>
-      </c>
-      <c r="C168" s="2"/>
+        <v>203</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D168" s="0" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F168" s="0" t="s">
-        <v>196</v>
+        <v>204</v>
+      </c>
+      <c r="I168" s="0" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B169" s="0" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D169" s="0" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F169" s="0" t="s">
-        <v>198</v>
+        <v>207</v>
+      </c>
+      <c r="I169" s="0" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B170" s="0" t="s">
-        <v>199</v>
-      </c>
-      <c r="C170" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="C170" s="2"/>
       <c r="D170" s="0" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="E170" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="F170" s="0" t="s">
-        <v>201</v>
-      </c>
-      <c r="G170" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="I170" s="0" t="s">
-        <v>202</v>
+        <v>32</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B171" s="0" t="s">
-        <v>203</v>
-      </c>
-      <c r="C171" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="C171" s="2"/>
       <c r="D171" s="0" t="n">
-        <v>52</v>
+        <v>2</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B172" s="0" t="s">
-        <v>204</v>
-      </c>
-      <c r="C172" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>212</v>
+      </c>
+      <c r="C172" s="2"/>
       <c r="D172" s="0" t="n">
-        <v>53</v>
+        <v>3</v>
       </c>
       <c r="F172" s="0" t="s">
-        <v>205</v>
-      </c>
-      <c r="I172" s="0" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B173" s="0" t="s">
-        <v>207</v>
-      </c>
-      <c r="C173" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>215</v>
+      </c>
+      <c r="C173" s="2"/>
       <c r="D173" s="0" t="n">
-        <v>54</v>
+        <v>4</v>
       </c>
       <c r="F173" s="0" t="s">
-        <v>208</v>
-      </c>
-      <c r="I173" s="0" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B174" s="0" t="s">
-        <v>31</v>
+        <v>218</v>
       </c>
       <c r="C174" s="2"/>
       <c r="D174" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E174" s="0" t="s">
-        <v>32</v>
+        <v>5</v>
+      </c>
+      <c r="F174" s="0" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B175" s="0" t="s">
-        <v>230</v>
+        <v>43</v>
       </c>
       <c r="C175" s="2"/>
       <c r="D175" s="0" t="n">
-        <v>2</v>
+        <v>6</v>
+      </c>
+      <c r="E175" s="0" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B176" s="0" t="s">
-        <v>213</v>
-      </c>
-      <c r="C176" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="C176" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D176" s="0" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F176" s="0" t="s">
-        <v>214</v>
+        <v>79</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B177" s="0" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="C177" s="2"/>
       <c r="D177" s="0" t="n">
-        <v>4</v>
-      </c>
-      <c r="F177" s="0" t="s">
-        <v>217</v>
+        <v>8</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B178" s="0" t="s">
         <v>229</v>
-      </c>
-      <c r="B178" s="0" t="s">
-        <v>219</v>
       </c>
       <c r="C178" s="2"/>
       <c r="D178" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="F178" s="0" t="s">
-        <v>220</v>
+        <v>9</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B179" s="0" t="s">
-        <v>43</v>
+        <v>230</v>
       </c>
       <c r="C179" s="2"/>
       <c r="D179" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="E179" s="0" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B180" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C180" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>231</v>
+      </c>
+      <c r="C180" s="2"/>
       <c r="D180" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="F180" s="0" t="s">
-        <v>79</v>
+        <v>11</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B181" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C181" s="2"/>
       <c r="D181" s="0" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B182" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C182" s="2"/>
       <c r="D182" s="0" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B183" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" s="0" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B184" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" s="0" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B185" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" s="0" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B186" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C186" s="2"/>
       <c r="D186" s="0" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A187" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="B187" s="0" t="s">
-        <v>237</v>
-      </c>
-      <c r="C187" s="2"/>
-      <c r="D187" s="0" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A188" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="B188" s="0" t="s">
-        <v>238</v>
-      </c>
-      <c r="C188" s="2"/>
-      <c r="D188" s="0" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A189" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="B189" s="0" t="s">
-        <v>239</v>
-      </c>
-      <c r="C189" s="2"/>
-      <c r="D189" s="0" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A190" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="B190" s="0" t="s">
-        <v>240</v>
-      </c>
-      <c r="C190" s="2"/>
-      <c r="D190" s="0" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4680,7 +4614,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A190" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A186" type="list">
       <formula1>_Lists!$B$2:$B$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4692,7 +4626,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C190" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C186" type="list">
       <formula1>_Lists!$C$2:$C$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4700,7 +4634,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D190" type="whole">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D186" type="whole">
       <formula1>-2000000000</formula1>
       <formula2>2000000000</formula2>
     </dataValidation>
@@ -4716,7 +4650,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G190" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G186" type="list">
       <formula1>_Lists!$D$2:$D$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4728,7 +4662,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" prompt="The only valid values here are no value, &quot;yes&quot; or &quot;no&quot;" promptTitle="Boolean value" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="H2:H190" type="list">
+    <dataValidation allowBlank="true" operator="between" prompt="The only valid values here are no value, &quot;yes&quot; or &quot;no&quot;" promptTitle="Boolean value" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="H2:H186" type="list">
       <formula1>_Lists!$A$2:$A$4</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
PDB-185: Stratigraphic names are now text, and drop-downs.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45694 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="284">
   <si>
     <t xml:space="preserve">testExportMetaTemplate</t>
   </si>
@@ -891,6 +891,9 @@
   </si>
   <si>
     <t xml:space="preserve">DRILL_TYPE_ID$NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t xml:space="preserve">Specify whether a grain-size comparator was used.
@@ -1040,7 +1043,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1051,10 +1054,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -1355,7 +1354,7 @@
       <c r="E6" s="0" t="s">
         <v>44</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="3" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1378,7 +1377,7 @@
       <c r="F7" s="0" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1398,7 +1397,7 @@
       <c r="E8" s="0" t="s">
         <v>51</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="3" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1418,7 +1417,7 @@
       <c r="E9" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1438,7 +1437,7 @@
       <c r="E10" s="0" t="s">
         <v>57</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="3" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1458,7 +1457,7 @@
       <c r="F11" s="0" t="s">
         <v>60</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="I11" s="3" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1478,7 +1477,7 @@
       <c r="E12" s="0" t="s">
         <v>63</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="3" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1498,7 +1497,7 @@
       <c r="F13" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="I13" s="3" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1521,7 +1520,7 @@
       <c r="F14" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="3" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1541,7 +1540,7 @@
       <c r="E15" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I15" s="3" t="s">
         <v>74</v>
       </c>
     </row>
@@ -1561,7 +1560,7 @@
       <c r="F16" s="0" t="s">
         <v>76</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="3" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1581,7 +1580,7 @@
       <c r="F17" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="I17" s="3" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1601,7 +1600,7 @@
       <c r="F18" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="I18" s="3" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1627,7 +1626,7 @@
       <c r="G19" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I19" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1645,7 +1644,7 @@
       <c r="F20" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="I20" s="3" t="s">
         <v>91</v>
       </c>
     </row>
@@ -1665,7 +1664,7 @@
       <c r="F21" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="I21" s="4" t="s">
+      <c r="I21" s="3" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1685,7 +1684,7 @@
       <c r="F22" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="I22" s="4" t="s">
+      <c r="I22" s="3" t="s">
         <v>97</v>
       </c>
     </row>
@@ -1708,7 +1707,7 @@
       <c r="G23" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="I23" s="4" t="s">
+      <c r="I23" s="3" t="s">
         <v>100</v>
       </c>
     </row>
@@ -1728,7 +1727,7 @@
       <c r="F24" s="0" t="s">
         <v>102</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="I24" s="3" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1748,7 +1747,7 @@
       <c r="F25" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="I25" s="4" t="s">
+      <c r="I25" s="3" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1768,7 +1767,7 @@
       <c r="F26" s="0" t="s">
         <v>108</v>
       </c>
-      <c r="I26" s="4" t="s">
+      <c r="I26" s="3" t="s">
         <v>109</v>
       </c>
     </row>
@@ -1785,10 +1784,16 @@
       <c r="D27" s="0" t="n">
         <v>27</v>
       </c>
+      <c r="E27" s="0" t="s">
+        <v>111</v>
+      </c>
       <c r="F27" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="I27" s="4" t="s">
+      <c r="G27" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I27" s="3" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1808,7 +1813,7 @@
       <c r="E28" s="0" t="s">
         <v>114</v>
       </c>
-      <c r="I28" s="4" t="s">
+      <c r="I28" s="3" t="s">
         <v>115</v>
       </c>
     </row>
@@ -1828,7 +1833,7 @@
       <c r="E29" s="0" t="s">
         <v>117</v>
       </c>
-      <c r="I29" s="4" t="s">
+      <c r="I29" s="3" t="s">
         <v>118</v>
       </c>
     </row>
@@ -1848,7 +1853,7 @@
       <c r="E30" s="0" t="s">
         <v>120</v>
       </c>
-      <c r="I30" s="4" t="s">
+      <c r="I30" s="3" t="s">
         <v>121</v>
       </c>
     </row>
@@ -1868,7 +1873,7 @@
       <c r="E31" s="0" t="s">
         <v>123</v>
       </c>
-      <c r="I31" s="4" t="s">
+      <c r="I31" s="3" t="s">
         <v>124</v>
       </c>
     </row>
@@ -1891,7 +1896,7 @@
       <c r="H32" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I32" s="4" t="s">
+      <c r="I32" s="3" t="s">
         <v>127</v>
       </c>
     </row>
@@ -1914,7 +1919,7 @@
       <c r="H33" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I33" s="4" t="s">
+      <c r="I33" s="3" t="s">
         <v>130</v>
       </c>
     </row>
@@ -1937,7 +1942,7 @@
       <c r="H34" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I34" s="4" t="s">
+      <c r="I34" s="3" t="s">
         <v>133</v>
       </c>
     </row>
@@ -1960,7 +1965,7 @@
       <c r="H35" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I35" s="4" t="s">
+      <c r="I35" s="3" t="s">
         <v>136</v>
       </c>
     </row>
@@ -1983,7 +1988,7 @@
       <c r="H36" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I36" s="5" t="s">
+      <c r="I36" s="4" t="s">
         <v>139</v>
       </c>
     </row>
@@ -2006,7 +2011,7 @@
       <c r="H37" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I37" s="4" t="s">
+      <c r="I37" s="3" t="s">
         <v>130</v>
       </c>
     </row>
@@ -2029,7 +2034,7 @@
       <c r="H38" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I38" s="4" t="s">
+      <c r="I38" s="3" t="s">
         <v>133</v>
       </c>
     </row>
@@ -2052,7 +2057,7 @@
       <c r="H39" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I39" s="4" t="s">
+      <c r="I39" s="3" t="s">
         <v>146</v>
       </c>
     </row>
@@ -2081,7 +2086,7 @@
       <c r="H40" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I40" s="4" t="s">
+      <c r="I40" s="3" t="s">
         <v>112</v>
       </c>
     </row>
@@ -2104,7 +2109,7 @@
       <c r="F41" s="0" t="s">
         <v>152</v>
       </c>
-      <c r="I41" s="4" t="s">
+      <c r="I41" s="3" t="s">
         <v>153</v>
       </c>
     </row>
@@ -2124,7 +2129,7 @@
       <c r="F42" s="0" t="s">
         <v>155</v>
       </c>
-      <c r="I42" s="4" t="s">
+      <c r="I42" s="3" t="s">
         <v>156</v>
       </c>
     </row>
@@ -2142,7 +2147,7 @@
       <c r="F43" s="0" t="s">
         <v>158</v>
       </c>
-      <c r="I43" s="4" t="s">
+      <c r="I43" s="3" t="s">
         <v>159</v>
       </c>
     </row>
@@ -2160,7 +2165,7 @@
       <c r="F44" s="0" t="s">
         <v>161</v>
       </c>
-      <c r="I44" s="4" t="s">
+      <c r="I44" s="3" t="s">
         <v>162</v>
       </c>
     </row>
@@ -2178,7 +2183,7 @@
       <c r="F45" s="0" t="s">
         <v>164</v>
       </c>
-      <c r="I45" s="4" t="s">
+      <c r="I45" s="3" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2198,7 +2203,7 @@
       <c r="F46" s="0" t="s">
         <v>167</v>
       </c>
-      <c r="I46" s="4" t="s">
+      <c r="I46" s="3" t="s">
         <v>168</v>
       </c>
     </row>
@@ -2218,7 +2223,7 @@
       <c r="F47" s="0" t="s">
         <v>170</v>
       </c>
-      <c r="I47" s="4" t="s">
+      <c r="I47" s="3" t="s">
         <v>171</v>
       </c>
     </row>
@@ -2238,7 +2243,7 @@
       <c r="F48" s="0" t="s">
         <v>173</v>
       </c>
-      <c r="I48" s="4" t="s">
+      <c r="I48" s="3" t="s">
         <v>174</v>
       </c>
     </row>
@@ -2259,7 +2264,7 @@
       <c r="F49" s="0" t="s">
         <v>176</v>
       </c>
-      <c r="I49" s="4" t="s">
+      <c r="I49" s="3" t="s">
         <v>177</v>
       </c>
     </row>
@@ -2279,7 +2284,7 @@
       <c r="F50" s="0" t="s">
         <v>179</v>
       </c>
-      <c r="I50" s="4" t="s">
+      <c r="I50" s="3" t="s">
         <v>180</v>
       </c>
     </row>
@@ -2299,7 +2304,7 @@
       <c r="F51" s="0" t="s">
         <v>182</v>
       </c>
-      <c r="I51" s="4" t="s">
+      <c r="I51" s="3" t="s">
         <v>183</v>
       </c>
     </row>
@@ -2319,7 +2324,7 @@
       <c r="F52" s="0" t="s">
         <v>185</v>
       </c>
-      <c r="I52" s="4" t="s">
+      <c r="I52" s="3" t="s">
         <v>186</v>
       </c>
     </row>
@@ -2339,7 +2344,7 @@
       <c r="F53" s="0" t="s">
         <v>188</v>
       </c>
-      <c r="I53" s="4" t="s">
+      <c r="I53" s="3" t="s">
         <v>189</v>
       </c>
     </row>
@@ -2359,7 +2364,7 @@
       <c r="F54" s="0" t="s">
         <v>191</v>
       </c>
-      <c r="I54" s="4" t="s">
+      <c r="I54" s="3" t="s">
         <v>192</v>
       </c>
     </row>
@@ -2379,7 +2384,7 @@
       <c r="F55" s="0" t="s">
         <v>194</v>
       </c>
-      <c r="I55" s="4" t="s">
+      <c r="I55" s="3" t="s">
         <v>195</v>
       </c>
     </row>
@@ -2399,7 +2404,7 @@
       <c r="F56" s="0" t="s">
         <v>197</v>
       </c>
-      <c r="I56" s="4" t="s">
+      <c r="I56" s="3" t="s">
         <v>198</v>
       </c>
     </row>
@@ -2419,7 +2424,7 @@
       <c r="F57" s="0" t="s">
         <v>200</v>
       </c>
-      <c r="I57" s="4" t="s">
+      <c r="I57" s="3" t="s">
         <v>201</v>
       </c>
     </row>
@@ -2439,7 +2444,7 @@
       <c r="F58" s="0" t="s">
         <v>203</v>
       </c>
-      <c r="I58" s="4" t="s">
+      <c r="I58" s="3" t="s">
         <v>204</v>
       </c>
     </row>
@@ -2457,7 +2462,7 @@
       <c r="F59" s="0" t="s">
         <v>206</v>
       </c>
-      <c r="I59" s="4" t="s">
+      <c r="I59" s="3" t="s">
         <v>207</v>
       </c>
     </row>
@@ -2477,7 +2482,7 @@
       <c r="F60" s="0" t="s">
         <v>209</v>
       </c>
-      <c r="I60" s="4" t="s">
+      <c r="I60" s="3" t="s">
         <v>210</v>
       </c>
     </row>
@@ -2503,7 +2508,7 @@
       <c r="G61" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="I61" s="4" t="s">
+      <c r="I61" s="3" t="s">
         <v>214</v>
       </c>
     </row>
@@ -2523,7 +2528,7 @@
       <c r="F62" s="0" t="s">
         <v>216</v>
       </c>
-      <c r="I62" s="4" t="s">
+      <c r="I62" s="3" t="s">
         <v>217</v>
       </c>
     </row>
@@ -2543,7 +2548,7 @@
       <c r="F63" s="0" t="s">
         <v>219</v>
       </c>
-      <c r="I63" s="4" t="s">
+      <c r="I63" s="3" t="s">
         <v>220</v>
       </c>
     </row>
@@ -2563,7 +2568,7 @@
       <c r="E64" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="I64" s="4" t="s">
+      <c r="I64" s="3" t="s">
         <v>222</v>
       </c>
     </row>
@@ -2885,9 +2890,15 @@
       <c r="D80" s="0" t="n">
         <v>17</v>
       </c>
+      <c r="E80" s="0" t="s">
+        <v>111</v>
+      </c>
       <c r="F80" s="0" t="s">
         <v>111</v>
       </c>
+      <c r="G80" s="0" t="s">
+        <v>12</v>
+      </c>
       <c r="I80" s="0" t="s">
         <v>244</v>
       </c>
@@ -3014,7 +3025,7 @@
       <c r="H86" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I86" s="4" t="s">
+      <c r="I86" s="3" t="s">
         <v>130</v>
       </c>
     </row>
@@ -3106,7 +3117,7 @@
       <c r="H90" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I90" s="4" t="s">
+      <c r="I90" s="3" t="s">
         <v>130</v>
       </c>
     </row>
@@ -3639,7 +3650,7 @@
       <c r="E118" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="I118" s="4" t="s">
+      <c r="I118" s="3" t="s">
         <v>267</v>
       </c>
     </row>
@@ -3657,7 +3668,7 @@
       <c r="F119" s="0" t="s">
         <v>227</v>
       </c>
-      <c r="I119" s="5" t="s">
+      <c r="I119" s="4" t="s">
         <v>225</v>
       </c>
     </row>
@@ -3675,7 +3686,7 @@
       <c r="F120" s="0" t="s">
         <v>230</v>
       </c>
-      <c r="I120" s="5" t="s">
+      <c r="I120" s="4" t="s">
         <v>228</v>
       </c>
     </row>
@@ -3693,7 +3704,7 @@
       <c r="F121" s="0" t="s">
         <v>233</v>
       </c>
-      <c r="I121" s="5" t="s">
+      <c r="I121" s="4" t="s">
         <v>231</v>
       </c>
     </row>
@@ -3711,7 +3722,7 @@
       <c r="F122" s="0" t="s">
         <v>269</v>
       </c>
-      <c r="I122" s="5" t="s">
+      <c r="I122" s="4" t="s">
         <v>234</v>
       </c>
     </row>
@@ -3731,7 +3742,7 @@
       <c r="F123" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="I123" s="5" t="s">
+      <c r="I123" s="4" t="s">
         <v>235</v>
       </c>
     </row>
@@ -3749,7 +3760,7 @@
       <c r="F124" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="I124" s="5" t="s">
+      <c r="I124" s="4" t="s">
         <v>236</v>
       </c>
     </row>
@@ -3773,7 +3784,7 @@
       <c r="G125" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="I125" s="5" t="s">
+      <c r="I125" s="4" t="s">
         <v>237</v>
       </c>
     </row>
@@ -3791,7 +3802,7 @@
       <c r="F126" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="I126" s="5"/>
+      <c r="I126" s="4"/>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="2" t="s">
@@ -3809,7 +3820,7 @@
       <c r="F127" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="I127" s="5" t="s">
+      <c r="I127" s="4" t="s">
         <v>239</v>
       </c>
     </row>
@@ -3829,7 +3840,7 @@
       <c r="F128" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="I128" s="5" t="s">
+      <c r="I128" s="4" t="s">
         <v>240</v>
       </c>
     </row>
@@ -3852,7 +3863,7 @@
       <c r="G129" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="I129" s="5" t="s">
+      <c r="I129" s="4" t="s">
         <v>241</v>
       </c>
     </row>
@@ -3872,7 +3883,7 @@
       <c r="F130" s="0" t="s">
         <v>102</v>
       </c>
-      <c r="I130" s="5" t="s">
+      <c r="I130" s="4" t="s">
         <v>242</v>
       </c>
     </row>
@@ -3892,7 +3903,7 @@
       <c r="F131" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="I131" s="5"/>
+      <c r="I131" s="4"/>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="2" t="s">
@@ -3910,7 +3921,7 @@
       <c r="F132" s="0" t="s">
         <v>108</v>
       </c>
-      <c r="I132" s="5" t="s">
+      <c r="I132" s="4" t="s">
         <v>243</v>
       </c>
     </row>
@@ -3927,10 +3938,16 @@
       <c r="D133" s="0" t="n">
         <v>17</v>
       </c>
+      <c r="E133" s="0" t="s">
+        <v>111</v>
+      </c>
       <c r="F133" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="I133" s="5" t="s">
+      <c r="G133" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I133" s="4" t="s">
         <v>244</v>
       </c>
     </row>
@@ -3948,9 +3965,9 @@
         <v>18</v>
       </c>
       <c r="E134" s="0" t="s">
-        <v>114</v>
-      </c>
-      <c r="I134" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="I134" s="3" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3970,7 +3987,7 @@
       <c r="E135" s="0" t="s">
         <v>117</v>
       </c>
-      <c r="I135" s="4" t="s">
+      <c r="I135" s="3" t="s">
         <v>118</v>
       </c>
     </row>
@@ -3990,7 +4007,7 @@
       <c r="E136" s="0" t="s">
         <v>120</v>
       </c>
-      <c r="I136" s="4" t="s">
+      <c r="I136" s="3" t="s">
         <v>121</v>
       </c>
     </row>
@@ -4010,7 +4027,7 @@
       <c r="E137" s="0" t="s">
         <v>123</v>
       </c>
-      <c r="I137" s="4" t="s">
+      <c r="I137" s="3" t="s">
         <v>124</v>
       </c>
     </row>
@@ -4033,7 +4050,7 @@
       <c r="H138" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I138" s="5" t="s">
+      <c r="I138" s="4" t="s">
         <v>249</v>
       </c>
     </row>
@@ -4056,7 +4073,7 @@
       <c r="H139" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I139" s="4" t="s">
+      <c r="I139" s="3" t="s">
         <v>130</v>
       </c>
     </row>
@@ -4079,7 +4096,7 @@
       <c r="H140" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I140" s="5" t="s">
+      <c r="I140" s="4" t="s">
         <v>250</v>
       </c>
     </row>
@@ -4102,7 +4119,7 @@
       <c r="H141" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I141" s="5" t="s">
+      <c r="I141" s="4" t="s">
         <v>251</v>
       </c>
     </row>
@@ -4125,7 +4142,7 @@
       <c r="H142" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I142" s="5" t="s">
+      <c r="I142" s="4" t="s">
         <v>252</v>
       </c>
     </row>
@@ -4148,7 +4165,7 @@
       <c r="H143" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I143" s="4" t="s">
+      <c r="I143" s="3" t="s">
         <v>130</v>
       </c>
     </row>
@@ -4171,7 +4188,7 @@
       <c r="H144" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I144" s="5" t="s">
+      <c r="I144" s="4" t="s">
         <v>253</v>
       </c>
     </row>
@@ -4194,7 +4211,7 @@
       <c r="H145" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I145" s="5" t="s">
+      <c r="I145" s="4" t="s">
         <v>254</v>
       </c>
     </row>
@@ -4223,7 +4240,7 @@
       <c r="H146" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I146" s="5" t="s">
+      <c r="I146" s="4" t="s">
         <v>255</v>
       </c>
     </row>
@@ -4246,7 +4263,7 @@
       <c r="F147" s="0" t="s">
         <v>152</v>
       </c>
-      <c r="I147" s="5" t="s">
+      <c r="I147" s="4" t="s">
         <v>256</v>
       </c>
     </row>
@@ -4266,7 +4283,7 @@
       <c r="F148" s="0" t="s">
         <v>155</v>
       </c>
-      <c r="I148" s="4" t="s">
+      <c r="I148" s="3" t="s">
         <v>156</v>
       </c>
     </row>
@@ -4284,7 +4301,7 @@
       <c r="F149" s="0" t="s">
         <v>158</v>
       </c>
-      <c r="I149" s="4" t="s">
+      <c r="I149" s="3" t="s">
         <v>159</v>
       </c>
     </row>
@@ -4304,7 +4321,7 @@
       <c r="F150" s="0" t="s">
         <v>161</v>
       </c>
-      <c r="I150" s="4" t="s">
+      <c r="I150" s="3" t="s">
         <v>162</v>
       </c>
     </row>
@@ -4322,7 +4339,7 @@
       <c r="F151" s="0" t="s">
         <v>164</v>
       </c>
-      <c r="I151" s="4" t="s">
+      <c r="I151" s="3" t="s">
         <v>165</v>
       </c>
     </row>
@@ -4342,7 +4359,7 @@
       <c r="F152" s="0" t="s">
         <v>167</v>
       </c>
-      <c r="I152" s="4" t="s">
+      <c r="I152" s="3" t="s">
         <v>168</v>
       </c>
     </row>
@@ -4362,7 +4379,7 @@
       <c r="F153" s="0" t="s">
         <v>170</v>
       </c>
-      <c r="I153" s="4" t="s">
+      <c r="I153" s="3" t="s">
         <v>171</v>
       </c>
     </row>
@@ -4380,7 +4397,7 @@
       <c r="F154" s="0" t="s">
         <v>173</v>
       </c>
-      <c r="I154" s="4" t="s">
+      <c r="I154" s="3" t="s">
         <v>174</v>
       </c>
     </row>
@@ -4401,8 +4418,8 @@
       <c r="F155" s="0" t="s">
         <v>176</v>
       </c>
-      <c r="I155" s="4" t="s">
-        <v>270</v>
+      <c r="I155" s="3" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4658,7 +4675,7 @@
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B170" s="0" t="s">
         <v>31</v>
@@ -4673,10 +4690,10 @@
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B171" s="0" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C171" s="2"/>
       <c r="D171" s="0" t="n">
@@ -4685,7 +4702,7 @@
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B172" s="0" t="s">
         <v>226</v>
@@ -4700,7 +4717,7 @@
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B173" s="0" t="s">
         <v>229</v>
@@ -4715,7 +4732,7 @@
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B174" s="0" t="s">
         <v>232</v>
@@ -4730,7 +4747,7 @@
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B175" s="0" t="s">
         <v>43</v>
@@ -4745,7 +4762,7 @@
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B176" s="0" t="s">
         <v>78</v>
@@ -4762,10 +4779,10 @@
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B177" s="0" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C177" s="2"/>
       <c r="D177" s="0" t="n">
@@ -4774,10 +4791,10 @@
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B178" s="0" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C178" s="2"/>
       <c r="D178" s="0" t="n">
@@ -4786,10 +4803,10 @@
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B179" s="0" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C179" s="2"/>
       <c r="D179" s="0" t="n">
@@ -4798,10 +4815,10 @@
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B180" s="0" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C180" s="2"/>
       <c r="D180" s="0" t="n">
@@ -4810,10 +4827,10 @@
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B181" s="0" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C181" s="2"/>
       <c r="D181" s="0" t="n">
@@ -4822,10 +4839,10 @@
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B182" s="0" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C182" s="2"/>
       <c r="D182" s="0" t="n">
@@ -4834,10 +4851,10 @@
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B183" s="0" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" s="0" t="n">
@@ -4846,10 +4863,10 @@
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B184" s="0" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" s="0" t="n">
@@ -4858,10 +4875,10 @@
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B185" s="0" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" s="0" t="n">
@@ -4870,10 +4887,10 @@
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B186" s="0" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C186" s="2"/>
       <c r="D186" s="0" t="n">

</xml_diff>

<commit_message>
Add abundant tag. PDB-215. Also make sure stuff gets imported into SEDIMENTARY_FEATURE. It wasn't before.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@45702 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="939" uniqueCount="289">
   <si>
     <t xml:space="preserve">testExportMetaTemplate</t>
   </si>
@@ -704,11 +704,26 @@
     <t xml:space="preserve">Additional Features</t>
   </si>
   <si>
+    <t xml:space="preserve">ADDITIONAL_FEATURES</t>
+  </si>
+  <si>
     <t xml:space="preserve">#SEDIMENTARY_FEATURE$SED_FEATURE_ID$NAME</t>
   </si>
   <si>
     <t xml:space="preserve">Enter any other comments about the lithology.
 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Additional Features – Abundant?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABUNDANT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SEDIMENTARY_FEATURE$ABUNDANT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whether the lithology is abundant</t>
   </si>
   <si>
     <t xml:space="preserve">Inferred Environment</t>
@@ -1218,7 +1233,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I186"/>
+  <dimension ref="A1:I189"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -2479,37 +2494,37 @@
       <c r="D60" s="0" t="n">
         <v>60</v>
       </c>
+      <c r="E60" s="0" t="s">
+        <v>209</v>
+      </c>
       <c r="F60" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D61" s="0" t="n">
         <v>61</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>213</v>
-      </c>
-      <c r="G61" s="0" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2517,19 +2532,25 @@
         <v>30</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D62" s="0" t="n">
-        <v>63</v>
+        <v>62</v>
+      </c>
+      <c r="E62" s="0" t="s">
+        <v>217</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>216</v>
+        <v>218</v>
+      </c>
+      <c r="G62" s="0" t="s">
+        <v>12</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2537,2363 +2558,2429 @@
         <v>30</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D63" s="0" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>221</v>
+        <v>30</v>
       </c>
       <c r="B64" s="0" t="s">
+        <v>223</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D64" s="0" t="n">
+        <v>64</v>
+      </c>
+      <c r="F64" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="I64" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B65" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="C64" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D64" s="0" t="n">
+      <c r="C65" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D65" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="E64" s="0" t="s">
+      <c r="E65" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="I64" s="3" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="B65" s="0" t="s">
-        <v>223</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D65" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E65" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="I65" s="0" t="s">
-        <v>224</v>
+      <c r="I65" s="3" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>43</v>
+        <v>228</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D66" s="0" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="I66" s="0" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>226</v>
-      </c>
-      <c r="C67" s="2"/>
+        <v>43</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D67" s="0" t="n">
-        <v>4</v>
-      </c>
-      <c r="F67" s="0" t="s">
-        <v>227</v>
+        <v>3</v>
+      </c>
+      <c r="E67" s="0" t="s">
+        <v>44</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" s="0" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="I68" s="0" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B69" s="0" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" s="0" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I69" s="0" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B70" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>237</v>
+      </c>
+      <c r="C70" s="2"/>
       <c r="D70" s="0" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F70" s="0" t="s">
-        <v>79</v>
+        <v>238</v>
       </c>
       <c r="I70" s="0" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B71" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="C71" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D71" s="0" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F71" s="0" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I71" s="0" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B72" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="C72" s="2"/>
       <c r="D72" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E72" s="0" t="s">
-        <v>85</v>
+        <v>8</v>
       </c>
       <c r="F72" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="G72" s="0" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="I72" s="0" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B73" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="C73" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D73" s="0" t="n">
-        <v>10</v>
+        <v>9</v>
+      </c>
+      <c r="E73" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="F73" s="0" t="s">
-        <v>90</v>
+        <v>86</v>
+      </c>
+      <c r="G73" s="0" t="s">
+        <v>87</v>
       </c>
       <c r="I73" s="0" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B74" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="C74" s="2"/>
       <c r="D74" s="0" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F74" s="0" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I74" s="0" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D75" s="0" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F75" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="G75" s="0" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="I75" s="0" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D76" s="0" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F76" s="0" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G76" s="0" t="s">
         <v>87</v>
       </c>
       <c r="I76" s="0" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B77" s="0" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D77" s="0" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F77" s="0" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G77" s="0" t="s">
         <v>87</v>
       </c>
       <c r="I77" s="0" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B78" s="0" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D78" s="0" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F78" s="0" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G78" s="0" t="s">
         <v>87</v>
       </c>
+      <c r="I78" s="0" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B79" s="0" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D79" s="0" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F79" s="0" t="s">
-        <v>108</v>
-      </c>
-      <c r="I79" s="0" t="s">
-        <v>243</v>
+        <v>105</v>
+      </c>
+      <c r="G79" s="0" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B80" s="0" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D80" s="0" t="n">
-        <v>17</v>
-      </c>
-      <c r="E80" s="0" t="s">
-        <v>111</v>
+        <v>16</v>
       </c>
       <c r="F80" s="0" t="s">
-        <v>111</v>
-      </c>
-      <c r="G80" s="0" t="s">
-        <v>12</v>
+        <v>108</v>
       </c>
       <c r="I80" s="0" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B81" s="0" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D81" s="0" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E81" s="0" t="s">
-        <v>114</v>
+        <v>111</v>
+      </c>
+      <c r="F81" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="G81" s="0" t="s">
+        <v>12</v>
       </c>
       <c r="I81" s="0" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B82" s="0" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D82" s="0" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E82" s="0" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I82" s="0" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B83" s="0" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D83" s="0" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E83" s="0" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="I83" s="0" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B84" s="0" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D84" s="0" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E84" s="0" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I84" s="0" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B85" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D85" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="E85" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="I85" s="0" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B86" s="0" t="s">
         <v>125</v>
       </c>
-      <c r="C85" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D85" s="0" t="n">
+      <c r="C86" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D86" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="E85" s="0" t="s">
+      <c r="E86" s="0" t="s">
         <v>126</v>
-      </c>
-      <c r="H85" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="I85" s="0" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="B86" s="0" t="s">
-        <v>128</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D86" s="0" t="n">
-        <v>23</v>
-      </c>
-      <c r="E86" s="0" t="s">
-        <v>129</v>
       </c>
       <c r="H86" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I86" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I86" s="0" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B87" s="0" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D87" s="0" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E87" s="0" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="H87" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I87" s="0" t="s">
-        <v>250</v>
+      <c r="I87" s="3" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D88" s="0" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E88" s="0" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="H88" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I88" s="0" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B89" s="0" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D89" s="0" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E89" s="0" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H89" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I89" s="0" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B90" s="0" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D90" s="0" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E90" s="0" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="H90" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I90" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I90" s="0" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B91" s="0" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D91" s="0" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E91" s="0" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H91" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I91" s="0" t="s">
-        <v>253</v>
+      <c r="I91" s="3" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D92" s="0" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H92" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I92" s="0" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C93" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D93" s="0" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E93" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="F93" s="0" t="s">
-        <v>149</v>
-      </c>
-      <c r="G93" s="0" t="s">
-        <v>87</v>
+        <v>145</v>
       </c>
       <c r="H93" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I93" s="0" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="C94" s="2"/>
+        <v>147</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D94" s="0" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E94" s="0" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F94" s="0" t="s">
-        <v>152</v>
+        <v>149</v>
+      </c>
+      <c r="G94" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="H94" s="0" t="s">
+        <v>5</v>
       </c>
       <c r="I94" s="0" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="C95" s="2"/>
       <c r="D95" s="0" t="n">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="E95" s="0" t="s">
+        <v>151</v>
       </c>
       <c r="F95" s="0" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="I95" s="0" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B96" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="C96" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D96" s="0" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F96" s="0" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I96" s="0" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B97" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="C97" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="C97" s="2"/>
       <c r="D97" s="0" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F97" s="0" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="I97" s="0" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="C98" s="2"/>
+        <v>160</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D98" s="0" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F98" s="0" t="s">
-        <v>164</v>
+        <v>161</v>
+      </c>
+      <c r="I98" s="0" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B99" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="C99" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="C99" s="2"/>
       <c r="D99" s="0" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F99" s="0" t="s">
-        <v>167</v>
-      </c>
-      <c r="I99" s="0" t="s">
-        <v>260</v>
+        <v>164</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B100" s="0" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D100" s="0" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F100" s="0" t="s">
-        <v>170</v>
+        <v>167</v>
+      </c>
+      <c r="I100" s="0" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B101" s="0" t="s">
-        <v>172</v>
-      </c>
-      <c r="C101" s="2"/>
+        <v>169</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D101" s="0" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F101" s="0" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B102" s="0" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" s="0" t="n">
-        <v>39</v>
-      </c>
-      <c r="E102" s="0" t="s">
-        <v>176</v>
+        <v>38</v>
       </c>
       <c r="F102" s="0" t="s">
-        <v>176</v>
-      </c>
-      <c r="I102" s="0" t="s">
-        <v>261</v>
+        <v>173</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B103" s="0" t="s">
-        <v>178</v>
-      </c>
-      <c r="C103" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>175</v>
+      </c>
+      <c r="C103" s="2"/>
       <c r="D103" s="0" t="n">
-        <v>40</v>
+        <v>39</v>
+      </c>
+      <c r="E103" s="0" t="s">
+        <v>176</v>
       </c>
       <c r="F103" s="0" t="s">
-        <v>179</v>
+        <v>176</v>
+      </c>
+      <c r="I103" s="0" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B104" s="0" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C104" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D104" s="0" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F104" s="0" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B105" s="0" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C105" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D105" s="0" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F105" s="0" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B106" s="0" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C106" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D106" s="0" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F106" s="0" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B107" s="0" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C107" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D107" s="0" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F107" s="0" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C108" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D108" s="0" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F108" s="0" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B109" s="0" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C109" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D109" s="0" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F109" s="0" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B110" s="0" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C110" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D110" s="0" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F110" s="0" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B111" s="0" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C111" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D111" s="0" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F111" s="0" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B112" s="0" t="s">
-        <v>205</v>
-      </c>
-      <c r="C112" s="2"/>
+        <v>202</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D112" s="0" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F112" s="0" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B113" s="0" t="s">
-        <v>208</v>
-      </c>
-      <c r="C113" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="C113" s="2"/>
       <c r="D113" s="0" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F113" s="0" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B114" s="0" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D114" s="0" t="n">
-        <v>51</v>
-      </c>
-      <c r="E114" s="0" t="s">
-        <v>212</v>
+        <v>50</v>
       </c>
       <c r="F114" s="0" t="s">
-        <v>213</v>
-      </c>
-      <c r="G114" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="I114" s="0" t="s">
-        <v>262</v>
+        <v>210</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B115" s="0" t="s">
+        <v>212</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D115" s="0" t="n">
+        <v>51</v>
+      </c>
+      <c r="E115" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="F115" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="I115" s="0" t="s">
         <v>215</v>
-      </c>
-      <c r="C115" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D115" s="0" t="n">
-        <v>53</v>
-      </c>
-      <c r="F115" s="0" t="s">
-        <v>216</v>
-      </c>
-      <c r="I115" s="0" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B116" s="0" t="s">
+        <v>216</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D116" s="0" t="n">
+        <v>52</v>
+      </c>
+      <c r="E116" s="0" t="s">
+        <v>217</v>
+      </c>
+      <c r="F116" s="0" t="s">
+        <v>218</v>
+      </c>
+      <c r="G116" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I116" s="0" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B117" s="0" t="s">
+        <v>220</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D117" s="0" t="n">
+        <v>53</v>
+      </c>
+      <c r="F117" s="0" t="s">
         <v>221</v>
       </c>
-      <c r="B116" s="0" t="s">
-        <v>218</v>
-      </c>
-      <c r="C116" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D116" s="0" t="n">
+      <c r="I117" s="0" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B118" s="0" t="s">
+        <v>223</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D118" s="0" t="n">
         <v>54</v>
       </c>
-      <c r="F116" s="0" t="s">
-        <v>219</v>
-      </c>
-      <c r="I116" s="0" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="117" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="B117" s="0" t="s">
+      <c r="F118" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="I118" s="0" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B119" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="C117" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D117" s="0" t="n">
+      <c r="C119" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D119" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="E117" s="0" t="s">
+      <c r="E119" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="I117" s="3" t="s">
+      <c r="I119" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="B118" s="0" t="s">
-        <v>266</v>
-      </c>
-      <c r="C118" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D118" s="0" t="n">
+    <row r="120" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B120" s="0" t="s">
+        <v>271</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D120" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="E118" s="0" t="s">
+      <c r="E120" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="I118" s="3" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="B119" s="0" t="s">
-        <v>226</v>
-      </c>
-      <c r="C119" s="2"/>
-      <c r="D119" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="F119" s="0" t="s">
-        <v>227</v>
-      </c>
-      <c r="I119" s="4" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="B120" s="0" t="s">
-        <v>229</v>
-      </c>
-      <c r="C120" s="2"/>
-      <c r="D120" s="0" t="n">
-        <v>4</v>
-      </c>
-      <c r="F120" s="0" t="s">
-        <v>230</v>
-      </c>
-      <c r="I120" s="4" t="s">
-        <v>228</v>
+      <c r="I120" s="3" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" s="0" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F121" s="0" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="I121" s="4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>268</v>
+        <v>234</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" s="0" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F122" s="0" t="s">
-        <v>269</v>
+        <v>235</v>
       </c>
       <c r="I122" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C123" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>237</v>
+      </c>
+      <c r="C123" s="2"/>
       <c r="D123" s="0" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F123" s="0" t="s">
-        <v>79</v>
+        <v>238</v>
       </c>
       <c r="I123" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B124" s="0" t="s">
-        <v>81</v>
+        <v>273</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" s="0" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F124" s="0" t="s">
-        <v>82</v>
+        <v>274</v>
       </c>
       <c r="I124" s="4" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="125" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B125" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="C125" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D125" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E125" s="0" t="s">
-        <v>85</v>
+        <v>7</v>
       </c>
       <c r="F125" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="G125" s="0" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="I125" s="4" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" s="0" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F126" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="I126" s="4"/>
-    </row>
-    <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>82</v>
+      </c>
+      <c r="I126" s="4" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="C127" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="C127" s="2"/>
       <c r="D127" s="0" t="n">
-        <v>11</v>
+        <v>9</v>
+      </c>
+      <c r="E127" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="F127" s="0" t="s">
-        <v>93</v>
+        <v>86</v>
+      </c>
+      <c r="G127" s="0" t="s">
+        <v>87</v>
       </c>
       <c r="I127" s="4" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="C128" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="C128" s="2"/>
       <c r="D128" s="0" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F128" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="I128" s="4" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="129" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>90</v>
+      </c>
+      <c r="I128" s="4"/>
+    </row>
+    <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D129" s="0" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F129" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="G129" s="0" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="I129" s="4" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B130" s="0" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C130" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D130" s="0" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F130" s="0" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="I130" s="4" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B131" s="0" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D131" s="0" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F131" s="0" t="s">
-        <v>105</v>
-      </c>
-      <c r="I131" s="4"/>
+        <v>99</v>
+      </c>
+      <c r="G131" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="I131" s="4" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B132" s="0" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D132" s="0" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F132" s="0" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="I132" s="4" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B133" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D133" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="F133" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="I133" s="4"/>
+    </row>
+    <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B134" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D134" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="F134" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="I134" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B135" s="0" t="s">
         <v>110</v>
       </c>
-      <c r="C133" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D133" s="0" t="n">
-        <v>17</v>
-      </c>
-      <c r="E133" s="0" t="s">
+      <c r="C135" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D135" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="E135" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="F133" s="0" t="s">
+      <c r="F135" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="G133" s="0" t="s">
+      <c r="G135" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="I133" s="4" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="134" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A134" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="B134" s="0" t="s">
-        <v>113</v>
-      </c>
-      <c r="C134" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D134" s="0" t="n">
-        <v>18</v>
-      </c>
-      <c r="E134" s="0" t="s">
-        <v>270</v>
-      </c>
-      <c r="I134" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="135" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A135" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="B135" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="C135" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D135" s="0" t="n">
-        <v>19</v>
-      </c>
-      <c r="E135" s="0" t="s">
-        <v>117</v>
-      </c>
-      <c r="I135" s="3" t="s">
-        <v>118</v>
+      <c r="I135" s="4" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B136" s="0" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C136" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D136" s="0" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E136" s="0" t="s">
-        <v>120</v>
+        <v>275</v>
       </c>
       <c r="I136" s="3" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B137" s="0" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="C137" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D137" s="0" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E137" s="0" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="I137" s="3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="138" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B138" s="0" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D138" s="0" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E138" s="0" t="s">
-        <v>126</v>
-      </c>
-      <c r="H138" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="I138" s="4" t="s">
-        <v>249</v>
+        <v>120</v>
+      </c>
+      <c r="I138" s="3" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B139" s="0" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="C139" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D139" s="0" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E139" s="0" t="s">
-        <v>129</v>
-      </c>
-      <c r="H139" s="0" t="s">
-        <v>5</v>
+        <v>123</v>
       </c>
       <c r="I139" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="140" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B140" s="0" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C140" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D140" s="0" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E140" s="0" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="H140" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I140" s="4" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B141" s="0" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C141" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D141" s="0" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E141" s="0" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="H141" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I141" s="4" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I141" s="3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B142" s="0" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C142" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D142" s="0" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E142" s="0" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H142" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I142" s="4" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B143" s="0" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C143" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D143" s="0" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E143" s="0" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="H143" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I143" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="144" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I143" s="4" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B144" s="0" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C144" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D144" s="0" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E144" s="0" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="H144" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I144" s="4" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B145" s="0" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C145" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D145" s="0" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E145" s="0" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="H145" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="I145" s="4" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I145" s="3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B146" s="0" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D146" s="0" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E146" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="F146" s="0" t="s">
-        <v>149</v>
-      </c>
-      <c r="G146" s="0" t="s">
-        <v>87</v>
+        <v>143</v>
       </c>
       <c r="H146" s="0" t="s">
         <v>5</v>
       </c>
       <c r="I146" s="4" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="147" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B147" s="0" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D147" s="0" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E147" s="0" t="s">
-        <v>151</v>
-      </c>
-      <c r="F147" s="0" t="s">
-        <v>152</v>
+        <v>145</v>
+      </c>
+      <c r="H147" s="0" t="s">
+        <v>5</v>
       </c>
       <c r="I147" s="4" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="148" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B148" s="0" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D148" s="0" t="n">
-        <v>32</v>
+        <v>30</v>
+      </c>
+      <c r="E148" s="0" t="s">
+        <v>148</v>
       </c>
       <c r="F148" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="I148" s="3" t="s">
-        <v>156</v>
+        <v>149</v>
+      </c>
+      <c r="G148" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="H148" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="I148" s="4" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B149" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="C149" s="2"/>
+        <v>150</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D149" s="0" t="n">
-        <v>33</v>
+        <v>31</v>
+      </c>
+      <c r="E149" s="0" t="s">
+        <v>151</v>
       </c>
       <c r="F149" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="I149" s="3" t="s">
-        <v>159</v>
+        <v>152</v>
+      </c>
+      <c r="I149" s="4" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B150" s="0" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C150" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D150" s="0" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F150" s="0" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="I150" s="3" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B151" s="0" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="C151" s="2"/>
       <c r="D151" s="0" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F151" s="0" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="I151" s="3" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B152" s="0" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D152" s="0" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F152" s="0" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="I152" s="3" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B153" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="C153" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="C153" s="2"/>
       <c r="D153" s="0" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F153" s="0" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="I153" s="3" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B154" s="0" t="s">
-        <v>172</v>
-      </c>
-      <c r="C154" s="2"/>
+        <v>166</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D154" s="0" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F154" s="0" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="I154" s="3" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B155" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D155" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="F155" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="I155" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B156" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="C156" s="2"/>
+      <c r="D156" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="F156" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="I156" s="3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="23.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B157" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="C155" s="2"/>
-      <c r="D155" s="0" t="n">
+      <c r="C157" s="2"/>
+      <c r="D157" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="E155" s="0" t="s">
+      <c r="E157" s="0" t="s">
         <v>176</v>
       </c>
-      <c r="F155" s="0" t="s">
+      <c r="F157" s="0" t="s">
         <v>176</v>
       </c>
-      <c r="I155" s="3" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A156" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="B156" s="0" t="s">
-        <v>178</v>
-      </c>
-      <c r="C156" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D156" s="0" t="n">
-        <v>40</v>
-      </c>
-      <c r="F156" s="0" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A157" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="B157" s="0" t="s">
-        <v>181</v>
-      </c>
-      <c r="C157" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D157" s="0" t="n">
-        <v>41</v>
-      </c>
-      <c r="F157" s="0" t="s">
-        <v>182</v>
+      <c r="I157" s="3" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B158" s="0" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C158" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D158" s="0" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F158" s="0" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B159" s="0" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="C159" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D159" s="0" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F159" s="0" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B160" s="0" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C160" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D160" s="0" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F160" s="0" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B161" s="0" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C161" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D161" s="0" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F161" s="0" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B162" s="0" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="C162" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D162" s="0" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F162" s="0" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B163" s="0" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="C163" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D163" s="0" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F163" s="0" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B164" s="0" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="C164" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D164" s="0" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F164" s="0" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B165" s="0" t="s">
-        <v>205</v>
-      </c>
-      <c r="C165" s="2"/>
+        <v>199</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D165" s="0" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F165" s="0" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B166" s="0" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="C166" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D166" s="0" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F166" s="0" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B167" s="0" t="s">
-        <v>211</v>
-      </c>
-      <c r="C167" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="C167" s="2"/>
       <c r="D167" s="0" t="n">
-        <v>51</v>
-      </c>
-      <c r="E167" s="0" t="s">
-        <v>212</v>
+        <v>49</v>
       </c>
       <c r="F167" s="0" t="s">
-        <v>213</v>
-      </c>
-      <c r="G167" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="I167" s="0" t="s">
-        <v>262</v>
+        <v>206</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B168" s="0" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D168" s="0" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F168" s="0" t="s">
-        <v>216</v>
-      </c>
-      <c r="I168" s="0" t="s">
-        <v>263</v>
+        <v>210</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B169" s="0" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D169" s="0" t="n">
-        <v>54</v>
+        <v>51</v>
+      </c>
+      <c r="E169" s="0" t="s">
+        <v>213</v>
       </c>
       <c r="F169" s="0" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="I169" s="0" t="s">
-        <v>264</v>
+        <v>215</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="2" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B170" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="C170" s="2"/>
+        <v>216</v>
+      </c>
+      <c r="C170" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D170" s="0" t="n">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="E170" s="0" t="s">
-        <v>32</v>
+        <v>217</v>
+      </c>
+      <c r="F170" s="0" t="s">
+        <v>218</v>
+      </c>
+      <c r="G170" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I170" s="0" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="2" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B171" s="0" t="s">
-        <v>273</v>
-      </c>
-      <c r="C171" s="2"/>
+        <v>220</v>
+      </c>
+      <c r="C171" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D171" s="0" t="n">
-        <v>2</v>
+        <v>53</v>
+      </c>
+      <c r="F171" s="0" t="s">
+        <v>221</v>
+      </c>
+      <c r="I171" s="0" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="2" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B172" s="0" t="s">
-        <v>226</v>
-      </c>
-      <c r="C172" s="2"/>
+        <v>223</v>
+      </c>
+      <c r="C172" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D172" s="0" t="n">
-        <v>3</v>
+        <v>54</v>
       </c>
       <c r="F172" s="0" t="s">
-        <v>227</v>
+        <v>224</v>
+      </c>
+      <c r="I172" s="0" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B173" s="0" t="s">
-        <v>229</v>
+        <v>31</v>
       </c>
       <c r="C173" s="2"/>
       <c r="D173" s="0" t="n">
-        <v>4</v>
-      </c>
-      <c r="F173" s="0" t="s">
-        <v>230</v>
+        <v>1</v>
+      </c>
+      <c r="E173" s="0" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B174" s="0" t="s">
-        <v>232</v>
+        <v>278</v>
       </c>
       <c r="C174" s="2"/>
       <c r="D174" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="F174" s="0" t="s">
-        <v>233</v>
+        <v>2</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B175" s="0" t="s">
-        <v>43</v>
+        <v>231</v>
       </c>
       <c r="C175" s="2"/>
       <c r="D175" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="E175" s="0" t="s">
-        <v>44</v>
+        <v>3</v>
+      </c>
+      <c r="F175" s="0" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B176" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="C176" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>234</v>
+      </c>
+      <c r="C176" s="2"/>
       <c r="D176" s="0" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F176" s="0" t="s">
-        <v>79</v>
+        <v>235</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B177" s="0" t="s">
-        <v>274</v>
+        <v>237</v>
       </c>
       <c r="C177" s="2"/>
       <c r="D177" s="0" t="n">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="F177" s="0" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B178" s="0" t="s">
-        <v>275</v>
+        <v>43</v>
       </c>
       <c r="C178" s="2"/>
       <c r="D178" s="0" t="n">
-        <v>9</v>
+        <v>6</v>
+      </c>
+      <c r="E178" s="0" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B179" s="0" t="s">
-        <v>276</v>
-      </c>
-      <c r="C179" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="C179" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D179" s="0" t="n">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="F179" s="0" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B180" s="0" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C180" s="2"/>
       <c r="D180" s="0" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B181" s="0" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C181" s="2"/>
       <c r="D181" s="0" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B182" s="0" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C182" s="2"/>
       <c r="D182" s="0" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B183" s="0" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" s="0" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B184" s="0" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" s="0" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B185" s="0" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" s="0" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B186" s="0" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C186" s="2"/>
       <c r="D186" s="0" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B187" s="0" t="s">
+        <v>286</v>
+      </c>
+      <c r="C187" s="2"/>
+      <c r="D187" s="0" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B188" s="0" t="s">
+        <v>287</v>
+      </c>
+      <c r="C188" s="2"/>
+      <c r="D188" s="0" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B189" s="0" t="s">
+        <v>288</v>
+      </c>
+      <c r="C189" s="2"/>
+      <c r="D189" s="0" t="n">
         <v>17</v>
       </c>
     </row>
@@ -4903,7 +4990,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A186" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A189" type="list">
       <formula1>_Lists!$B$2:$B$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4915,7 +5002,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C186" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C189" type="list">
       <formula1>_Lists!$C$2:$C$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4923,7 +5010,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D186" type="whole">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D189" type="whole">
       <formula1>-2000000000</formula1>
       <formula2>2000000000</formula2>
     </dataValidation>
@@ -4939,7 +5026,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G186" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G189" type="list">
       <formula1>_Lists!$D$2:$D$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4951,7 +5038,7 @@
       <formula1>""</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" prompt="The only valid values here are no value, &quot;yes&quot; or &quot;no&quot;" promptTitle="Boolean value" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="H2:H186" type="list">
+    <dataValidation allowBlank="true" operator="between" prompt="The only valid values here are no value, &quot;yes&quot; or &quot;no&quot;" promptTitle="Boolean value" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="H2:H189" type="list">
       <formula1>_Lists!$A$2:$A$4</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
SS-114: Do not duplicate persons during an import.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@46547 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
+++ b/doc/importer/MG_IMPORT_SPREADSHEET_TYPE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="939" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="941" uniqueCount="288">
   <si>
     <t xml:space="preserve">testExportMetaTemplate</t>
   </si>
@@ -906,9 +906,6 @@
   </si>
   <si>
     <t xml:space="preserve">DRILL_TYPE_ID$NAME</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t xml:space="preserve">Specify whether a grain-size comparator was used.
@@ -1081,12 +1078,12 @@
     </xf>
   </cellXfs>
   <cellStyles count="6">
-    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3" customBuiltin="false"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6" customBuiltin="false"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4" customBuiltin="false"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7" customBuiltin="false"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5" customBuiltin="false"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
 </styleSheet>
 </file>
@@ -1097,7 +1094,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="2" style="0" width="8.67"/>
@@ -1126,7 +1123,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="5" style="0" width="8.67"/>
@@ -1234,7 +1231,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I189"/>
-  <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.38"/>
@@ -3585,6 +3582,9 @@
       <c r="D114" s="0" t="n">
         <v>50</v>
       </c>
+      <c r="E114" s="0" t="s">
+        <v>209</v>
+      </c>
       <c r="F114" s="0" t="s">
         <v>210</v>
       </c>
@@ -4029,7 +4029,7 @@
         <v>18</v>
       </c>
       <c r="E136" s="0" t="s">
-        <v>275</v>
+        <v>114</v>
       </c>
       <c r="I136" s="3" t="s">
         <v>115</v>
@@ -4483,7 +4483,7 @@
         <v>176</v>
       </c>
       <c r="I157" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4667,6 +4667,9 @@
       <c r="D168" s="0" t="n">
         <v>50</v>
       </c>
+      <c r="E168" s="0" t="s">
+        <v>209</v>
+      </c>
       <c r="F168" s="0" t="s">
         <v>210</v>
       </c>
@@ -4762,7 +4765,7 @@
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B173" s="0" t="s">
         <v>31</v>
@@ -4777,10 +4780,10 @@
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B174" s="0" t="s">
         <v>277</v>
-      </c>
-      <c r="B174" s="0" t="s">
-        <v>278</v>
       </c>
       <c r="C174" s="2"/>
       <c r="D174" s="0" t="n">
@@ -4789,7 +4792,7 @@
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B175" s="0" t="s">
         <v>231</v>
@@ -4804,7 +4807,7 @@
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B176" s="0" t="s">
         <v>234</v>
@@ -4819,7 +4822,7 @@
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B177" s="0" t="s">
         <v>237</v>
@@ -4834,7 +4837,7 @@
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B178" s="0" t="s">
         <v>43</v>
@@ -4849,7 +4852,7 @@
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B179" s="0" t="s">
         <v>78</v>
@@ -4866,10 +4869,10 @@
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B180" s="0" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C180" s="2"/>
       <c r="D180" s="0" t="n">
@@ -4878,10 +4881,10 @@
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B181" s="0" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C181" s="2"/>
       <c r="D181" s="0" t="n">
@@ -4890,10 +4893,10 @@
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B182" s="0" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C182" s="2"/>
       <c r="D182" s="0" t="n">
@@ -4902,10 +4905,10 @@
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B183" s="0" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" s="0" t="n">
@@ -4914,10 +4917,10 @@
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B184" s="0" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" s="0" t="n">
@@ -4926,10 +4929,10 @@
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B185" s="0" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" s="0" t="n">
@@ -4938,10 +4941,10 @@
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B186" s="0" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C186" s="2"/>
       <c r="D186" s="0" t="n">
@@ -4950,10 +4953,10 @@
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B187" s="0" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C187" s="2"/>
       <c r="D187" s="0" t="n">
@@ -4962,10 +4965,10 @@
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B188" s="0" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C188" s="2"/>
       <c r="D188" s="0" t="n">
@@ -4974,10 +4977,10 @@
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B189" s="0" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C189" s="2"/>
       <c r="D189" s="0" t="n">

</xml_diff>